<commit_message>
feat: allow Sol and Opus delivery managers
</commit_message>
<xml_diff>
--- a/outputs/interchange-design/interchange.xlsx
+++ b/outputs/interchange-design/interchange.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profiles" sheetId="1" r:id="Ra4b65256c3f2498f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Routing" sheetId="2" r:id="R38015e488229470a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monitoring" sheetId="3" r:id="R0fb63387998c4474"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Recovery" sheetId="4" r:id="R788440c1802d4820"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profiles" sheetId="1" r:id="R334863f27e4949b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Routing" sheetId="2" r:id="Rfd6b77a5a2754646"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monitoring" sheetId="3" r:id="R0de9f6b836fe4930"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Recovery" sheetId="4" r:id="Ra57e9e3ac184494e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -55,7 +55,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="23">
+  <x:fills count="27">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -85,6 +85,26 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFCE4D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -240,7 +260,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="116">
+  <x:cellXfs count="137">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -544,6 +564,55 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="23" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="23" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="24" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="24" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="23" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="25" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="25" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="25" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="26" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="26" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="26" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -787,7 +856,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>Policy source: Interchange policy v0.3.0</x:v>
+        <x:v>Policy source: Interchange policy v0.3.1</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -861,8 +930,8 @@
         <x:v>Allowed fixed profiles</x:v>
       </x:c>
       <x:c r="B8" s="30" t="n">
-        <x:f>COUNTIFS($G$16:$G$34,"Allowed fixed profile")</x:f>
-        <x:v>19</x:v>
+        <x:f>COUNTIFS($G$16:$G$36,"Allowed fixed profile")</x:f>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C8" s="22" t="str">
         <x:v>Select only when the assigned role, pool, and task fit.</x:v>
@@ -879,7 +948,7 @@
         <x:v>Smoke-tested fixed profiles</x:v>
       </x:c>
       <x:c r="B9" s="31" t="n">
-        <x:f>COUNTIFS($H$16:$H$34,"Smoke-tested")</x:f>
+        <x:f>COUNTIFS($H$16:$H$36,"Smoke-tested")</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="C9" s="24" t="str">
@@ -897,8 +966,8 @@
         <x:v>Documented profiles pending exact runtime check</x:v>
       </x:c>
       <x:c r="B10" s="32" t="n">
-        <x:f>COUNTIFS($H$16:$H$34,"CLI model and effort documented; exact runtime unverified")+COUNTIFS($H$16:$H$34,"Profile documented; exact runtime unverified")</x:f>
-        <x:v>5</x:v>
+        <x:f>COUNTIFS($H$16:$H$36,"CLI model and effort documented; exact runtime unverified")+COUNTIFS($H$16:$H$36,"Profile documented; exact runtime unverified")</x:f>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C10" s="24" t="str">
         <x:v>Grok, Opus and Fable entries must not be treated as smoke-tested profiles.</x:v>
@@ -993,85 +1062,85 @@
     </x:row>
     <x:row r="16" ht="38" customHeight="1">
       <x:c r="A16" s="22" t="str">
-        <x:v>dm-astra-medium</x:v>
+        <x:v>dm-opus-high</x:v>
       </x:c>
       <x:c r="B16" s="22" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Claude</x:v>
       </x:c>
       <x:c r="C16" s="22" t="str">
-        <x:v>gpt-6-astra</x:v>
+        <x:v>claude-opus-5</x:v>
       </x:c>
       <x:c r="D16" s="22" t="str">
-        <x:v>medium</x:v>
+        <x:v>high</x:v>
       </x:c>
       <x:c r="E16" s="22" t="str">
-        <x:v>delivery manager</x:v>
+        <x:v>delivery manager: approved alternative with explicit handover when switching houses</x:v>
       </x:c>
       <x:c r="F16" s="34" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G16" s="93" t="str">
+      <x:c r="G16" s="116" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H16" s="97" t="str">
-        <x:v>Supported by metadata; routing unverified</x:v>
+      <x:c r="H16" s="120" t="str">
+        <x:v>Profile documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I16" s="22" t="str">
-        <x:v>Supported by current tool metadata; routing uncalibrated</x:v>
+        <x:v>Model and effort documented; exact runtime and cross-house manager dispatch unverified</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="38" customHeight="1">
       <x:c r="A17" s="24" t="str">
-        <x:v>lead-astra-medium</x:v>
+        <x:v>dm-sol-high</x:v>
       </x:c>
       <x:c r="B17" s="24" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="C17" s="24" t="str">
-        <x:v>gpt-6-astra</x:v>
+        <x:v>gpt-5.6-sol</x:v>
       </x:c>
       <x:c r="D17" s="24" t="str">
-        <x:v>medium</x:v>
+        <x:v>high</x:v>
       </x:c>
       <x:c r="E17" s="24" t="str">
-        <x:v>lead: high ambiguity or cross-workstream architecture</x:v>
+        <x:v>delivery manager: approved alternative when starting with Sol high</x:v>
       </x:c>
       <x:c r="F17" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G17" s="94" t="str">
+      <x:c r="G17" s="117" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H17" s="98" t="str">
+      <x:c r="H17" s="121" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I17" s="24" t="str">
-        <x:v>Supported by current tool metadata; routing uncalibrated</x:v>
+        <x:v>Supported by current tool metadata; manager routing uncalibrated</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="38" customHeight="1">
       <x:c r="A18" s="24" t="str">
-        <x:v>lead-sol-medium</x:v>
+        <x:v>dm-astra-medium</x:v>
       </x:c>
       <x:c r="B18" s="24" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="C18" s="24" t="str">
-        <x:v>gpt-5.6-sol</x:v>
+        <x:v>gpt-6-astra</x:v>
       </x:c>
       <x:c r="D18" s="24" t="str">
         <x:v>medium</x:v>
       </x:c>
       <x:c r="E18" s="24" t="str">
-        <x:v>lead: bounded architecture and moderate coupling</x:v>
+        <x:v>delivery manager</x:v>
       </x:c>
       <x:c r="F18" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G18" s="94" t="str">
+      <x:c r="G18" s="117" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H18" s="98" t="str">
+      <x:c r="H18" s="121" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I18" s="24" t="str">
@@ -1080,27 +1149,27 @@
     </x:row>
     <x:row r="19" ht="38" customHeight="1">
       <x:c r="A19" s="24" t="str">
-        <x:v>lead-sol-high</x:v>
+        <x:v>lead-astra-medium</x:v>
       </x:c>
       <x:c r="B19" s="24" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="C19" s="24" t="str">
-        <x:v>gpt-5.6-sol</x:v>
+        <x:v>gpt-6-astra</x:v>
       </x:c>
       <x:c r="D19" s="24" t="str">
-        <x:v>high</x:v>
+        <x:v>medium</x:v>
       </x:c>
       <x:c r="E19" s="24" t="str">
-        <x:v>lead: consequential design and risk</x:v>
+        <x:v>lead: high ambiguity or cross-workstream architecture</x:v>
       </x:c>
       <x:c r="F19" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G19" s="94" t="str">
+      <x:c r="G19" s="117" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H19" s="98" t="str">
+      <x:c r="H19" s="121" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I19" s="24" t="str">
@@ -1109,27 +1178,27 @@
     </x:row>
     <x:row r="20" ht="38" customHeight="1">
       <x:c r="A20" s="24" t="str">
-        <x:v>lead-terra-xhigh</x:v>
+        <x:v>lead-sol-medium</x:v>
       </x:c>
       <x:c r="B20" s="24" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="C20" s="24" t="str">
-        <x:v>gpt-5.6-terra</x:v>
+        <x:v>gpt-5.6-sol</x:v>
       </x:c>
       <x:c r="D20" s="24" t="str">
-        <x:v>xhigh</x:v>
+        <x:v>medium</x:v>
       </x:c>
       <x:c r="E20" s="24" t="str">
-        <x:v>lead: defined contracts and bounded workstream</x:v>
+        <x:v>lead: bounded architecture and moderate coupling</x:v>
       </x:c>
       <x:c r="F20" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G20" s="94" t="str">
+      <x:c r="G20" s="117" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H20" s="98" t="str">
+      <x:c r="H20" s="121" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I20" s="24" t="str">
@@ -1138,27 +1207,27 @@
     </x:row>
     <x:row r="21" ht="38" customHeight="1">
       <x:c r="A21" s="24" t="str">
-        <x:v>lead-terra-max</x:v>
+        <x:v>lead-sol-high</x:v>
       </x:c>
       <x:c r="B21" s="24" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="C21" s="24" t="str">
-        <x:v>gpt-5.6-terra</x:v>
+        <x:v>gpt-5.6-sol</x:v>
       </x:c>
       <x:c r="D21" s="24" t="str">
-        <x:v>max</x:v>
+        <x:v>high</x:v>
       </x:c>
       <x:c r="E21" s="24" t="str">
-        <x:v>lead: defined architecture with difficult integration</x:v>
+        <x:v>lead: consequential design and risk</x:v>
       </x:c>
       <x:c r="F21" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G21" s="94" t="str">
+      <x:c r="G21" s="117" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H21" s="98" t="str">
+      <x:c r="H21" s="121" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I21" s="24" t="str">
@@ -1167,274 +1236,274 @@
     </x:row>
     <x:row r="22" ht="38" customHeight="1">
       <x:c r="A22" s="24" t="str">
-        <x:v>worker-luna-xhigh</x:v>
+        <x:v>lead-terra-xhigh</x:v>
       </x:c>
       <x:c r="B22" s="24" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="C22" s="24" t="str">
-        <x:v>gpt-5.6-luna</x:v>
+        <x:v>gpt-5.6-terra</x:v>
       </x:c>
       <x:c r="D22" s="24" t="str">
         <x:v>xhigh</x:v>
       </x:c>
       <x:c r="E22" s="24" t="str">
-        <x:v>bounded leaf exploration or explicit small change</x:v>
+        <x:v>lead: defined contracts and bounded workstream</x:v>
       </x:c>
       <x:c r="F22" s="35" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="G22" s="94" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G22" s="117" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H22" s="98" t="str">
+      <x:c r="H22" s="121" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I22" s="24" t="str">
-        <x:v>Supported; lower effort forbidden by owner</x:v>
+        <x:v>Supported by current tool metadata; routing uncalibrated</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="38" customHeight="1">
       <x:c r="A23" s="24" t="str">
-        <x:v>worker-luna-max</x:v>
+        <x:v>lead-terra-max</x:v>
       </x:c>
       <x:c r="B23" s="24" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="C23" s="24" t="str">
-        <x:v>gpt-5.6-luna</x:v>
+        <x:v>gpt-5.6-terra</x:v>
       </x:c>
       <x:c r="D23" s="24" t="str">
         <x:v>max</x:v>
       </x:c>
       <x:c r="E23" s="24" t="str">
-        <x:v>bounded leaf with denser evidence</x:v>
+        <x:v>lead: defined architecture with difficult integration</x:v>
       </x:c>
       <x:c r="F23" s="35" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="G23" s="94" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G23" s="117" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H23" s="98" t="str">
+      <x:c r="H23" s="121" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I23" s="24" t="str">
-        <x:v>Supported; lower effort forbidden by owner</x:v>
+        <x:v>Supported by current tool metadata; routing uncalibrated</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="38" customHeight="1">
       <x:c r="A24" s="24" t="str">
-        <x:v>worker-terra-xhigh</x:v>
+        <x:v>worker-luna-xhigh</x:v>
       </x:c>
       <x:c r="B24" s="24" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="C24" s="24" t="str">
-        <x:v>gpt-5.6-terra</x:v>
+        <x:v>gpt-5.6-luna</x:v>
       </x:c>
       <x:c r="D24" s="24" t="str">
         <x:v>xhigh</x:v>
       </x:c>
       <x:c r="E24" s="24" t="str">
-        <x:v>bounded builder or independent verifier</x:v>
+        <x:v>bounded leaf exploration or explicit small change</x:v>
       </x:c>
       <x:c r="F24" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G24" s="94" t="str">
+      <x:c r="G24" s="117" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H24" s="98" t="str">
+      <x:c r="H24" s="121" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I24" s="24" t="str">
-        <x:v>Supported; role assignment separate from model</x:v>
+        <x:v>Supported; lower effort forbidden by owner</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="38" customHeight="1">
       <x:c r="A25" s="24" t="str">
-        <x:v>worker-muse-xhigh</x:v>
+        <x:v>worker-luna-max</x:v>
       </x:c>
       <x:c r="B25" s="24" t="str">
-        <x:v>OpenCode / Go pool</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="C25" s="24" t="str">
-        <x:v>opencode-go/muse-spark-1.3-contributor</x:v>
+        <x:v>gpt-5.6-luna</x:v>
       </x:c>
       <x:c r="D25" s="24" t="str">
-        <x:v>xhigh</x:v>
+        <x:v>max</x:v>
       </x:c>
       <x:c r="E25" s="24" t="str">
-        <x:v>preferred initial cheap leaf candidate</x:v>
+        <x:v>bounded leaf with denser evidence</x:v>
       </x:c>
       <x:c r="F25" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G25" s="94" t="str">
+      <x:c r="G25" s="117" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H25" s="100" t="str">
-        <x:v>Smoke-tested</x:v>
+      <x:c r="H25" s="121" t="str">
+        <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I25" s="24" t="str">
-        <x:v>CLI send/resume/recall smoke-tested; quality advantage is owner hypothesis</x:v>
+        <x:v>Supported; lower effort forbidden by owner</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="38" customHeight="1">
       <x:c r="A26" s="24" t="str">
-        <x:v>worker-grok-high</x:v>
+        <x:v>worker-terra-xhigh</x:v>
       </x:c>
       <x:c r="B26" s="24" t="str">
-        <x:v>Grok</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="C26" s="24" t="str">
-        <x:v>grok-4.6</x:v>
+        <x:v>gpt-5.6-terra</x:v>
       </x:c>
       <x:c r="D26" s="24" t="str">
-        <x:v>high</x:v>
+        <x:v>xhigh</x:v>
       </x:c>
       <x:c r="E26" s="24" t="str">
-        <x:v>primary low/mid complexity developer</x:v>
+        <x:v>bounded builder or independent verifier</x:v>
       </x:c>
       <x:c r="F26" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G26" s="94" t="str">
+      <x:c r="G26" s="117" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H26" s="98" t="str">
-        <x:v>CLI model and effort documented; exact runtime unverified</x:v>
+      <x:c r="H26" s="121" t="str">
+        <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I26" s="24" t="str">
-        <x:v>grok models lists grok-4.6; effort flags documented; exact profile smoke test pending</x:v>
+        <x:v>Supported; role assignment separate from model</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="38" customHeight="1">
       <x:c r="A27" s="24" t="str">
-        <x:v>worker-grok-xhigh</x:v>
+        <x:v>worker-muse-xhigh</x:v>
       </x:c>
       <x:c r="B27" s="24" t="str">
-        <x:v>Grok</x:v>
+        <x:v>OpenCode / Go pool</x:v>
       </x:c>
       <x:c r="C27" s="24" t="str">
-        <x:v>grok-4.6</x:v>
+        <x:v>opencode-go/muse-spark-1.3-contributor</x:v>
       </x:c>
       <x:c r="D27" s="24" t="str">
         <x:v>xhigh</x:v>
       </x:c>
       <x:c r="E27" s="24" t="str">
-        <x:v>primary upper-mid complexity developer</x:v>
+        <x:v>preferred initial cheap leaf candidate</x:v>
       </x:c>
       <x:c r="F27" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G27" s="94" t="str">
+      <x:c r="G27" s="117" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H27" s="98" t="str">
-        <x:v>CLI model and effort documented; exact runtime unverified</x:v>
+      <x:c r="H27" s="123" t="str">
+        <x:v>Smoke-tested</x:v>
       </x:c>
       <x:c r="I27" s="24" t="str">
-        <x:v>grok models lists grok-4.6; effort flags documented; exact profile smoke test pending</x:v>
+        <x:v>CLI send/resume/recall smoke-tested; quality advantage is owner hypothesis</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="38" customHeight="1">
       <x:c r="A28" s="24" t="str">
-        <x:v>worker-opus-medium</x:v>
+        <x:v>worker-grok-high</x:v>
       </x:c>
       <x:c r="B28" s="24" t="str">
-        <x:v>Claude</x:v>
+        <x:v>Grok</x:v>
       </x:c>
       <x:c r="C28" s="24" t="str">
-        <x:v>claude-opus-5</x:v>
+        <x:v>grok-4.6</x:v>
       </x:c>
       <x:c r="D28" s="24" t="str">
-        <x:v>medium</x:v>
+        <x:v>high</x:v>
       </x:c>
       <x:c r="E28" s="24" t="str">
-        <x:v>primary low/mid and upper-mid complexity developer</x:v>
+        <x:v>primary low/mid complexity developer</x:v>
       </x:c>
       <x:c r="F28" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G28" s="94" t="str">
+      <x:c r="G28" s="117" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H28" s="98" t="str">
-        <x:v>Profile documented; exact runtime unverified</x:v>
+      <x:c r="H28" s="121" t="str">
+        <x:v>CLI model and effort documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I28" s="24" t="str">
-        <x:v>Full model ID and effort documented; exact profile runtime identity and smoke test pending</x:v>
+        <x:v>grok models lists grok-4.6; effort flags documented; exact profile smoke test pending</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="38" customHeight="1">
       <x:c r="A29" s="24" t="str">
-        <x:v>worker-opus-high</x:v>
+        <x:v>worker-grok-xhigh</x:v>
       </x:c>
       <x:c r="B29" s="24" t="str">
-        <x:v>Claude</x:v>
+        <x:v>Grok</x:v>
       </x:c>
       <x:c r="C29" s="24" t="str">
-        <x:v>claude-opus-5</x:v>
+        <x:v>grok-4.6</x:v>
       </x:c>
       <x:c r="D29" s="24" t="str">
-        <x:v>high</x:v>
+        <x:v>xhigh</x:v>
       </x:c>
       <x:c r="E29" s="24" t="str">
-        <x:v>primary high complexity developer</x:v>
+        <x:v>primary upper-mid complexity developer</x:v>
       </x:c>
       <x:c r="F29" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G29" s="94" t="str">
+      <x:c r="G29" s="117" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H29" s="98" t="str">
-        <x:v>Profile documented; exact runtime unverified</x:v>
+      <x:c r="H29" s="121" t="str">
+        <x:v>CLI model and effort documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I29" s="24" t="str">
-        <x:v>Full model ID and effort documented; exact profile runtime identity and smoke test pending</x:v>
+        <x:v>grok models lists grok-4.6; effort flags documented; exact profile smoke test pending</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="38" customHeight="1">
       <x:c r="A30" s="24" t="str">
-        <x:v>worker-sol-medium</x:v>
+        <x:v>worker-opus-medium</x:v>
       </x:c>
       <x:c r="B30" s="24" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Claude</x:v>
       </x:c>
       <x:c r="C30" s="24" t="str">
-        <x:v>gpt-5.6-sol</x:v>
+        <x:v>claude-opus-5</x:v>
       </x:c>
       <x:c r="D30" s="24" t="str">
         <x:v>medium</x:v>
       </x:c>
       <x:c r="E30" s="24" t="str">
-        <x:v>primary low/mid complexity developer</x:v>
+        <x:v>primary low/mid and upper-mid complexity developer</x:v>
       </x:c>
       <x:c r="F30" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G30" s="94" t="str">
+      <x:c r="G30" s="117" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H30" s="98" t="str">
-        <x:v>Supported by metadata; routing unverified</x:v>
+      <x:c r="H30" s="121" t="str">
+        <x:v>Profile documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I30" s="24" t="str">
-        <x:v>Current tool metadata supports profile; task-class performance uncalibrated</x:v>
+        <x:v>Full model ID and effort documented; exact profile runtime identity and smoke test pending</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="38" customHeight="1">
       <x:c r="A31" s="24" t="str">
-        <x:v>worker-sol-high</x:v>
+        <x:v>worker-opus-high</x:v>
       </x:c>
       <x:c r="B31" s="24" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Claude</x:v>
       </x:c>
       <x:c r="C31" s="24" t="str">
-        <x:v>gpt-5.6-sol</x:v>
+        <x:v>claude-opus-5</x:v>
       </x:c>
       <x:c r="D31" s="24" t="str">
         <x:v>high</x:v>
@@ -1445,100 +1514,158 @@
       <x:c r="F31" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G31" s="94" t="str">
+      <x:c r="G31" s="117" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H31" s="98" t="str">
-        <x:v>Supported by metadata; routing unverified</x:v>
+      <x:c r="H31" s="121" t="str">
+        <x:v>Profile documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I31" s="24" t="str">
-        <x:v>Current tool metadata supports profile; task-class performance uncalibrated</x:v>
+        <x:v>Full model ID and effort documented; exact profile runtime identity and smoke test pending</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="38" customHeight="1">
       <x:c r="A32" s="24" t="str">
-        <x:v>worker-terra-max</x:v>
+        <x:v>worker-sol-medium</x:v>
       </x:c>
       <x:c r="B32" s="24" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="C32" s="24" t="str">
-        <x:v>gpt-5.6-terra</x:v>
+        <x:v>gpt-5.6-sol</x:v>
       </x:c>
       <x:c r="D32" s="24" t="str">
-        <x:v>max</x:v>
+        <x:v>medium</x:v>
       </x:c>
       <x:c r="E32" s="24" t="str">
-        <x:v>demanding implementation with settled contracts and bounded scope</x:v>
+        <x:v>primary low/mid complexity developer</x:v>
       </x:c>
       <x:c r="F32" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G32" s="94" t="str">
+      <x:c r="G32" s="117" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H32" s="98" t="str">
+      <x:c r="H32" s="121" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I32" s="24" t="str">
-        <x:v>Current tool metadata supports profile; effort is not a substitute for resolving ambiguity</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33" ht="76" customHeight="1">
+        <x:v>Current tool metadata supports profile; task-class performance uncalibrated</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="38" customHeight="1">
       <x:c r="A33" s="24" t="str">
-        <x:v>brainstorm-fable-medium</x:v>
+        <x:v>worker-sol-high</x:v>
       </x:c>
       <x:c r="B33" s="24" t="str">
-        <x:v>Claude</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="C33" s="24" t="str">
-        <x:v>claude-fable-5-1</x:v>
+        <x:v>gpt-5.6-sol</x:v>
       </x:c>
       <x:c r="D33" s="24" t="str">
-        <x:v>medium</x:v>
+        <x:v>high</x:v>
       </x:c>
       <x:c r="E33" s="24" t="str">
-        <x:v>new-product ideation and brainstorming</x:v>
+        <x:v>primary high complexity developer</x:v>
       </x:c>
       <x:c r="F33" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G33" s="94" t="str">
+      <x:c r="G33" s="117" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H33" s="98" t="str">
-        <x:v>Profile documented; exact runtime unverified</x:v>
+      <x:c r="H33" s="121" t="str">
+        <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I33" s="24" t="str">
-        <x:v>Official model/effort documentation; exact runtime and included-plan eligibility not verified</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34" ht="76" customHeight="1">
+        <x:v>Current tool metadata supports profile; task-class performance uncalibrated</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="38" customHeight="1">
       <x:c r="A34" s="24" t="str">
-        <x:v>brainstorm-astra-medium</x:v>
+        <x:v>worker-terra-max</x:v>
       </x:c>
       <x:c r="B34" s="24" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="C34" s="24" t="str">
-        <x:v>gpt-6-astra</x:v>
+        <x:v>gpt-5.6-terra</x:v>
       </x:c>
       <x:c r="D34" s="24" t="str">
-        <x:v>medium</x:v>
+        <x:v>max</x:v>
       </x:c>
       <x:c r="E34" s="24" t="str">
-        <x:v>new-product ideation and brainstorming</x:v>
+        <x:v>demanding implementation with settled contracts and bounded scope</x:v>
       </x:c>
       <x:c r="F34" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G34" s="94" t="str">
+      <x:c r="G34" s="117" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H34" s="98" t="str">
+      <x:c r="H34" s="121" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I34" s="24" t="str">
+        <x:v>Current tool metadata supports profile; effort is not a substitute for resolving ambiguity</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="76" customHeight="1">
+      <x:c r="A35" s="24" t="str">
+        <x:v>brainstorm-fable-medium</x:v>
+      </x:c>
+      <x:c r="B35" s="24" t="str">
+        <x:v>Claude</x:v>
+      </x:c>
+      <x:c r="C35" s="24" t="str">
+        <x:v>claude-fable-5-1</x:v>
+      </x:c>
+      <x:c r="D35" s="24" t="str">
+        <x:v>medium</x:v>
+      </x:c>
+      <x:c r="E35" s="24" t="str">
+        <x:v>new-product ideation and brainstorming</x:v>
+      </x:c>
+      <x:c r="F35" s="35" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="G35" s="117" t="str">
+        <x:v>Allowed fixed profile</x:v>
+      </x:c>
+      <x:c r="H35" s="121" t="str">
+        <x:v>Profile documented; exact runtime unverified</x:v>
+      </x:c>
+      <x:c r="I35" s="24" t="str">
+        <x:v>Official model/effort documentation; exact runtime and included-plan eligibility not verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="76" customHeight="1">
+      <x:c r="A36" s="24" t="str">
+        <x:v>brainstorm-astra-medium</x:v>
+      </x:c>
+      <x:c r="B36" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="C36" s="24" t="str">
+        <x:v>gpt-6-astra</x:v>
+      </x:c>
+      <x:c r="D36" s="24" t="str">
+        <x:v>medium</x:v>
+      </x:c>
+      <x:c r="E36" s="24" t="str">
+        <x:v>new-product ideation and brainstorming</x:v>
+      </x:c>
+      <x:c r="F36" s="35" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="G36" s="117" t="str">
+        <x:v>Allowed fixed profile</x:v>
+      </x:c>
+      <x:c r="H36" s="121" t="str">
+        <x:v>Supported by metadata; routing unverified</x:v>
+      </x:c>
+      <x:c r="I36" s="24" t="str">
         <x:v>Current tool metadata supports profile; no comparative ideation benchmark</x:v>
       </x:c>
     </x:row>
@@ -1576,7 +1703,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>Policy source: Interchange policy v0.3.0</x:v>
+        <x:v>Policy source: Interchange policy v0.3.1</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2" t="str">
@@ -1754,7 +1881,7 @@
         <x:v>dm-astra-medium</x:v>
       </x:c>
       <x:c r="C17" s="24" t="str">
-        <x:v>Owner decision if approved roster unavailable</x:v>
+        <x:v>dm-sol-high or dm-opus-high; use directly when already in that configuration; verify transport and handover for house switches</x:v>
       </x:c>
       <x:c r="D17" s="24" t="str">
         <x:v>Manager receives compact exceptions and evidence, not raw logs</x:v>
@@ -1781,20 +1908,20 @@
       <x:c r="D20"/>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="103" t="str">
+      <x:c r="A21" s="126" t="str">
         <x:v>Selection rules</x:v>
       </x:c>
-      <x:c r="B21" s="104"/>
-      <x:c r="C21" s="104"/>
-      <x:c r="D21" s="105"/>
+      <x:c r="B21" s="127"/>
+      <x:c r="C21" s="127"/>
+      <x:c r="D21" s="128"/>
     </x:row>
     <x:row r="22" ht="42" customHeight="1">
-      <x:c r="A22" s="111" t="str">
+      <x:c r="A22" s="134" t="str">
         <x:v>Approved selection rule</x:v>
       </x:c>
-      <x:c r="B22" s="112"/>
-      <x:c r="C22" s="112"/>
-      <x:c r="D22" s="113"/>
+      <x:c r="B22" s="135"/>
+      <x:c r="C22" s="135"/>
+      <x:c r="D22" s="136"/>
     </x:row>
     <x:row r="23" ht="42" customHeight="1">
       <x:c r="A23" s="91" t="str">
@@ -1956,7 +2083,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>Policy source: Interchange policy v0.3.0</x:v>
+        <x:v>Policy source: Interchange policy v0.3.1</x:v>
       </x:c>
       <x:c r="B3" s="2" t="str">
         <x:v>Approved on</x:v>
@@ -2123,7 +2250,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>Policy source: Interchange policy v0.3.0</x:v>
+        <x:v>Policy source: Interchange policy v0.3.1</x:v>
       </x:c>
       <x:c r="B3" s="2" t="str">
         <x:v>Approved on</x:v>

</xml_diff>

<commit_message>
fix: scope house exclusivity by manager
</commit_message>
<xml_diff>
--- a/outputs/interchange-design/interchange.xlsx
+++ b/outputs/interchange-design/interchange.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profiles" sheetId="1" r:id="R334863f27e4949b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Routing" sheetId="2" r:id="Rfd6b77a5a2754646"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monitoring" sheetId="3" r:id="R0de9f6b836fe4930"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Recovery" sheetId="4" r:id="Ra57e9e3ac184494e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profiles" sheetId="1" r:id="Rbeba48ecde57412c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Routing" sheetId="2" r:id="R2259a9e0154744b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monitoring" sheetId="3" r:id="R440acc007ff54f69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Recovery" sheetId="4" r:id="Re7159dde90714418"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -55,7 +55,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="27">
+  <x:fills count="31">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -85,6 +85,26 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFCE4D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -260,7 +280,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="137">
+  <x:cellXfs count="155">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -612,6 +632,46 @@
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="26" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="27" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="27" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="28" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="28" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="27" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="29" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="29" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="29" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="30" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="30" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="30" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -856,7 +916,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>Policy source: Interchange policy v0.3.1</x:v>
+        <x:v>Policy source: Interchange policy v0.3.2</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -1079,10 +1139,10 @@
       <x:c r="F16" s="34" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G16" s="116" t="str">
+      <x:c r="G16" s="137" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H16" s="120" t="str">
+      <x:c r="H16" s="139" t="str">
         <x:v>Profile documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I16" s="22" t="str">
@@ -1108,10 +1168,10 @@
       <x:c r="F17" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G17" s="117" t="str">
+      <x:c r="G17" s="138" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H17" s="121" t="str">
+      <x:c r="H17" s="140" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I17" s="24" t="str">
@@ -1137,10 +1197,10 @@
       <x:c r="F18" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G18" s="117" t="str">
+      <x:c r="G18" s="138" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H18" s="121" t="str">
+      <x:c r="H18" s="140" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I18" s="24" t="str">
@@ -1166,10 +1226,10 @@
       <x:c r="F19" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G19" s="117" t="str">
+      <x:c r="G19" s="138" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H19" s="121" t="str">
+      <x:c r="H19" s="140" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I19" s="24" t="str">
@@ -1195,10 +1255,10 @@
       <x:c r="F20" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G20" s="117" t="str">
+      <x:c r="G20" s="138" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H20" s="121" t="str">
+      <x:c r="H20" s="140" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I20" s="24" t="str">
@@ -1224,10 +1284,10 @@
       <x:c r="F21" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G21" s="117" t="str">
+      <x:c r="G21" s="138" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H21" s="121" t="str">
+      <x:c r="H21" s="140" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I21" s="24" t="str">
@@ -1253,10 +1313,10 @@
       <x:c r="F22" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G22" s="117" t="str">
+      <x:c r="G22" s="138" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H22" s="121" t="str">
+      <x:c r="H22" s="140" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I22" s="24" t="str">
@@ -1282,10 +1342,10 @@
       <x:c r="F23" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G23" s="117" t="str">
+      <x:c r="G23" s="138" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H23" s="121" t="str">
+      <x:c r="H23" s="140" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I23" s="24" t="str">
@@ -1311,10 +1371,10 @@
       <x:c r="F24" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G24" s="117" t="str">
+      <x:c r="G24" s="138" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H24" s="121" t="str">
+      <x:c r="H24" s="140" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I24" s="24" t="str">
@@ -1340,10 +1400,10 @@
       <x:c r="F25" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G25" s="117" t="str">
+      <x:c r="G25" s="138" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H25" s="121" t="str">
+      <x:c r="H25" s="140" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I25" s="24" t="str">
@@ -1369,10 +1429,10 @@
       <x:c r="F26" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G26" s="117" t="str">
+      <x:c r="G26" s="138" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H26" s="121" t="str">
+      <x:c r="H26" s="140" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I26" s="24" t="str">
@@ -1398,10 +1458,10 @@
       <x:c r="F27" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G27" s="117" t="str">
+      <x:c r="G27" s="138" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H27" s="123" t="str">
+      <x:c r="H27" s="141" t="str">
         <x:v>Smoke-tested</x:v>
       </x:c>
       <x:c r="I27" s="24" t="str">
@@ -1427,10 +1487,10 @@
       <x:c r="F28" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G28" s="117" t="str">
+      <x:c r="G28" s="138" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H28" s="121" t="str">
+      <x:c r="H28" s="140" t="str">
         <x:v>CLI model and effort documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I28" s="24" t="str">
@@ -1456,10 +1516,10 @@
       <x:c r="F29" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G29" s="117" t="str">
+      <x:c r="G29" s="138" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H29" s="121" t="str">
+      <x:c r="H29" s="140" t="str">
         <x:v>CLI model and effort documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I29" s="24" t="str">
@@ -1485,10 +1545,10 @@
       <x:c r="F30" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G30" s="117" t="str">
+      <x:c r="G30" s="138" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H30" s="121" t="str">
+      <x:c r="H30" s="140" t="str">
         <x:v>Profile documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I30" s="24" t="str">
@@ -1514,10 +1574,10 @@
       <x:c r="F31" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G31" s="117" t="str">
+      <x:c r="G31" s="138" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H31" s="121" t="str">
+      <x:c r="H31" s="140" t="str">
         <x:v>Profile documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I31" s="24" t="str">
@@ -1543,10 +1603,10 @@
       <x:c r="F32" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G32" s="117" t="str">
+      <x:c r="G32" s="138" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H32" s="121" t="str">
+      <x:c r="H32" s="140" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I32" s="24" t="str">
@@ -1572,10 +1632,10 @@
       <x:c r="F33" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G33" s="117" t="str">
+      <x:c r="G33" s="138" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H33" s="121" t="str">
+      <x:c r="H33" s="140" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I33" s="24" t="str">
@@ -1601,10 +1661,10 @@
       <x:c r="F34" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G34" s="117" t="str">
+      <x:c r="G34" s="138" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H34" s="121" t="str">
+      <x:c r="H34" s="140" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I34" s="24" t="str">
@@ -1630,10 +1690,10 @@
       <x:c r="F35" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G35" s="117" t="str">
+      <x:c r="G35" s="138" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H35" s="121" t="str">
+      <x:c r="H35" s="140" t="str">
         <x:v>Profile documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I35" s="24" t="str">
@@ -1659,10 +1719,10 @@
       <x:c r="F36" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G36" s="117" t="str">
+      <x:c r="G36" s="138" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H36" s="121" t="str">
+      <x:c r="H36" s="140" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I36" s="24" t="str">
@@ -1703,7 +1763,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>Policy source: Interchange policy v0.3.1</x:v>
+        <x:v>Policy source: Interchange policy v0.3.2</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2" t="str">
@@ -1908,20 +1968,20 @@
       <x:c r="D20"/>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="126" t="str">
+      <x:c r="A21" s="144" t="str">
         <x:v>Selection rules</x:v>
       </x:c>
-      <x:c r="B21" s="127"/>
-      <x:c r="C21" s="127"/>
-      <x:c r="D21" s="128"/>
+      <x:c r="B21" s="145"/>
+      <x:c r="C21" s="145"/>
+      <x:c r="D21" s="146"/>
     </x:row>
     <x:row r="22" ht="42" customHeight="1">
-      <x:c r="A22" s="134" t="str">
+      <x:c r="A22" s="152" t="str">
         <x:v>Approved selection rule</x:v>
       </x:c>
-      <x:c r="B22" s="135"/>
-      <x:c r="C22" s="135"/>
-      <x:c r="D22" s="136"/>
+      <x:c r="B22" s="153"/>
+      <x:c r="C22" s="153"/>
+      <x:c r="D22" s="154"/>
     </x:row>
     <x:row r="23" ht="42" customHeight="1">
       <x:c r="A23" s="91" t="str">
@@ -2013,7 +2073,7 @@
     </x:row>
     <x:row r="34" ht="42" customHeight="1">
       <x:c r="A34" s="92" t="str">
-        <x:v>12. House exclusivity takes precedence over parallelism preferences: Sol high or higher and Astra any effort reserve Codex; Opus high or higher and Fable 5.1 any effort reserve Claude.</x:v>
+        <x:v>12. House exclusivity has two scopes. Astra at any effort reserves Codex globally and Fable 5.1 at any effort reserves Claude globally. Sol high or higher reserves Codex only for assignments under the same delivery manager; Opus high or higher reserves Claude only for assignments under the same delivery manager.</x:v>
       </x:c>
       <x:c r="B34" s="69"/>
       <x:c r="C34" s="69"/>
@@ -2021,7 +2081,7 @@
     </x:row>
     <x:row r="35" ht="42" customHeight="1">
       <x:c r="A35" s="92" t="str">
-        <x:v>13. New-product brainstorming may use Fable 5.1 medium or Astra medium. Both reserve their entire house while active; prefer another eligible house or queue competing work.</x:v>
+        <x:v>13. New-product brainstorming may use Fable 5.1 medium or Astra medium. Both create global house reservations while active; prefer another eligible house or queue competing work.</x:v>
       </x:c>
       <x:c r="B35" s="69"/>
       <x:c r="C35" s="69"/>
@@ -2083,7 +2143,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>Policy source: Interchange policy v0.3.1</x:v>
+        <x:v>Policy source: Interchange policy v0.3.2</x:v>
       </x:c>
       <x:c r="B3" s="2" t="str">
         <x:v>Approved on</x:v>
@@ -2250,7 +2310,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>Policy source: Interchange policy v0.3.1</x:v>
+        <x:v>Policy source: Interchange policy v0.3.2</x:v>
       </x:c>
       <x:c r="B3" s="2" t="str">
         <x:v>Approved on</x:v>

</xml_diff>

<commit_message>
feat: harden Interchange supervision and adapters
</commit_message>
<xml_diff>
--- a/outputs/interchange-design/interchange.xlsx
+++ b/outputs/interchange-design/interchange.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profiles" sheetId="1" r:id="Rbeba48ecde57412c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Routing" sheetId="2" r:id="R2259a9e0154744b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monitoring" sheetId="3" r:id="R440acc007ff54f69"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Recovery" sheetId="4" r:id="Re7159dde90714418"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profiles" sheetId="1" r:id="Rdb05d2334a084321"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Routing" sheetId="2" r:id="R4a8f0ce1555046dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monitoring" sheetId="3" r:id="R22d28bd2e77f4b53"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Recovery" sheetId="4" r:id="Rc554ec4257a34146"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -55,7 +55,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="31">
+  <x:fills count="39">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -85,6 +85,46 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFCE4D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -280,7 +320,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="155">
+  <x:cellXfs count="191">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -672,6 +712,86 @@
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="30" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="31" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="31" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="32" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="32" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="31" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="33" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="33" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="33" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="34" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="34" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="34" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="35" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="35" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="36" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="36" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="35" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="37" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="37" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="37" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="38" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="38" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="38" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -916,7 +1036,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>Policy source: Interchange policy v0.3.2</x:v>
+        <x:v>Policy source: Interchange policy v0.4.0</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -1139,10 +1259,10 @@
       <x:c r="F16" s="34" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G16" s="137" t="str">
+      <x:c r="G16" s="173" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H16" s="139" t="str">
+      <x:c r="H16" s="175" t="str">
         <x:v>Profile documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I16" s="22" t="str">
@@ -1168,10 +1288,10 @@
       <x:c r="F17" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G17" s="138" t="str">
+      <x:c r="G17" s="174" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H17" s="140" t="str">
+      <x:c r="H17" s="176" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I17" s="24" t="str">
@@ -1197,10 +1317,10 @@
       <x:c r="F18" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G18" s="138" t="str">
+      <x:c r="G18" s="174" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H18" s="140" t="str">
+      <x:c r="H18" s="176" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I18" s="24" t="str">
@@ -1226,10 +1346,10 @@
       <x:c r="F19" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G19" s="138" t="str">
+      <x:c r="G19" s="174" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H19" s="140" t="str">
+      <x:c r="H19" s="176" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I19" s="24" t="str">
@@ -1255,10 +1375,10 @@
       <x:c r="F20" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G20" s="138" t="str">
+      <x:c r="G20" s="174" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H20" s="140" t="str">
+      <x:c r="H20" s="176" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I20" s="24" t="str">
@@ -1284,10 +1404,10 @@
       <x:c r="F21" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G21" s="138" t="str">
+      <x:c r="G21" s="174" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H21" s="140" t="str">
+      <x:c r="H21" s="176" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I21" s="24" t="str">
@@ -1313,10 +1433,10 @@
       <x:c r="F22" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G22" s="138" t="str">
+      <x:c r="G22" s="174" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H22" s="140" t="str">
+      <x:c r="H22" s="176" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I22" s="24" t="str">
@@ -1342,10 +1462,10 @@
       <x:c r="F23" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G23" s="138" t="str">
+      <x:c r="G23" s="174" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H23" s="140" t="str">
+      <x:c r="H23" s="176" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I23" s="24" t="str">
@@ -1371,10 +1491,10 @@
       <x:c r="F24" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G24" s="138" t="str">
+      <x:c r="G24" s="174" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H24" s="140" t="str">
+      <x:c r="H24" s="176" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I24" s="24" t="str">
@@ -1400,10 +1520,10 @@
       <x:c r="F25" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G25" s="138" t="str">
+      <x:c r="G25" s="174" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H25" s="140" t="str">
+      <x:c r="H25" s="176" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I25" s="24" t="str">
@@ -1429,10 +1549,10 @@
       <x:c r="F26" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G26" s="138" t="str">
+      <x:c r="G26" s="174" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H26" s="140" t="str">
+      <x:c r="H26" s="176" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I26" s="24" t="str">
@@ -1458,10 +1578,10 @@
       <x:c r="F27" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G27" s="138" t="str">
+      <x:c r="G27" s="174" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H27" s="141" t="str">
+      <x:c r="H27" s="177" t="str">
         <x:v>Smoke-tested</x:v>
       </x:c>
       <x:c r="I27" s="24" t="str">
@@ -1487,10 +1607,10 @@
       <x:c r="F28" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G28" s="138" t="str">
+      <x:c r="G28" s="174" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H28" s="140" t="str">
+      <x:c r="H28" s="176" t="str">
         <x:v>CLI model and effort documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I28" s="24" t="str">
@@ -1516,10 +1636,10 @@
       <x:c r="F29" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G29" s="138" t="str">
+      <x:c r="G29" s="174" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H29" s="140" t="str">
+      <x:c r="H29" s="176" t="str">
         <x:v>CLI model and effort documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I29" s="24" t="str">
@@ -1545,10 +1665,10 @@
       <x:c r="F30" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G30" s="138" t="str">
+      <x:c r="G30" s="174" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H30" s="140" t="str">
+      <x:c r="H30" s="176" t="str">
         <x:v>Profile documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I30" s="24" t="str">
@@ -1574,10 +1694,10 @@
       <x:c r="F31" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G31" s="138" t="str">
+      <x:c r="G31" s="174" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H31" s="140" t="str">
+      <x:c r="H31" s="176" t="str">
         <x:v>Profile documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I31" s="24" t="str">
@@ -1603,10 +1723,10 @@
       <x:c r="F32" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G32" s="138" t="str">
+      <x:c r="G32" s="174" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H32" s="140" t="str">
+      <x:c r="H32" s="176" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I32" s="24" t="str">
@@ -1632,10 +1752,10 @@
       <x:c r="F33" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G33" s="138" t="str">
+      <x:c r="G33" s="174" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H33" s="140" t="str">
+      <x:c r="H33" s="176" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I33" s="24" t="str">
@@ -1661,10 +1781,10 @@
       <x:c r="F34" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G34" s="138" t="str">
+      <x:c r="G34" s="174" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H34" s="140" t="str">
+      <x:c r="H34" s="176" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I34" s="24" t="str">
@@ -1690,10 +1810,10 @@
       <x:c r="F35" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G35" s="138" t="str">
+      <x:c r="G35" s="174" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H35" s="140" t="str">
+      <x:c r="H35" s="176" t="str">
         <x:v>Profile documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I35" s="24" t="str">
@@ -1719,10 +1839,10 @@
       <x:c r="F36" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G36" s="138" t="str">
+      <x:c r="G36" s="174" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H36" s="140" t="str">
+      <x:c r="H36" s="176" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I36" s="24" t="str">
@@ -1763,7 +1883,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>Policy source: Interchange policy v0.3.2</x:v>
+        <x:v>Policy source: Interchange policy v0.4.0</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2" t="str">
@@ -1968,20 +2088,20 @@
       <x:c r="D20"/>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="144" t="str">
+      <x:c r="A21" s="180" t="str">
         <x:v>Selection rules</x:v>
       </x:c>
-      <x:c r="B21" s="145"/>
-      <x:c r="C21" s="145"/>
-      <x:c r="D21" s="146"/>
+      <x:c r="B21" s="181"/>
+      <x:c r="C21" s="181"/>
+      <x:c r="D21" s="182"/>
     </x:row>
     <x:row r="22" ht="42" customHeight="1">
-      <x:c r="A22" s="152" t="str">
+      <x:c r="A22" s="188" t="str">
         <x:v>Approved selection rule</x:v>
       </x:c>
-      <x:c r="B22" s="153"/>
-      <x:c r="C22" s="153"/>
-      <x:c r="D22" s="154"/>
+      <x:c r="B22" s="189"/>
+      <x:c r="C22" s="189"/>
+      <x:c r="D22" s="190"/>
     </x:row>
     <x:row r="23" ht="42" customHeight="1">
       <x:c r="A23" s="91" t="str">
@@ -2094,6 +2214,46 @@
       <x:c r="B36" s="69"/>
       <x:c r="C36" s="69"/>
       <x:c r="D36" s="69"/>
+    </x:row>
+    <x:row r="37" ht="42" customHeight="1">
+      <x:c r="A37" s="92" t="str">
+        <x:v>15. The delivery manager keeps its turn active with a real bounded wait while workers run. It may finish only after terminal handbacks or explicit transfer to another live supervisor.</x:v>
+      </x:c>
+      <x:c r="B37" s="69"/>
+      <x:c r="C37" s="69"/>
+      <x:c r="D37" s="69"/>
+    </x:row>
+    <x:row r="38" ht="42" customHeight="1">
+      <x:c r="A38" s="92" t="str">
+        <x:v>16. External provider streams are drained outside manager context. Retrieve compact lifecycle changes and the mechanically extracted final assistant result, not accumulated raw output.</x:v>
+      </x:c>
+      <x:c r="B38" s="69"/>
+      <x:c r="C38" s="69"/>
+      <x:c r="D38" s="69"/>
+    </x:row>
+    <x:row r="39" ht="42" customHeight="1">
+      <x:c r="A39" s="92" t="str">
+        <x:v>17. A provider parent exit does not transfer writer ownership. Verify process tree, worktree command/CWD holders and provider background-agent registry before any replacement writer.</x:v>
+      </x:c>
+      <x:c r="B39" s="69"/>
+      <x:c r="C39" s="69"/>
+      <x:c r="D39" s="69"/>
+    </x:row>
+    <x:row r="40" ht="42" customHeight="1">
+      <x:c r="A40" s="92" t="str">
+        <x:v>18. Stop Claude after two consecutive no-progress auto-compactions; checkpoint and use one fresh narrow retry rather than resuming the thrashing session.</x:v>
+      </x:c>
+      <x:c r="B40" s="69"/>
+      <x:c r="C40" s="69"/>
+      <x:c r="D40" s="69"/>
+    </x:row>
+    <x:row r="41" ht="42" customHeight="1">
+      <x:c r="A41" s="92" t="str">
+        <x:v>19. Owner concurrency exceptions are finite and journalled after an occupancy probe; leads and managers cannot self-authorize them.</x:v>
+      </x:c>
+      <x:c r="B41" s="69"/>
+      <x:c r="C41" s="69"/>
+      <x:c r="D41" s="69"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2112,6 +2272,11 @@
     <x:mergeCell ref="A34:D34"/>
     <x:mergeCell ref="A35:D35"/>
     <x:mergeCell ref="A36:D36"/>
+    <x:mergeCell ref="A37:D37"/>
+    <x:mergeCell ref="A38:D38"/>
+    <x:mergeCell ref="A39:D39"/>
+    <x:mergeCell ref="A40:D40"/>
+    <x:mergeCell ref="A41:D41"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2143,7 +2308,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>Policy source: Interchange policy v0.3.2</x:v>
+        <x:v>Policy source: Interchange policy v0.4.0</x:v>
       </x:c>
       <x:c r="B3" s="2" t="str">
         <x:v>Approved on</x:v>
@@ -2180,7 +2345,7 @@
         <x:v>How to apply it</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="44" customHeight="1">
+    <x:row r="8" ht="50" customHeight="1">
       <x:c r="A8" s="22" t="str">
         <x:v>Completion</x:v>
       </x:c>
@@ -2191,7 +2356,7 @@
         <x:v>Ready for review only; thinking, tools, quotes and stdout fragments cannot signal acceptance</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="44" customHeight="1">
+    <x:row r="9" ht="50" customHeight="1">
       <x:c r="A9" s="24" t="str">
         <x:v>First retrieval</x:v>
       </x:c>
@@ -2202,7 +2367,7 @@
         <x:v>Local process reader may receive events immediately; no repeated model prompts</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="44" customHeight="1">
+    <x:row r="10" ht="50" customHeight="1">
       <x:c r="A10" s="24" t="str">
         <x:v>Later retrieval</x:v>
       </x:c>
@@ -2213,7 +2378,7 @@
         <x:v>Completion or blocker events wake immediately; checks respect review/hard deadlines</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="44" customHeight="1">
+    <x:row r="11" ht="50" customHeight="1">
       <x:c r="A11" s="24" t="str">
         <x:v>Review deadline</x:v>
       </x:c>
@@ -2224,7 +2389,7 @@
         <x:v>Ask for evidence, blocker, remaining work and revised estimate once; no silent extension</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="44" customHeight="1">
+    <x:row r="12" ht="50" customHeight="1">
       <x:c r="A12" s="24" t="str">
         <x:v>Hard deadline</x:v>
       </x:c>
@@ -2235,7 +2400,7 @@
         <x:v>Interrupt; confirm termination and child-process state before replacing writer</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="44" customHeight="1">
+    <x:row r="13" ht="50" customHeight="1">
       <x:c r="A13" s="24" t="str">
         <x:v>Earlier review</x:v>
       </x:c>
@@ -2246,7 +2411,7 @@
         <x:v>Output volume and unchanged activity never reset task elapsed time</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="44" customHeight="1">
+    <x:row r="14" ht="50" customHeight="1">
       <x:c r="A14" s="24" t="str">
         <x:v>Recovery limit</x:v>
       </x:c>
@@ -2257,7 +2422,7 @@
         <x:v>Then delivery manager; one bounded independent diagnosis before owner escalation</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="44" customHeight="1">
+    <x:row r="15" ht="50" customHeight="1">
       <x:c r="A15" s="24" t="str">
         <x:v>Adaptive calibration</x:v>
       </x:c>
@@ -2268,7 +2433,7 @@
         <x:v>Weekly policy changes require owner approval; no automatic widening during runaway</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="44" customHeight="1">
+    <x:row r="16" ht="50" customHeight="1">
       <x:c r="A16" s="24" t="str">
         <x:v>Usage</x:v>
       </x:c>
@@ -2277,6 +2442,50 @@
       </x:c>
       <x:c r="C16" s="24" t="str">
         <x:v>Store input/output/cache/reasoning separately; do not assume provider counters are additive</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="50" customHeight="1">
+      <x:c r="A17" s="24" t="str">
+        <x:v>Supervision ownership</x:v>
+      </x:c>
+      <x:c r="B17" s="24" t="str">
+        <x:v>Manager turn remains active until terminal handback or explicit live-supervisor transfer</x:v>
+      </x:c>
+      <x:c r="C17" s="24" t="str">
+        <x:v>A wait timeout, session ID or future promise is not a continuation mechanism</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="50" customHeight="1">
+      <x:c r="A18" s="24" t="str">
+        <x:v>Output isolation</x:v>
+      </x:c>
+      <x:c r="B18" s="24" t="str">
+        <x:v>Adapter drains provider streams outside manager context</x:v>
+      </x:c>
+      <x:c r="C18" s="24" t="str">
+        <x:v>Manager receives lifecycle changes, final assistant result, usage, warnings and exit state only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="50" customHeight="1">
+      <x:c r="A19" s="24" t="str">
+        <x:v>Attempt ceilings</x:v>
+      </x:c>
+      <x:c r="B19" s="24" t="str">
+        <x:v>Finite wall-time and turn ceilings; token/cost ceilings where timely counters exist</x:v>
+      </x:c>
+      <x:c r="C19" s="24" t="str">
+        <x:v>Stop deterministic blockers; do not spend a ceiling rediscovering known failures</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="50" customHeight="1">
+      <x:c r="A20" s="24" t="str">
+        <x:v>Claude compaction</x:v>
+      </x:c>
+      <x:c r="B20" s="24" t="str">
+        <x:v>Stop after 2 consecutive auto-compactions without artifact, evidence or gate progress</x:v>
+      </x:c>
+      <x:c r="C20" s="24" t="str">
+        <x:v>Classify autocompact_thrashing as context/transport failure; retry fresh and narrow, never resume that context</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2310,7 +2519,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>Policy source: Interchange policy v0.3.2</x:v>
+        <x:v>Policy source: Interchange policy v0.4.0</x:v>
       </x:c>
       <x:c r="B3" s="2" t="str">
         <x:v>Approved on</x:v>
@@ -2345,195 +2554,226 @@
       </x:c>
       <x:c r="C7" s="2"/>
     </x:row>
-    <x:row r="8" ht="44" customHeight="1">
+    <x:row r="8" ht="48" customHeight="1">
       <x:c r="A8" s="22" t="str">
         <x:v>Workspaces</x:v>
       </x:c>
       <x:c r="B8" s="22" t="str">
         <x:v>Lead allocates one worktree per writable assignment per repository; one current writer; successors reuse after verified transfer</x:v>
       </x:c>
-      <x:c r="C8" s="2"/>
-    </x:row>
-    <x:row r="9" ht="44" customHeight="1">
+      <x:c r="C8"/>
+    </x:row>
+    <x:row r="9" ht="48" customHeight="1">
       <x:c r="A9" s="24" t="str">
         <x:v>Shared context</x:v>
       </x:c>
       <x:c r="B9" s="24" t="str">
         <x:v>Small universal rules + role/task-specific governing references at recorded revision; no mandatory full-vault read</x:v>
       </x:c>
-      <x:c r="C9" s="2"/>
-    </x:row>
-    <x:row r="10" ht="44" customHeight="1">
+      <x:c r="C9"/>
+    </x:row>
+    <x:row r="10" ht="48" customHeight="1">
       <x:c r="A10" s="24" t="str">
         <x:v>Authority</x:v>
       </x:c>
       <x:c r="B10" s="24" t="str">
         <x:v>MarvinaMiranda owns shared governance; adopted repo owns product meaning; GitHub owns live delivery state; code/tests own proof</x:v>
       </x:c>
-      <x:c r="C10" s="2"/>
-    </x:row>
-    <x:row r="11" ht="44" customHeight="1">
+      <x:c r="C10"/>
+    </x:row>
+    <x:row r="11" ht="48" customHeight="1">
       <x:c r="A11" s="24" t="str">
         <x:v>Personal settings</x:v>
       </x:c>
       <x:c r="B11" s="24" t="str">
         <x:v>Outside shared Git: account/pool bindings, local path map, budgets and session state; no embedded credentials</x:v>
       </x:c>
-      <x:c r="C11" s="2"/>
-    </x:row>
-    <x:row r="12" ht="44" customHeight="1">
+      <x:c r="C11"/>
+    </x:row>
+    <x:row r="12" ht="48" customHeight="1">
       <x:c r="A12" s="24" t="str">
         <x:v>Spending</x:v>
       </x:c>
       <x:c r="B12" s="24" t="str">
         <x:v>No extra purchases or automatic recharge; existing OpenCode Go allowance/balance may be used for Muse only</x:v>
       </x:c>
-      <x:c r="C12" s="2"/>
-    </x:row>
-    <x:row r="13" ht="44" customHeight="1">
+      <x:c r="C12"/>
+    </x:row>
+    <x:row r="13" ht="48" customHeight="1">
       <x:c r="A13" s="24" t="str">
         <x:v>Communication</x:v>
       </x:c>
       <x:c r="B13" s="24" t="str">
         <x:v>Caveman required for internal handovers with clarity exceptions; exact commands/evidence preserved; no guaranteed savings percentage</x:v>
       </x:c>
-      <x:c r="C13" s="2"/>
-    </x:row>
-    <x:row r="14" ht="44" customHeight="1">
+      <x:c r="C13"/>
+    </x:row>
+    <x:row r="14" ht="48" customHeight="1">
       <x:c r="A14" s="24" t="str">
         <x:v>Merge</x:v>
       </x:c>
       <x:c r="B14" s="24" t="str">
         <x:v>Only designated lead/delivery manager; exact test base; current SHA independently reviewed; all gates pass; reviewer approval normally required</x:v>
       </x:c>
-      <x:c r="C14" s="2"/>
-    </x:row>
-    <x:row r="15" ht="44" customHeight="1">
+      <x:c r="C14"/>
+    </x:row>
+    <x:row r="15" ht="48" customHeight="1">
       <x:c r="A15" s="24" t="str">
         <x:v>Review bypass</x:v>
       </x:c>
       <x:c r="B15" s="24" t="str">
         <x:v>Only required approval may be bypassed after passing independent Codex PR review and all other gates; record reason/SHA; no worker merge credentials</x:v>
       </x:c>
-      <x:c r="C15" s="2"/>
-    </x:row>
-    <x:row r="16" ht="44" customHeight="1">
+      <x:c r="C15"/>
+    </x:row>
+    <x:row r="16" ht="48" customHeight="1">
       <x:c r="A16" s="24" t="str">
         <x:v>Other environments</x:v>
       </x:c>
       <x:c r="B16" s="24" t="str">
         <x:v>uat/main, releases and separate deployment/security holds remain human-controlled</x:v>
       </x:c>
-      <x:c r="C16" s="2"/>
-    </x:row>
-    <x:row r="17" ht="44" customHeight="1">
+      <x:c r="C16"/>
+    </x:row>
+    <x:row r="17" ht="48" customHeight="1">
       <x:c r="A17" s="24" t="str">
         <x:v>Feedback</x:v>
       </x:c>
       <x:c r="B17" s="24" t="str">
         <x:v>Use GOV-0016 central LSN and GOV-0020 evaluation records; weekly evidence-based proposals require owner approval before changing policy</x:v>
       </x:c>
-      <x:c r="C17" s="2"/>
-    </x:row>
-    <x:row r="18" ht="44" customHeight="1">
+      <x:c r="C17"/>
+    </x:row>
+    <x:row r="18" ht="48" customHeight="1">
       <x:c r="A18" s="24" t="str">
         <x:v>Foreground scope</x:v>
       </x:c>
       <x:c r="B18" s="24" t="str">
-        <x:v>Codex active coordinates; durable results retained on exit; unattended Codex wakeup not yet implemented</x:v>
-      </x:c>
-      <x:c r="C18" s="2"/>
-    </x:row>
-    <x:row r="19" ht="44" customHeight="1">
+        <x:v>Manager keeps a real bounded wait active while workers run; final response requires terminal handbacks or explicit live-supervisor transfer; unattended wakeup not yet implemented</x:v>
+      </x:c>
+      <x:c r="C18"/>
+    </x:row>
+    <x:row r="19" ht="48" customHeight="1">
       <x:c r="A19" s="24" t="str">
+        <x:v>Concurrency exception</x:v>
+      </x:c>
+      <x:c r="B19" s="24" t="str">
+        <x:v>Only owner may grant a time-bounded journalled exception after occupancy probe; name scope, assignments, isolation, expiry and revocation; no extra spend or overlapping writers</x:v>
+      </x:c>
+      <x:c r="C19"/>
+    </x:row>
+    <x:row r="20" ht="48" customHeight="1">
+      <x:c r="A20" s="24" t="str">
         <x:v>Packaging</x:v>
       </x:c>
-      <x:c r="B19" s="24" t="str">
+      <x:c r="B20" s="24" t="str">
         <x:v>agent-skills repository, skills/interchange package; Caveman bundled unchanged with pinned source and MIT licence</x:v>
       </x:c>
-      <x:c r="C19" s="2"/>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="2"/>
-      <x:c r="B20" s="2"/>
-      <x:c r="C20" s="2"/>
+      <x:c r="C20"/>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="2"/>
-      <x:c r="B21" s="2"/>
-      <x:c r="C21" s="2"/>
+      <x:c r="A21"/>
+      <x:c r="B21"/>
+      <x:c r="C21"/>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="9" t="str">
+      <x:c r="A22"/>
+      <x:c r="B22"/>
+      <x:c r="C22"/>
+    </x:row>
+    <x:row r="23" ht="26" customHeight="1">
+      <x:c r="A23" s="180" t="str">
         <x:v>Recovery playbook</x:v>
       </x:c>
-      <x:c r="B22" s="10"/>
-      <x:c r="C22" s="11"/>
-    </x:row>
-    <x:row r="23" ht="26" customHeight="1">
-      <x:c r="A23" s="16" t="str">
+      <x:c r="B23" s="181"/>
+      <x:c r="C23" s="182"/>
+    </x:row>
+    <x:row r="24" ht="44" customHeight="1">
+      <x:c r="A24" s="188" t="str">
         <x:v>Failure</x:v>
       </x:c>
-      <x:c r="B23" s="17" t="str">
+      <x:c r="B24" s="189" t="str">
         <x:v>First action</x:v>
       </x:c>
-      <x:c r="C23" s="18" t="str">
+      <x:c r="C24" s="190" t="str">
         <x:v>Escalation</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" ht="44" customHeight="1">
-      <x:c r="A24" s="22" t="str">
+    <x:row r="25" ht="56" customHeight="1">
+      <x:c r="A25" s="22" t="str">
         <x:v>Network or CLI failure</x:v>
       </x:c>
-      <x:c r="B24" s="22" t="str">
+      <x:c r="B25" s="22" t="str">
         <x:v>Check process, session and artifacts; resume same session first</x:v>
       </x:c>
-      <x:c r="C24" s="22" t="str">
+      <x:c r="C25" s="22" t="str">
         <x:v>Transfer checkpoint to eligible house after original writer stopped</x:v>
       </x:c>
     </x:row>
-    <x:row r="25" ht="44" customHeight="1">
-      <x:c r="A25" s="24" t="str">
+    <x:row r="26" ht="56" customHeight="1">
+      <x:c r="A26" s="24" t="str">
         <x:v>Quota exhausted</x:v>
       </x:c>
-      <x:c r="B25" s="24" t="str">
+      <x:c r="B26" s="24" t="str">
         <x:v>Identify account and exact usage pool; preserve checkpoint</x:v>
       </x:c>
-      <x:c r="C25" s="24" t="str">
+      <x:c r="C26" s="24" t="str">
         <x:v>Eligible available house without extra spending</x:v>
       </x:c>
     </x:row>
-    <x:row r="26" ht="44" customHeight="1">
-      <x:c r="A26" s="24" t="str">
+    <x:row r="27" ht="56" customHeight="1">
+      <x:c r="A27" s="24" t="str">
         <x:v>Implementation loop</x:v>
       </x:c>
-      <x:c r="B26" s="24" t="str">
+      <x:c r="B27" s="24" t="str">
         <x:v>Stop repeated approach; evidence-based lead diagnosis</x:v>
       </x:c>
-      <x:c r="C26" s="24" t="str">
+      <x:c r="C27" s="24" t="str">
         <x:v>Different approved model/effort, then different house when justified</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="44" customHeight="1">
-      <x:c r="A27" s="24" t="str">
+    <x:row r="28" ht="56" customHeight="1">
+      <x:c r="A28" s="24" t="str">
         <x:v>Cross-repo or repeated blocker</x:v>
       </x:c>
-      <x:c r="B27" s="24" t="str">
+      <x:c r="B28" s="24" t="str">
         <x:v>War room with one incident lead and bounded investigators</x:v>
       </x:c>
-      <x:c r="C27" s="24" t="str">
+      <x:c r="C28" s="24" t="str">
         <x:v>Delivery manager; owner for unresolved decision or permission</x:v>
       </x:c>
     </x:row>
-    <x:row r="28" ht="44" customHeight="1">
-      <x:c r="A28" s="24" t="str">
+    <x:row r="29" ht="56" customHeight="1">
+      <x:c r="A29" s="24" t="str">
         <x:v>Marker missing or mismatched</x:v>
       </x:c>
-      <x:c r="B28" s="24" t="str">
+      <x:c r="B29" s="24" t="str">
         <x:v>Treat run as incomplete; inspect stored final result and exit</x:v>
       </x:c>
-      <x:c r="C28" s="24" t="str">
+      <x:c r="C29" s="24" t="str">
         <x:v>Recover session; never rerun writes blindly</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="56" customHeight="1">
+      <x:c r="A30" s="24" t="str">
+        <x:v>Claude autocompact thrashing</x:v>
+      </x:c>
+      <x:c r="B30" s="24" t="str">
+        <x:v>After 2 consecutive no-progress auto-compactions, checkpoint and stop before a third</x:v>
+      </x:c>
+      <x:c r="C30" s="24" t="str">
+        <x:v>Verify process tree, worktree holders and Claude background-agent registry; retry once with a fresh narrow packet and bounded larger context</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="56" customHeight="1">
+      <x:c r="A31" s="24" t="str">
+        <x:v>Abnormal provider parent exit</x:v>
+      </x:c>
+      <x:c r="B31" s="24" t="str">
+        <x:v>Retain writer ownership until parent/descendants, worktree command/CWD holders and provider background-agent registry are all clear</x:v>
+      </x:c>
+      <x:c r="C31" s="24" t="str">
+        <x:v>Inspect worktree state and locks; transfer only after timestamped evidence, otherwise lead resolves</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
feat(interchange): separate brains from workers
</commit_message>
<xml_diff>
--- a/outputs/interchange-design/interchange.xlsx
+++ b/outputs/interchange-design/interchange.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profiles" sheetId="1" r:id="Rdb05d2334a084321"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Routing" sheetId="2" r:id="R4a8f0ce1555046dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monitoring" sheetId="3" r:id="R22d28bd2e77f4b53"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Recovery" sheetId="4" r:id="Rc554ec4257a34146"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profiles" sheetId="1" r:id="R54bb1c1b109c4a81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Routing" sheetId="2" r:id="Ra5fa34cf7b594df6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monitoring" sheetId="3" r:id="R9861e40f1bfe4770"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Recovery" sheetId="4" r:id="Re075d54395954ed3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -55,7 +55,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="39">
+  <x:fills count="51">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -85,6 +85,66 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFCE4D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -320,7 +380,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="191">
+  <x:cellXfs count="251">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -792,6 +852,144 @@
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="38" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="39" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="39" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="40" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="40" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="39" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="41" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="41" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="41" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="41" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="41" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="42" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="42" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="42" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="42" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="42" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="42" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="42" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="42" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="43" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="43" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="44" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="44" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="44" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="43" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="45" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="45" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="45" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="45" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="45" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="46" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="46" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="46" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="46" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="46" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="46" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="46" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="46" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="47" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="47" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="48" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="48" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="47" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="49" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="49" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="49" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="50" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="50" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="50" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1036,7 +1234,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>Policy source: Interchange policy v0.4.0</x:v>
+        <x:v>Policy source: Interchange policy v0.6.0</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -1044,7 +1242,7 @@
         <x:v>Approved on</x:v>
       </x:c>
       <x:c r="E3" s="5" t="n">
-        <x:v>46274</x:v>
+        <x:v>46278</x:v>
       </x:c>
       <x:c r="F3" s="2"/>
       <x:c r="G3" s="4" t="str">
@@ -1110,8 +1308,8 @@
         <x:v>Allowed fixed profiles</x:v>
       </x:c>
       <x:c r="B8" s="30" t="n">
-        <x:f>COUNTIFS($G$16:$G$36,"Allowed fixed profile")</x:f>
-        <x:v>21</x:v>
+        <x:f>COUNTIFS($G$16:$G$40,"Allowed fixed profile")</x:f>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C8" s="22" t="str">
         <x:v>Select only when the assigned role, pool, and task fit.</x:v>
@@ -1128,7 +1326,7 @@
         <x:v>Smoke-tested fixed profiles</x:v>
       </x:c>
       <x:c r="B9" s="31" t="n">
-        <x:f>COUNTIFS($H$16:$H$36,"Smoke-tested")</x:f>
+        <x:f>COUNTIFS($H$16:$H$40,"Smoke-tested")</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="C9" s="24" t="str">
@@ -1146,7 +1344,7 @@
         <x:v>Documented profiles pending exact runtime check</x:v>
       </x:c>
       <x:c r="B10" s="32" t="n">
-        <x:f>COUNTIFS($H$16:$H$36,"CLI model and effort documented; exact runtime unverified")+COUNTIFS($H$16:$H$36,"Profile documented; exact runtime unverified")</x:f>
+        <x:f>COUNTIFS($H$16:$H$40,"CLI model and effort documented; exact runtime unverified")+COUNTIFS($H$16:$H$40,"Profile documented; exact runtime unverified")</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="C10" s="24" t="str">
@@ -1254,15 +1452,15 @@
         <x:v>high</x:v>
       </x:c>
       <x:c r="E16" s="22" t="str">
-        <x:v>delivery manager: approved alternative with explicit handover when switching houses</x:v>
+        <x:v>delivery manager: mechanical coordination and continuity; route unresolved interpretation to an approved brain</x:v>
       </x:c>
       <x:c r="F16" s="34" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G16" s="173" t="str">
+      <x:c r="G16" s="233" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H16" s="175" t="str">
+      <x:c r="H16" s="235" t="str">
         <x:v>Profile documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I16" s="22" t="str">
@@ -1283,15 +1481,15 @@
         <x:v>high</x:v>
       </x:c>
       <x:c r="E17" s="24" t="str">
-        <x:v>delivery manager: approved alternative when starting with Sol high</x:v>
+        <x:v>delivery manager and default product/architecture brain</x:v>
       </x:c>
       <x:c r="F17" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G17" s="174" t="str">
+      <x:c r="G17" s="234" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H17" s="176" t="str">
+      <x:c r="H17" s="236" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I17" s="24" t="str">
@@ -1312,15 +1510,15 @@
         <x:v>medium</x:v>
       </x:c>
       <x:c r="E18" s="24" t="str">
-        <x:v>delivery manager</x:v>
+        <x:v>delivery manager and brain for unusually large cross-workstream ambiguity</x:v>
       </x:c>
       <x:c r="F18" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G18" s="174" t="str">
+      <x:c r="G18" s="234" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H18" s="176" t="str">
+      <x:c r="H18" s="236" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I18" s="24" t="str">
@@ -1341,15 +1539,15 @@
         <x:v>medium</x:v>
       </x:c>
       <x:c r="E19" s="24" t="str">
-        <x:v>lead: high ambiguity or cross-workstream architecture</x:v>
+        <x:v>brain lead: unusually large ambiguity or cross-workstream architecture</x:v>
       </x:c>
       <x:c r="F19" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G19" s="174" t="str">
+      <x:c r="G19" s="234" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H19" s="176" t="str">
+      <x:c r="H19" s="236" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I19" s="24" t="str">
@@ -1370,15 +1568,15 @@
         <x:v>medium</x:v>
       </x:c>
       <x:c r="E20" s="24" t="str">
-        <x:v>lead: bounded architecture and moderate coupling</x:v>
+        <x:v>mechanical workstream coordinator for settled contracts; no interpretive authority</x:v>
       </x:c>
       <x:c r="F20" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G20" s="174" t="str">
+      <x:c r="G20" s="234" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H20" s="176" t="str">
+      <x:c r="H20" s="236" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I20" s="24" t="str">
@@ -1399,15 +1597,15 @@
         <x:v>high</x:v>
       </x:c>
       <x:c r="E21" s="24" t="str">
-        <x:v>lead: consequential design and risk</x:v>
+        <x:v>default brain lead: product, architecture, consequence and tradeoff decisions</x:v>
       </x:c>
       <x:c r="F21" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G21" s="174" t="str">
+      <x:c r="G21" s="234" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H21" s="176" t="str">
+      <x:c r="H21" s="236" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I21" s="24" t="str">
@@ -1416,306 +1614,306 @@
     </x:row>
     <x:row r="22" ht="38" customHeight="1">
       <x:c r="A22" s="24" t="str">
-        <x:v>lead-terra-xhigh</x:v>
+        <x:v>reviewer-sol-high</x:v>
       </x:c>
       <x:c r="B22" s="24" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="C22" s="24" t="str">
-        <x:v>gpt-5.6-terra</x:v>
+        <x:v>gpt-5.6-sol</x:v>
       </x:c>
       <x:c r="D22" s="24" t="str">
-        <x:v>xhigh</x:v>
+        <x:v>high</x:v>
       </x:c>
       <x:c r="E22" s="24" t="str">
-        <x:v>lead: defined contracts and bounded workstream</x:v>
+        <x:v>independent semantic and risk review brain; no implementation or self-review</x:v>
       </x:c>
       <x:c r="F22" s="35" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="G22" s="174" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="G22" s="234" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H22" s="176" t="str">
+      <x:c r="H22" s="236" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I22" s="24" t="str">
-        <x:v>Supported by current tool metadata; routing uncalibrated</x:v>
+        <x:v>Sol high review found meaning-level defects in governed delivery; reviewer remains independent of writer and current-head bound</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="38" customHeight="1">
       <x:c r="A23" s="24" t="str">
-        <x:v>lead-terra-max</x:v>
+        <x:v>reviewer-astra-medium</x:v>
       </x:c>
       <x:c r="B23" s="24" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="C23" s="24" t="str">
-        <x:v>gpt-5.6-terra</x:v>
+        <x:v>gpt-6-astra</x:v>
       </x:c>
       <x:c r="D23" s="24" t="str">
-        <x:v>max</x:v>
+        <x:v>medium</x:v>
       </x:c>
       <x:c r="E23" s="24" t="str">
-        <x:v>lead: defined architecture with difficult integration</x:v>
+        <x:v>independent semantic review brain for unusually large cross-workstream scope; no implementation or self-review</x:v>
       </x:c>
       <x:c r="F23" s="35" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="G23" s="174" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="G23" s="234" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H23" s="176" t="str">
+      <x:c r="H23" s="236" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I23" s="24" t="str">
-        <x:v>Supported by current tool metadata; routing uncalibrated</x:v>
+        <x:v>Supported by current tool metadata; reviewer routing uncalibrated</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="38" customHeight="1">
       <x:c r="A24" s="24" t="str">
-        <x:v>worker-luna-xhigh</x:v>
+        <x:v>lead-terra-xhigh</x:v>
       </x:c>
       <x:c r="B24" s="24" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="C24" s="24" t="str">
-        <x:v>gpt-5.6-luna</x:v>
+        <x:v>gpt-5.6-terra</x:v>
       </x:c>
       <x:c r="D24" s="24" t="str">
         <x:v>xhigh</x:v>
       </x:c>
       <x:c r="E24" s="24" t="str">
-        <x:v>bounded leaf exploration or explicit small change</x:v>
+        <x:v>mechanical lead: defined contracts and bounded workstream; escalate interpretation</x:v>
       </x:c>
       <x:c r="F24" s="35" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="G24" s="174" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G24" s="234" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H24" s="176" t="str">
+      <x:c r="H24" s="236" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I24" s="24" t="str">
-        <x:v>Supported; lower effort forbidden by owner</x:v>
+        <x:v>Supported by current tool metadata; routing uncalibrated</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="38" customHeight="1">
       <x:c r="A25" s="24" t="str">
-        <x:v>worker-luna-max</x:v>
+        <x:v>lead-terra-max</x:v>
       </x:c>
       <x:c r="B25" s="24" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="C25" s="24" t="str">
-        <x:v>gpt-5.6-luna</x:v>
+        <x:v>gpt-5.6-terra</x:v>
       </x:c>
       <x:c r="D25" s="24" t="str">
         <x:v>max</x:v>
       </x:c>
       <x:c r="E25" s="24" t="str">
-        <x:v>bounded leaf with denser evidence</x:v>
+        <x:v>mechanical lead: difficult integration within defined architecture; escalate interpretation</x:v>
       </x:c>
       <x:c r="F25" s="35" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="G25" s="174" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G25" s="234" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H25" s="176" t="str">
+      <x:c r="H25" s="236" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I25" s="24" t="str">
-        <x:v>Supported; lower effort forbidden by owner</x:v>
+        <x:v>Supported by current tool metadata; routing uncalibrated</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="38" customHeight="1">
       <x:c r="A26" s="24" t="str">
-        <x:v>worker-terra-xhigh</x:v>
+        <x:v>worker-luna-xhigh</x:v>
       </x:c>
       <x:c r="B26" s="24" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="C26" s="24" t="str">
-        <x:v>gpt-5.6-terra</x:v>
+        <x:v>gpt-5.6-luna</x:v>
       </x:c>
       <x:c r="D26" s="24" t="str">
         <x:v>xhigh</x:v>
       </x:c>
       <x:c r="E26" s="24" t="str">
-        <x:v>bounded builder or independent verifier</x:v>
+        <x:v>bounded leaf exploration or explicit small change</x:v>
       </x:c>
       <x:c r="F26" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G26" s="174" t="str">
+      <x:c r="G26" s="234" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H26" s="176" t="str">
+      <x:c r="H26" s="236" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I26" s="24" t="str">
-        <x:v>Supported; role assignment separate from model</x:v>
+        <x:v>Supported; lower effort forbidden by owner</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="38" customHeight="1">
       <x:c r="A27" s="24" t="str">
-        <x:v>worker-muse-xhigh</x:v>
+        <x:v>worker-luna-max</x:v>
       </x:c>
       <x:c r="B27" s="24" t="str">
-        <x:v>OpenCode / Go pool</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="C27" s="24" t="str">
-        <x:v>opencode-go/muse-spark-1.3-contributor</x:v>
+        <x:v>gpt-5.6-luna</x:v>
       </x:c>
       <x:c r="D27" s="24" t="str">
-        <x:v>xhigh</x:v>
+        <x:v>max</x:v>
       </x:c>
       <x:c r="E27" s="24" t="str">
-        <x:v>preferred initial cheap leaf candidate</x:v>
+        <x:v>bounded leaf with denser evidence</x:v>
       </x:c>
       <x:c r="F27" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G27" s="174" t="str">
+      <x:c r="G27" s="234" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H27" s="177" t="str">
-        <x:v>Smoke-tested</x:v>
+      <x:c r="H27" s="236" t="str">
+        <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I27" s="24" t="str">
-        <x:v>CLI send/resume/recall smoke-tested; quality advantage is owner hypothesis</x:v>
+        <x:v>Supported; lower effort forbidden by owner</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="38" customHeight="1">
       <x:c r="A28" s="24" t="str">
-        <x:v>worker-grok-high</x:v>
+        <x:v>worker-terra-xhigh</x:v>
       </x:c>
       <x:c r="B28" s="24" t="str">
-        <x:v>Grok</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="C28" s="24" t="str">
-        <x:v>grok-4.6</x:v>
+        <x:v>gpt-5.6-terra</x:v>
       </x:c>
       <x:c r="D28" s="24" t="str">
-        <x:v>high</x:v>
+        <x:v>xhigh</x:v>
       </x:c>
       <x:c r="E28" s="24" t="str">
-        <x:v>primary low/mid complexity developer</x:v>
+        <x:v>bounded builder or independent verifier</x:v>
       </x:c>
       <x:c r="F28" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G28" s="174" t="str">
+      <x:c r="G28" s="234" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H28" s="176" t="str">
-        <x:v>CLI model and effort documented; exact runtime unverified</x:v>
+      <x:c r="H28" s="236" t="str">
+        <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I28" s="24" t="str">
-        <x:v>grok models lists grok-4.6; effort flags documented; exact profile smoke test pending</x:v>
+        <x:v>Supported; role assignment separate from model</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="38" customHeight="1">
       <x:c r="A29" s="24" t="str">
-        <x:v>worker-grok-xhigh</x:v>
+        <x:v>worker-muse-xhigh</x:v>
       </x:c>
       <x:c r="B29" s="24" t="str">
-        <x:v>Grok</x:v>
+        <x:v>OpenCode / Go pool</x:v>
       </x:c>
       <x:c r="C29" s="24" t="str">
-        <x:v>grok-4.6</x:v>
+        <x:v>opencode-go/muse-spark-1.3-contributor</x:v>
       </x:c>
       <x:c r="D29" s="24" t="str">
         <x:v>xhigh</x:v>
       </x:c>
       <x:c r="E29" s="24" t="str">
-        <x:v>primary upper-mid complexity developer</x:v>
+        <x:v>light mechanical and read/seek leaf: repository search, localization, evidence, narrow checks or small explicit edits</x:v>
       </x:c>
       <x:c r="F29" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G29" s="174" t="str">
+      <x:c r="G29" s="234" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H29" s="176" t="str">
-        <x:v>CLI model and effort documented; exact runtime unverified</x:v>
+      <x:c r="H29" s="237" t="str">
+        <x:v>Smoke-tested</x:v>
       </x:c>
       <x:c r="I29" s="24" t="str">
-        <x:v>grok models lists grok-4.6; effort flags documented; exact profile smoke test pending</x:v>
+        <x:v>CLI send/resume/recall smoke-tested; quality advantage is owner hypothesis</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="38" customHeight="1">
       <x:c r="A30" s="24" t="str">
-        <x:v>worker-opus-medium</x:v>
+        <x:v>worker-deepseek-flash-high</x:v>
       </x:c>
       <x:c r="B30" s="24" t="str">
-        <x:v>Claude</x:v>
+        <x:v>OpenCode / Go pool</x:v>
       </x:c>
       <x:c r="C30" s="24" t="str">
-        <x:v>claude-opus-5</x:v>
+        <x:v>opencode-go/deepseek-v4.1-flash</x:v>
       </x:c>
       <x:c r="D30" s="24" t="str">
-        <x:v>medium</x:v>
+        <x:v>high</x:v>
       </x:c>
       <x:c r="E30" s="24" t="str">
-        <x:v>primary low/mid and upper-mid complexity developer</x:v>
+        <x:v>preferred bounded implementation worker with clear acceptance and settled architecture</x:v>
       </x:c>
       <x:c r="F30" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G30" s="174" t="str">
+      <x:c r="G30" s="234" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H30" s="176" t="str">
-        <x:v>Profile documented; exact runtime unverified</x:v>
+      <x:c r="H30" s="236" t="str">
+        <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I30" s="24" t="str">
-        <x:v>Full model ID and effort documented; exact profile runtime identity and smoke test pending</x:v>
+        <x:v>Eleven governed DeepSeek Flash runs across two repositories; high is the approved default. Independent semantic review remains mandatory.</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="38" customHeight="1">
       <x:c r="A31" s="24" t="str">
-        <x:v>worker-opus-high</x:v>
+        <x:v>worker-deepseek-flash-max</x:v>
       </x:c>
       <x:c r="B31" s="24" t="str">
-        <x:v>Claude</x:v>
+        <x:v>OpenCode / Go pool</x:v>
       </x:c>
       <x:c r="C31" s="24" t="str">
-        <x:v>claude-opus-5</x:v>
+        <x:v>opencode-go/deepseek-v4.1-flash</x:v>
       </x:c>
       <x:c r="D31" s="24" t="str">
-        <x:v>high</x:v>
+        <x:v>max</x:v>
       </x:c>
       <x:c r="E31" s="24" t="str">
-        <x:v>primary high complexity developer</x:v>
+        <x:v>mechanical implementation of a novel public contract shape already settled by an approved brain</x:v>
       </x:c>
       <x:c r="F31" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G31" s="174" t="str">
+      <x:c r="G31" s="234" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H31" s="176" t="str">
-        <x:v>Profile documented; exact runtime unverified</x:v>
+      <x:c r="H31" s="236" t="str">
+        <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I31" s="24" t="str">
-        <x:v>Full model ID and effort documented; exact profile runtime identity and smoke test pending</x:v>
+        <x:v>One evaluated max assignment showed value on novel public identity work; current policy restricts max to mechanical implementation after a brain settles the shape. Independent semantic review remains mandatory.</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="38" customHeight="1">
       <x:c r="A32" s="24" t="str">
-        <x:v>worker-sol-medium</x:v>
+        <x:v>worker-grok-high</x:v>
       </x:c>
       <x:c r="B32" s="24" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Grok</x:v>
       </x:c>
       <x:c r="C32" s="24" t="str">
-        <x:v>gpt-5.6-sol</x:v>
+        <x:v>grok-4.6</x:v>
       </x:c>
       <x:c r="D32" s="24" t="str">
-        <x:v>medium</x:v>
+        <x:v>high</x:v>
       </x:c>
       <x:c r="E32" s="24" t="str">
         <x:v>primary low/mid complexity developer</x:v>
@@ -1723,129 +1921,245 @@
       <x:c r="F32" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G32" s="174" t="str">
+      <x:c r="G32" s="234" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H32" s="176" t="str">
-        <x:v>Supported by metadata; routing unverified</x:v>
+      <x:c r="H32" s="236" t="str">
+        <x:v>CLI model and effort documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I32" s="24" t="str">
-        <x:v>Current tool metadata supports profile; task-class performance uncalibrated</x:v>
+        <x:v>grok models lists grok-4.6; effort flags documented; exact profile smoke test pending</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="38" customHeight="1">
       <x:c r="A33" s="24" t="str">
-        <x:v>worker-sol-high</x:v>
+        <x:v>worker-grok-xhigh</x:v>
       </x:c>
       <x:c r="B33" s="24" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Grok</x:v>
       </x:c>
       <x:c r="C33" s="24" t="str">
-        <x:v>gpt-5.6-sol</x:v>
+        <x:v>grok-4.6</x:v>
       </x:c>
       <x:c r="D33" s="24" t="str">
-        <x:v>high</x:v>
+        <x:v>xhigh</x:v>
       </x:c>
       <x:c r="E33" s="24" t="str">
-        <x:v>primary high complexity developer</x:v>
+        <x:v>primary upper-mid complexity developer</x:v>
       </x:c>
       <x:c r="F33" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G33" s="174" t="str">
+      <x:c r="G33" s="234" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H33" s="176" t="str">
-        <x:v>Supported by metadata; routing unverified</x:v>
+      <x:c r="H33" s="236" t="str">
+        <x:v>CLI model and effort documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I33" s="24" t="str">
-        <x:v>Current tool metadata supports profile; task-class performance uncalibrated</x:v>
+        <x:v>grok models lists grok-4.6; effort flags documented; exact profile smoke test pending</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="38" customHeight="1">
       <x:c r="A34" s="24" t="str">
-        <x:v>worker-terra-max</x:v>
+        <x:v>worker-opus-medium</x:v>
       </x:c>
       <x:c r="B34" s="24" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Claude</x:v>
       </x:c>
       <x:c r="C34" s="24" t="str">
-        <x:v>gpt-5.6-terra</x:v>
+        <x:v>claude-opus-5</x:v>
       </x:c>
       <x:c r="D34" s="24" t="str">
-        <x:v>max</x:v>
+        <x:v>medium</x:v>
       </x:c>
       <x:c r="E34" s="24" t="str">
-        <x:v>demanding implementation with settled contracts and bounded scope</x:v>
+        <x:v>primary low/mid and upper-mid complexity developer</x:v>
       </x:c>
       <x:c r="F34" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G34" s="174" t="str">
+      <x:c r="G34" s="234" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H34" s="176" t="str">
-        <x:v>Supported by metadata; routing unverified</x:v>
+      <x:c r="H34" s="236" t="str">
+        <x:v>Profile documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I34" s="24" t="str">
-        <x:v>Current tool metadata supports profile; effort is not a substitute for resolving ambiguity</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35" ht="76" customHeight="1">
+        <x:v>Full model ID and effort documented; exact profile runtime identity and smoke test pending</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="38" customHeight="1">
       <x:c r="A35" s="24" t="str">
-        <x:v>brainstorm-fable-medium</x:v>
+        <x:v>worker-opus-high</x:v>
       </x:c>
       <x:c r="B35" s="24" t="str">
         <x:v>Claude</x:v>
       </x:c>
       <x:c r="C35" s="24" t="str">
-        <x:v>claude-fable-5-1</x:v>
+        <x:v>claude-opus-5</x:v>
       </x:c>
       <x:c r="D35" s="24" t="str">
-        <x:v>medium</x:v>
+        <x:v>high</x:v>
       </x:c>
       <x:c r="E35" s="24" t="str">
-        <x:v>new-product ideation and brainstorming</x:v>
+        <x:v>primary high complexity developer</x:v>
       </x:c>
       <x:c r="F35" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G35" s="174" t="str">
+      <x:c r="G35" s="234" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H35" s="176" t="str">
+      <x:c r="H35" s="236" t="str">
         <x:v>Profile documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I35" s="24" t="str">
-        <x:v>Official model/effort documentation; exact runtime and included-plan eligibility not verified</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="36" ht="76" customHeight="1">
+        <x:v>Full model ID and effort documented; exact profile runtime identity and smoke test pending</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="38" customHeight="1">
       <x:c r="A36" s="24" t="str">
-        <x:v>brainstorm-astra-medium</x:v>
+        <x:v>worker-sol-medium</x:v>
       </x:c>
       <x:c r="B36" s="24" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="C36" s="24" t="str">
-        <x:v>gpt-6-astra</x:v>
+        <x:v>gpt-5.6-sol</x:v>
       </x:c>
       <x:c r="D36" s="24" t="str">
         <x:v>medium</x:v>
       </x:c>
       <x:c r="E36" s="24" t="str">
-        <x:v>new-product ideation and brainstorming</x:v>
+        <x:v>primary low/mid complexity developer</x:v>
       </x:c>
       <x:c r="F36" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G36" s="174" t="str">
+      <x:c r="G36" s="234" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H36" s="176" t="str">
+      <x:c r="H36" s="236" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I36" s="24" t="str">
+        <x:v>Current tool metadata supports profile; task-class performance uncalibrated</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="38" customHeight="1">
+      <x:c r="A37" s="24" t="str">
+        <x:v>worker-sol-high</x:v>
+      </x:c>
+      <x:c r="B37" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="C37" s="24" t="str">
+        <x:v>gpt-5.6-sol</x:v>
+      </x:c>
+      <x:c r="D37" s="24" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="E37" s="24" t="str">
+        <x:v>primary high complexity developer</x:v>
+      </x:c>
+      <x:c r="F37" s="35" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="G37" s="234" t="str">
+        <x:v>Allowed fixed profile</x:v>
+      </x:c>
+      <x:c r="H37" s="236" t="str">
+        <x:v>Supported by metadata; routing unverified</x:v>
+      </x:c>
+      <x:c r="I37" s="24" t="str">
+        <x:v>Current tool metadata supports profile; task-class performance uncalibrated</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="38" customHeight="1">
+      <x:c r="A38" s="24" t="str">
+        <x:v>worker-terra-max</x:v>
+      </x:c>
+      <x:c r="B38" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="C38" s="24" t="str">
+        <x:v>gpt-5.6-terra</x:v>
+      </x:c>
+      <x:c r="D38" s="24" t="str">
+        <x:v>max</x:v>
+      </x:c>
+      <x:c r="E38" s="24" t="str">
+        <x:v>demanding implementation with settled contracts and bounded scope</x:v>
+      </x:c>
+      <x:c r="F38" s="35" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="G38" s="234" t="str">
+        <x:v>Allowed fixed profile</x:v>
+      </x:c>
+      <x:c r="H38" s="236" t="str">
+        <x:v>Supported by metadata; routing unverified</x:v>
+      </x:c>
+      <x:c r="I38" s="24" t="str">
+        <x:v>Current tool metadata supports profile; effort is not a substitute for resolving ambiguity</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="76" customHeight="1">
+      <x:c r="A39" s="24" t="str">
+        <x:v>brainstorm-fable-medium</x:v>
+      </x:c>
+      <x:c r="B39" s="24" t="str">
+        <x:v>Claude</x:v>
+      </x:c>
+      <x:c r="C39" s="24" t="str">
+        <x:v>claude-fable-5-1</x:v>
+      </x:c>
+      <x:c r="D39" s="24" t="str">
+        <x:v>medium</x:v>
+      </x:c>
+      <x:c r="E39" s="24" t="str">
+        <x:v>product-ideation brain; no implementation; included-plan/no-extra-cost preflight required</x:v>
+      </x:c>
+      <x:c r="F39" s="35" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="G39" s="234" t="str">
+        <x:v>Allowed fixed profile</x:v>
+      </x:c>
+      <x:c r="H39" s="236" t="str">
+        <x:v>Profile documented; exact runtime unverified</x:v>
+      </x:c>
+      <x:c r="I39" s="24" t="str">
+        <x:v>Official model/effort documentation; exact runtime and included-plan eligibility not verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="76" customHeight="1">
+      <x:c r="A40" s="24" t="str">
+        <x:v>brainstorm-astra-medium</x:v>
+      </x:c>
+      <x:c r="B40" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="C40" s="24" t="str">
+        <x:v>gpt-6-astra</x:v>
+      </x:c>
+      <x:c r="D40" s="24" t="str">
+        <x:v>medium</x:v>
+      </x:c>
+      <x:c r="E40" s="24" t="str">
+        <x:v>product-ideation brain for unusually large or cross-workstream concepts</x:v>
+      </x:c>
+      <x:c r="F40" s="35" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="G40" s="234" t="str">
+        <x:v>Allowed fixed profile</x:v>
+      </x:c>
+      <x:c r="H40" s="236" t="str">
+        <x:v>Supported by metadata; routing unverified</x:v>
+      </x:c>
+      <x:c r="I40" s="24" t="str">
         <x:v>Current tool metadata supports profile; no comparative ideation benchmark</x:v>
       </x:c>
     </x:row>
@@ -1883,14 +2197,14 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>Policy source: Interchange policy v0.4.0</x:v>
+        <x:v>Policy source: Interchange policy v0.6.0</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2" t="str">
         <x:v>Approved on</x:v>
       </x:c>
       <x:c r="D3" s="5" t="n">
-        <x:v>46274</x:v>
+        <x:v>46278</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -1943,193 +2257,211 @@
     </x:row>
     <x:row r="9" ht="46" customHeight="1">
       <x:c r="A9" s="24" t="str">
-        <x:v>One direct lookup</x:v>
+        <x:v>Product, behavior or architecture judgment</x:v>
       </x:c>
       <x:c r="B9" s="24" t="str">
-        <x:v>Local search/tool</x:v>
+        <x:v>lead-sol-high or dm-sol-high</x:v>
       </x:c>
       <x:c r="C9" s="24" t="str">
-        <x:v>Bounded explorer only if context merits it</x:v>
+        <x:v>lead-astra-medium or dm-astra-medium for unusually large cross-workstream ambiguity</x:v>
       </x:c>
       <x:c r="D9" s="24" t="str">
-        <x:v>Avoid dispatch and repeated context overhead</x:v>
+        <x:v>Only approved brain profiles interpret missing requirements, choose tradeoffs or settle contracts</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="46" customHeight="1">
       <x:c r="A10" s="24" t="str">
-        <x:v>Small bounded support task</x:v>
+        <x:v>One direct lookup</x:v>
       </x:c>
       <x:c r="B10" s="24" t="str">
-        <x:v>worker-muse-xhigh</x:v>
+        <x:v>Local search/tool when immediate; worker-muse-xhigh when parallel dispatch frees the brain or is faster overall</x:v>
       </x:c>
       <x:c r="C10" s="24" t="str">
-        <x:v>worker-luna-xhigh; worker-luna-max when evidence density warrants</x:v>
+        <x:v>worker-luna-xhigh for bounded read-only evidence when Muse is unavailable</x:v>
       </x:c>
       <x:c r="D10" s="24" t="str">
-        <x:v>Exploration, explicit small edits or test preparation; retain lower-cost leaf lane</x:v>
+        <x:v>Count startup, supervision and handback overhead; delegate when it improves accepted-result time or cost</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="46" customHeight="1">
       <x:c r="A11" s="24" t="str">
-        <x:v>Low/mid complexity development</x:v>
+        <x:v>Light mechanical and read/seek task</x:v>
       </x:c>
       <x:c r="B11" s="24" t="str">
-        <x:v>worker-grok-high; worker-opus-medium; worker-terra-xhigh; worker-sol-medium</x:v>
+        <x:v>worker-muse-xhigh</x:v>
       </x:c>
       <x:c r="C11" s="24" t="str">
-        <x:v>Another eligible profile from this pool</x:v>
+        <x:v>worker-luna-xhigh; worker-luna-max when evidence density warrants</x:v>
       </x:c>
       <x:c r="D11" s="24" t="str">
-        <x:v>Preferred pool, not fixed rank: clear acceptance, known patterns, bounded dependencies; choose fit then speed and available quota</x:v>
+        <x:v>Repository search, localization, evidence collection, narrow checks and small explicit edits; no interpretation</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="46" customHeight="1">
       <x:c r="A12" s="24" t="str">
-        <x:v>Upper-mid complexity development</x:v>
+        <x:v>Low/mid complexity development</x:v>
       </x:c>
       <x:c r="B12" s="24" t="str">
-        <x:v>worker-grok-xhigh; worker-opus-medium</x:v>
+        <x:v>worker-deepseek-flash-high; worker-grok-high; worker-opus-medium; worker-terra-xhigh; worker-sol-medium</x:v>
       </x:c>
       <x:c r="C12" s="24" t="str">
-        <x:v>worker-sol-high or worker-opus-high when ambiguity or consequence warrants escalation</x:v>
+        <x:v>Another eligible profile from this pool</x:v>
       </x:c>
       <x:c r="D12" s="24" t="str">
-        <x:v>Difficult implementation within settled architecture; two primary choices are not claimed equal in capability</x:v>
+        <x:v>Settled behavior, objective acceptance and bounded dependencies; ambiguity already resolved by a brain</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="46" customHeight="1">
       <x:c r="A13" s="24" t="str">
-        <x:v>High complexity development</x:v>
+        <x:v>Upper-mid complexity development</x:v>
       </x:c>
       <x:c r="B13" s="24" t="str">
-        <x:v>worker-sol-high; worker-opus-high</x:v>
+        <x:v>worker-deepseek-flash-high; worker-grok-xhigh; worker-opus-medium</x:v>
       </x:c>
       <x:c r="C13" s="24" t="str">
-        <x:v>Lead/manager resolves architecture or scope before further execution</x:v>
+        <x:v>lead-sol-high resolves ambiguity or consequence; then choose worker-sol-high, worker-opus-high or another qualified mechanical profile</x:v>
       </x:c>
       <x:c r="D13" s="24" t="str">
-        <x:v>Substantial reasoning, sensitive boundaries or coupled contracts; keep mandatory independent risk review</x:v>
+        <x:v>Difficult mechanical implementation within settled architecture; return tradeoffs instead of choosing</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="46" customHeight="1">
       <x:c r="A14" s="24" t="str">
-        <x:v>Demanding but well-defined implementation</x:v>
+        <x:v>High complexity development</x:v>
       </x:c>
       <x:c r="B14" s="24" t="str">
-        <x:v>worker-terra-max</x:v>
+        <x:v>lead-sol-high resolves judgment; worker-opus-high or another qualified mechanical profile executes settled packets</x:v>
       </x:c>
       <x:c r="C14" s="24" t="str">
-        <x:v>High-complexity pool if evidence shows a reasoning blocker</x:v>
+        <x:v>lead-astra-medium resolves unusually large cross-workstream ambiguity before mechanical execution</x:v>
       </x:c>
       <x:c r="D14" s="24" t="str">
-        <x:v>Dense implementation or integration with exact contracts and tests; never assign to outlast a loop</x:v>
+        <x:v>Separate consequential decisions from implementation; independent review remains mandatory</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="46" customHeight="1">
       <x:c r="A15" s="24" t="str">
-        <x:v>Workstream with fixed contracts</x:v>
+        <x:v>Demanding but well-defined implementation</x:v>
       </x:c>
       <x:c r="B15" s="24" t="str">
-        <x:v>lead-terra-xhigh</x:v>
+        <x:v>worker-terra-max; worker-deepseek-flash-high</x:v>
       </x:c>
       <x:c r="C15" s="24" t="str">
-        <x:v>lead-terra-max or lead-sol-medium</x:v>
+        <x:v>High-complexity pool if evidence shows a reasoning blocker; never DeepSeek V4 Pro</x:v>
       </x:c>
       <x:c r="D15" s="24" t="str">
-        <x:v>Lead authority is explicitly assigned; a worker on the same model remains a leaf</x:v>
+        <x:v>Dense mechanical implementation or integration with exact contracts and tests; never assign interpretation or use effort to outlast a loop</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="46" customHeight="1">
       <x:c r="A16" s="24" t="str">
-        <x:v>Consequential architecture or high coupling</x:v>
+        <x:v>Novel public contract implementation</x:v>
       </x:c>
       <x:c r="B16" s="24" t="str">
-        <x:v>lead-sol-high</x:v>
+        <x:v>lead-sol-high settles shape; worker-deepseek-flash-max implements the exact contract</x:v>
       </x:c>
       <x:c r="C16" s="24" t="str">
-        <x:v>lead-astra-medium</x:v>
+        <x:v>lead-astra-medium settles unusually large cross-workstream contract ambiguity before execution</x:v>
       </x:c>
       <x:c r="D16" s="24" t="str">
-        <x:v>Escalate ambiguity or consequence beyond owned workstream</x:v>
+        <x:v>DeepSeek max receives a decided shape and objective contract tests; it does not choose the public contract</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="46" customHeight="1">
       <x:c r="A17" s="24" t="str">
-        <x:v>Cross-workstream planning and decisions</x:v>
+        <x:v>Workstream with fixed contracts</x:v>
       </x:c>
       <x:c r="B17" s="24" t="str">
-        <x:v>dm-astra-medium</x:v>
+        <x:v>lead-terra-xhigh</x:v>
       </x:c>
       <x:c r="C17" s="24" t="str">
-        <x:v>dm-sol-high or dm-opus-high; use directly when already in that configuration; verify transport and handover for house switches</x:v>
+        <x:v>lead-terra-max or lead-sol-medium</x:v>
       </x:c>
       <x:c r="D17" s="24" t="str">
-        <x:v>Manager receives compact exceptions and evidence, not raw logs</x:v>
+        <x:v>Mechanical lead authority may coordinate and delegate settled packets; ambiguity returns to lead-sol-high or lead-astra-medium</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="46" customHeight="1">
       <x:c r="A18" s="24" t="str">
-        <x:v>Independent acceptance</x:v>
+        <x:v>Consequential architecture or high coupling</x:v>
       </x:c>
       <x:c r="B18" s="24" t="str">
-        <x:v>Separate qualified reviewer session</x:v>
+        <x:v>lead-sol-high</x:v>
       </x:c>
       <x:c r="C18" s="24" t="str">
-        <x:v>Another eligible house; same house allowed with reason</x:v>
+        <x:v>lead-astra-medium for unusually large cross-workstream ambiguity</x:v>
       </x:c>
       <x:c r="D18" s="24" t="str">
-        <x:v>Reviewer inspects actual head/artifacts and never fixes its own findings</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20"/>
-      <x:c r="B20"/>
-      <x:c r="C20"/>
-      <x:c r="D20"/>
+        <x:v>Approved brain resolves product, architecture, consequence and coupling before execution</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="46" customHeight="1">
+      <x:c r="A19" s="24" t="str">
+        <x:v>Cross-workstream planning and decisions</x:v>
+      </x:c>
+      <x:c r="B19" s="24" t="str">
+        <x:v>dm-sol-high</x:v>
+      </x:c>
+      <x:c r="C19" s="24" t="str">
+        <x:v>dm-astra-medium for unusually large ambiguity; dm-opus-high may coordinate but routes judgment to a brain</x:v>
+      </x:c>
+      <x:c r="D19" s="24" t="str">
+        <x:v>Manager receives compact exceptions and evidence; only an assigned brain resolves interpretation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="46" customHeight="1">
+      <x:c r="A20" s="24" t="str">
+        <x:v>Independent semantic or risk acceptance</x:v>
+      </x:c>
+      <x:c r="B20" s="24" t="str">
+        <x:v>reviewer-sol-high</x:v>
+      </x:c>
+      <x:c r="C20" s="24" t="str">
+        <x:v>reviewer-astra-medium for unusually large cross-workstream scope</x:v>
+      </x:c>
+      <x:c r="D20" s="24" t="str">
+        <x:v>Mechanical gate collection may be delegated, but acceptance judgment belongs to an independent brain on the exact head</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="180" t="str">
+      <x:c r="A21"/>
+      <x:c r="B21"/>
+      <x:c r="C21"/>
+      <x:c r="D21"/>
+    </x:row>
+    <x:row r="22" ht="42" customHeight="1">
+      <x:c r="A22"/>
+      <x:c r="B22"/>
+      <x:c r="C22"/>
+      <x:c r="D22"/>
+    </x:row>
+    <x:row r="23" ht="42" customHeight="1">
+      <x:c r="A23" s="240" t="str">
         <x:v>Selection rules</x:v>
       </x:c>
-      <x:c r="B21" s="181"/>
-      <x:c r="C21" s="181"/>
-      <x:c r="D21" s="182"/>
-    </x:row>
-    <x:row r="22" ht="42" customHeight="1">
-      <x:c r="A22" s="188" t="str">
+      <x:c r="B23" s="241"/>
+      <x:c r="C23" s="241"/>
+      <x:c r="D23" s="242"/>
+    </x:row>
+    <x:row r="24" ht="42" customHeight="1">
+      <x:c r="A24" s="248" t="str">
         <x:v>Approved selection rule</x:v>
       </x:c>
-      <x:c r="B22" s="189"/>
-      <x:c r="C22" s="189"/>
-      <x:c r="D22" s="190"/>
-    </x:row>
-    <x:row r="23" ht="42" customHeight="1">
-      <x:c r="A23" s="91" t="str">
+      <x:c r="B24" s="249"/>
+      <x:c r="C24" s="249"/>
+      <x:c r="D24" s="250"/>
+    </x:row>
+    <x:row r="25" ht="42" customHeight="1">
+      <x:c r="A25" s="91" t="str">
         <x:v>1. Only Codex, Grok CLI, Claude Code and OpenCode are active houses. Cursor removed from Interchange routing, not uninstalled.</x:v>
       </x:c>
-      <x:c r="B23" s="67"/>
-      <x:c r="C23" s="67"/>
-      <x:c r="D23" s="67"/>
-    </x:row>
-    <x:row r="24" ht="42" customHeight="1">
-      <x:c r="A24" s="92" t="str">
-        <x:v>2. Grok work uses Grok CLI only, model grok-4.6 with high or xhigh. No Cursor route.</x:v>
-      </x:c>
-      <x:c r="B24" s="69"/>
-      <x:c r="C24" s="69"/>
-      <x:c r="D24" s="69"/>
-    </x:row>
-    <x:row r="25" ht="42" customHeight="1">
-      <x:c r="A25" s="92" t="str">
-        <x:v>3. Claude development uses claude-opus-5 medium or high. Sonnet and automatic fallback to it are excluded.</x:v>
-      </x:c>
-      <x:c r="B25" s="69"/>
-      <x:c r="C25" s="69"/>
-      <x:c r="D25" s="69"/>
+      <x:c r="B25" s="67"/>
+      <x:c r="C25" s="67"/>
+      <x:c r="D25" s="67"/>
     </x:row>
     <x:row r="26" ht="42" customHeight="1">
       <x:c r="A26" s="92" t="str">
-        <x:v>4. Treat task bands as routing preferences, not benchmark rankings. Assess ambiguity, consequence, coupling and implementation difficulty separately.</x:v>
+        <x:v>2. Grok work uses Grok CLI only, model grok-4.6 with high or xhigh. No Cursor route.</x:v>
       </x:c>
       <x:c r="B26" s="69"/>
       <x:c r="C26" s="69"/>
@@ -2137,7 +2469,7 @@
     </x:row>
     <x:row r="27" ht="42" customHeight="1">
       <x:c r="A27" s="92" t="str">
-        <x:v>5. Within an eligible pool, use task-fit evidence first, then expected accepted-result latency and available account/pool quota. Pool order is not a ranking.</x:v>
+        <x:v>3. Claude development uses claude-opus-5 medium or high. Sonnet and automatic fallback to it are excluded.</x:v>
       </x:c>
       <x:c r="B27" s="69"/>
       <x:c r="C27" s="69"/>
@@ -2145,7 +2477,7 @@
     </x:row>
     <x:row r="28" ht="42" customHeight="1">
       <x:c r="A28" s="92" t="str">
-        <x:v>6. Use different houses for parallel independent jobs of similar nature when suitable; preserve cached context and session continuity when that is cheaper or faster.</x:v>
+        <x:v>4. Brain boundary: only assigned Sol high, Astra medium and Fable 5.1 medium brain profiles resolve product, behavior, architecture or tradeoff ambiguity. Fable is for product ideation; Astra is for unusually large cross-workstream ambiguity; Sol high is the default.</x:v>
       </x:c>
       <x:c r="B28" s="69"/>
       <x:c r="C28" s="69"/>
@@ -2153,7 +2485,7 @@
     </x:row>
     <x:row r="29" ht="42" customHeight="1">
       <x:c r="A29" s="92" t="str">
-        <x:v>7. More reasoning is not universally more intelligence or better value. Terra max handles difficult settled implementation, not unresolved product decisions.</x:v>
+        <x:v>5. Semantic and risk acceptance is a brain task: use an independent Sol high reviewer, or Astra medium for unusually large cross-workstream scope. Mechanical workers may collect gates but cannot issue acceptance judgment.</x:v>
       </x:c>
       <x:c r="B29" s="69"/>
       <x:c r="C29" s="69"/>
@@ -2161,7 +2493,7 @@
     </x:row>
     <x:row r="30" ht="42" customHeight="1">
       <x:c r="A30" s="92" t="str">
-        <x:v>8. No automatic repeated effort increases. Stop, diagnose or reassign under existing watchdog and recovery limits.</x:v>
+        <x:v>6. Coordination is not judgment authority. Opus delivery managers and mechanical leads may coordinate, monitor and integrate, but route unresolved interpretation to an approved brain.</x:v>
       </x:c>
       <x:c r="B30" s="69"/>
       <x:c r="C30" s="69"/>
@@ -2169,7 +2501,7 @@
     </x:row>
     <x:row r="31" ht="42" customHeight="1">
       <x:c r="A31" s="92" t="str">
-        <x:v>9. Do not send every tiny job to the primary developer pool. Muse/Luna remain eligible bounded support workers.</x:v>
+        <x:v>7. Mechanical packets contain settled behavior, objective acceptance, owned paths, allowed variance and an escalation condition. Workers return evidence and the smallest question when a choice requires interpretation.</x:v>
       </x:c>
       <x:c r="B31" s="69"/>
       <x:c r="C31" s="69"/>
@@ -2177,7 +2509,7 @@
     </x:row>
     <x:row r="32" ht="42" customHeight="1">
       <x:c r="A32" s="92" t="str">
-        <x:v>10. High consequence can require stronger review even for a small edit. Model choice never removes acceptance gates.</x:v>
+        <x:v>8. Use fast, low-cost mechanical workers when startup, supervision and integration overhead still improves accepted-result time or cost. Parallelize independent objectively testable packets after decisions, interfaces and write ownership are fixed.</x:v>
       </x:c>
       <x:c r="B32" s="69"/>
       <x:c r="C32" s="69"/>
@@ -2185,7 +2517,7 @@
     </x:row>
     <x:row r="33" ht="42" customHeight="1">
       <x:c r="A33" s="92" t="str">
-        <x:v>11. Verify effective model and effort at dispatch. Newly configured Grok/Opus combinations are not yet claimed smoke-tested; no unapproved substitution.</x:v>
+        <x:v>9. Muse Spark 1.3 is the preferred light mechanical and read/seek lane for repository search, file localization, evidence collection, narrow checks and small explicit edits.</x:v>
       </x:c>
       <x:c r="B33" s="69"/>
       <x:c r="C33" s="69"/>
@@ -2193,7 +2525,7 @@
     </x:row>
     <x:row r="34" ht="42" customHeight="1">
       <x:c r="A34" s="92" t="str">
-        <x:v>12. House exclusivity has two scopes. Astra at any effort reserves Codex globally and Fable 5.1 at any effort reserves Claude globally. Sol high or higher reserves Codex only for assignments under the same delivery manager; Opus high or higher reserves Claude only for assignments under the same delivery manager.</x:v>
+        <x:v>10. Do not fragment work when dispatch, context transfer or integration overhead would erase the expected speed or cost gain.</x:v>
       </x:c>
       <x:c r="B34" s="69"/>
       <x:c r="C34" s="69"/>
@@ -2201,7 +2533,7 @@
     </x:row>
     <x:row r="35" ht="42" customHeight="1">
       <x:c r="A35" s="92" t="str">
-        <x:v>13. New-product brainstorming may use Fable 5.1 medium or Astra medium. Both create global house reservations while active; prefer another eligible house or queue competing work.</x:v>
+        <x:v>11. More reasoning is not universally more intelligence or better value. Terra max handles difficult settled implementation, not unresolved product decisions.</x:v>
       </x:c>
       <x:c r="B35" s="69"/>
       <x:c r="C35" s="69"/>
@@ -2209,7 +2541,7 @@
     </x:row>
     <x:row r="36" ht="42" customHeight="1">
       <x:c r="A36" s="92" t="str">
-        <x:v>14. Fable model authorization does not permit paid usage credits or extra spending. Verify included allowance before any headless request.</x:v>
+        <x:v>12. No automatic repeated effort increases. Stop, diagnose or reassign under existing watchdog and recovery limits.</x:v>
       </x:c>
       <x:c r="B36" s="69"/>
       <x:c r="C36" s="69"/>
@@ -2217,7 +2549,7 @@
     </x:row>
     <x:row r="37" ht="42" customHeight="1">
       <x:c r="A37" s="92" t="str">
-        <x:v>15. The delivery manager keeps its turn active with a real bounded wait while workers run. It may finish only after terminal handbacks or explicit transfer to another live supervisor.</x:v>
+        <x:v>13. High consequence can require stronger review even for a small edit. Model choice never removes acceptance gates.</x:v>
       </x:c>
       <x:c r="B37" s="69"/>
       <x:c r="C37" s="69"/>
@@ -2225,7 +2557,7 @@
     </x:row>
     <x:row r="38" ht="42" customHeight="1">
       <x:c r="A38" s="92" t="str">
-        <x:v>16. External provider streams are drained outside manager context. Retrieve compact lifecycle changes and the mechanically extracted final assistant result, not accumulated raw output.</x:v>
+        <x:v>14. Verify effective model and effort at dispatch. Newly configured Grok/Opus combinations are not yet claimed smoke-tested; no unapproved substitution.</x:v>
       </x:c>
       <x:c r="B38" s="69"/>
       <x:c r="C38" s="69"/>
@@ -2233,7 +2565,7 @@
     </x:row>
     <x:row r="39" ht="42" customHeight="1">
       <x:c r="A39" s="92" t="str">
-        <x:v>17. A provider parent exit does not transfer writer ownership. Verify process tree, worktree command/CWD holders and provider background-agent registry before any replacement writer.</x:v>
+        <x:v>15. House exclusivity has two scopes. Astra at any effort reserves Codex globally and Fable 5.1 at any effort reserves Claude globally. Sol high or higher reserves Codex only for assignments under the same delivery manager; Opus high or higher reserves Claude only for assignments under the same delivery manager.</x:v>
       </x:c>
       <x:c r="B39" s="69"/>
       <x:c r="C39" s="69"/>
@@ -2241,7 +2573,7 @@
     </x:row>
     <x:row r="40" ht="42" customHeight="1">
       <x:c r="A40" s="92" t="str">
-        <x:v>18. Stop Claude after two consecutive no-progress auto-compactions; checkpoint and use one fresh narrow retry rather than resuming the thrashing session.</x:v>
+        <x:v>16. New-product brainstorming may use Fable 5.1 medium or Astra medium. Both create global house reservations while active; prefer another eligible house or queue competing work.</x:v>
       </x:c>
       <x:c r="B40" s="69"/>
       <x:c r="C40" s="69"/>
@@ -2249,16 +2581,78 @@
     </x:row>
     <x:row r="41" ht="42" customHeight="1">
       <x:c r="A41" s="92" t="str">
-        <x:v>19. Owner concurrency exceptions are finite and journalled after an occupancy probe; leads and managers cannot self-authorize them.</x:v>
+        <x:v>17. Fable model authorization does not permit paid usage credits or extra spending. Verify included allowance before any headless request.</x:v>
       </x:c>
       <x:c r="B41" s="69"/>
       <x:c r="C41" s="69"/>
       <x:c r="D41" s="69"/>
     </x:row>
+    <x:row r="42" ht="42" customHeight="1">
+      <x:c r="A42" s="92" t="str">
+        <x:v>18. The delivery manager keeps its turn active with a real bounded wait while workers run. It may finish only after terminal handbacks or explicit transfer to another live supervisor.</x:v>
+      </x:c>
+      <x:c r="B42" s="69"/>
+      <x:c r="C42" s="69"/>
+      <x:c r="D42" s="69"/>
+    </x:row>
+    <x:row r="43" ht="42" customHeight="1">
+      <x:c r="A43" s="92" t="str">
+        <x:v>19. External provider streams are drained outside manager context. Retrieve compact lifecycle changes and the mechanically extracted final assistant result, not accumulated raw output.</x:v>
+      </x:c>
+      <x:c r="B43" s="69"/>
+      <x:c r="C43" s="69"/>
+      <x:c r="D43" s="69"/>
+    </x:row>
+    <x:row r="44" ht="42" customHeight="1">
+      <x:c r="A44" s="92" t="str">
+        <x:v>20. A provider parent exit does not transfer writer ownership. Verify process tree, worktree command/CWD holders and provider background-agent registry before any replacement writer.</x:v>
+      </x:c>
+      <x:c r="B44" s="69"/>
+      <x:c r="C44" s="69"/>
+      <x:c r="D44" s="69"/>
+    </x:row>
+    <x:row r="45" ht="42" customHeight="1">
+      <x:c r="A45" s="92" t="str">
+        <x:v>21. Stop Claude after two consecutive no-progress auto-compactions; checkpoint and use one fresh narrow retry rather than resuming the thrashing session.</x:v>
+      </x:c>
+      <x:c r="B45" s="69"/>
+      <x:c r="C45" s="69"/>
+      <x:c r="D45" s="69"/>
+    </x:row>
+    <x:row r="46" ht="42" customHeight="1">
+      <x:c r="A46" s="92" t="str">
+        <x:v>22. Owner concurrency exceptions are finite and journalled after an occupancy probe; leads and managers cannot self-authorize them.</x:v>
+      </x:c>
+      <x:c r="B46" s="69"/>
+      <x:c r="C46" s="69"/>
+      <x:c r="D46" s="69"/>
+    </x:row>
+    <x:row r="47" ht="42" customHeight="1">
+      <x:c r="A47" s="92" t="str">
+        <x:v>23. DeepSeek V4.1 Flash uses the provider code opencode-go/deepseek-v4.1-flash. The human-readable name and provider code identify the same approved model. The provider renamed this code from opencode-go/deepseek-flash, which no longer appears in `opencode models`; the version now lives in the code itself.</x:v>
+      </x:c>
+      <x:c r="B47" s="69"/>
+      <x:c r="C47" s="69"/>
+      <x:c r="D47" s="69"/>
+    </x:row>
+    <x:row r="48" ht="42" customHeight="1">
+      <x:c r="A48" s="92" t="str">
+        <x:v>24. DeepSeek high is the default for bounded implementation. DeepSeek max mechanically implements novel public contract, identity, schema or serialization shapes only after an approved brain settles the shape and objective contract tests.</x:v>
+      </x:c>
+      <x:c r="B48" s="69"/>
+      <x:c r="C48" s="69"/>
+      <x:c r="D48" s="69"/>
+    </x:row>
+    <x:row r="49" ht="42" customHeight="1">
+      <x:c r="A49" s="92" t="str">
+        <x:v>25. DeepSeek V4 Pro, DeepSeek V4 Flash and the vision-exp variants are excluded: opencode-go/deepseek-v4-pro, opencode-go/deepseek-v4-flash and opencode-go/deepseek-v4-flash-vision-exp are DIFFERENT models, not fallbacks for V4.1 Flash. If opencode-go/deepseek-v4.1-flash is unavailable, stop and reroute to a different approved house; never substitute another DeepSeek model.</x:v>
+      </x:c>
+      <x:c r="B49" s="69"/>
+      <x:c r="C49" s="69"/>
+      <x:c r="D49" s="69"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A22:D22"/>
-    <x:mergeCell ref="A23:D23"/>
     <x:mergeCell ref="A24:D24"/>
     <x:mergeCell ref="A25:D25"/>
     <x:mergeCell ref="A26:D26"/>
@@ -2277,6 +2671,14 @@
     <x:mergeCell ref="A39:D39"/>
     <x:mergeCell ref="A40:D40"/>
     <x:mergeCell ref="A41:D41"/>
+    <x:mergeCell ref="A42:D42"/>
+    <x:mergeCell ref="A43:D43"/>
+    <x:mergeCell ref="A44:D44"/>
+    <x:mergeCell ref="A45:D45"/>
+    <x:mergeCell ref="A46:D46"/>
+    <x:mergeCell ref="A47:D47"/>
+    <x:mergeCell ref="A48:D48"/>
+    <x:mergeCell ref="A49:D49"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2308,13 +2710,13 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>Policy source: Interchange policy v0.4.0</x:v>
+        <x:v>Policy source: Interchange policy v0.6.0</x:v>
       </x:c>
       <x:c r="B3" s="2" t="str">
         <x:v>Approved on</x:v>
       </x:c>
       <x:c r="C3" s="5" t="n">
-        <x:v>46274</x:v>
+        <x:v>46278</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -2519,13 +2921,13 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>Policy source: Interchange policy v0.4.0</x:v>
+        <x:v>Policy source: Interchange policy v0.6.0</x:v>
       </x:c>
       <x:c r="B3" s="2" t="str">
         <x:v>Approved on</x:v>
       </x:c>
       <x:c r="C3" s="5" t="n">
-        <x:v>46274</x:v>
+        <x:v>46278</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -2595,7 +2997,7 @@
         <x:v>Spending</x:v>
       </x:c>
       <x:c r="B12" s="24" t="str">
-        <x:v>No extra purchases or automatic recharge; existing OpenCode Go allowance/balance may be used for Muse only</x:v>
+        <x:v>No extra purchases or automatic recharge; existing OpenCode Go allowance/balance may be used for approved Muse and DeepSeek Flash profiles; DeepSeek V4 Pro is excluded</x:v>
       </x:c>
       <x:c r="C12"/>
     </x:row>
@@ -2682,20 +3084,20 @@
       <x:c r="C22"/>
     </x:row>
     <x:row r="23" ht="26" customHeight="1">
-      <x:c r="A23" s="180" t="str">
+      <x:c r="A23" s="240" t="str">
         <x:v>Recovery playbook</x:v>
       </x:c>
-      <x:c r="B23" s="181"/>
-      <x:c r="C23" s="182"/>
+      <x:c r="B23" s="241"/>
+      <x:c r="C23" s="242"/>
     </x:row>
     <x:row r="24" ht="44" customHeight="1">
-      <x:c r="A24" s="188" t="str">
+      <x:c r="A24" s="248" t="str">
         <x:v>Failure</x:v>
       </x:c>
-      <x:c r="B24" s="189" t="str">
+      <x:c r="B24" s="249" t="str">
         <x:v>First action</x:v>
       </x:c>
-      <x:c r="C24" s="190" t="str">
+      <x:c r="C24" s="250" t="str">
         <x:v>Escalation</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
feat(interchange): separate brains from workers (#4)
</commit_message>
<xml_diff>
--- a/outputs/interchange-design/interchange.xlsx
+++ b/outputs/interchange-design/interchange.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profiles" sheetId="1" r:id="Rdb05d2334a084321"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Routing" sheetId="2" r:id="R4a8f0ce1555046dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monitoring" sheetId="3" r:id="R22d28bd2e77f4b53"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Recovery" sheetId="4" r:id="Rc554ec4257a34146"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profiles" sheetId="1" r:id="R54bb1c1b109c4a81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Routing" sheetId="2" r:id="Ra5fa34cf7b594df6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monitoring" sheetId="3" r:id="R9861e40f1bfe4770"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Recovery" sheetId="4" r:id="Re075d54395954ed3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -55,7 +55,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="39">
+  <x:fills count="51">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -85,6 +85,66 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFCE4D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -320,7 +380,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="191">
+  <x:cellXfs count="251">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -792,6 +852,144 @@
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="38" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="39" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="39" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="40" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="40" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="39" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="41" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="41" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="41" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="41" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="41" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="42" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="42" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="42" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="42" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="42" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="42" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="42" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="42" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="43" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="43" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="44" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="44" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="44" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="43" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="45" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="45" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="45" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="45" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="45" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="46" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="46" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="46" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="46" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="46" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="46" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="46" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="46" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="47" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="47" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="48" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="48" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="47" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="49" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="49" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="49" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="50" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="50" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="50" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1036,7 +1234,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>Policy source: Interchange policy v0.4.0</x:v>
+        <x:v>Policy source: Interchange policy v0.6.0</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -1044,7 +1242,7 @@
         <x:v>Approved on</x:v>
       </x:c>
       <x:c r="E3" s="5" t="n">
-        <x:v>46274</x:v>
+        <x:v>46278</x:v>
       </x:c>
       <x:c r="F3" s="2"/>
       <x:c r="G3" s="4" t="str">
@@ -1110,8 +1308,8 @@
         <x:v>Allowed fixed profiles</x:v>
       </x:c>
       <x:c r="B8" s="30" t="n">
-        <x:f>COUNTIFS($G$16:$G$36,"Allowed fixed profile")</x:f>
-        <x:v>21</x:v>
+        <x:f>COUNTIFS($G$16:$G$40,"Allowed fixed profile")</x:f>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C8" s="22" t="str">
         <x:v>Select only when the assigned role, pool, and task fit.</x:v>
@@ -1128,7 +1326,7 @@
         <x:v>Smoke-tested fixed profiles</x:v>
       </x:c>
       <x:c r="B9" s="31" t="n">
-        <x:f>COUNTIFS($H$16:$H$36,"Smoke-tested")</x:f>
+        <x:f>COUNTIFS($H$16:$H$40,"Smoke-tested")</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="C9" s="24" t="str">
@@ -1146,7 +1344,7 @@
         <x:v>Documented profiles pending exact runtime check</x:v>
       </x:c>
       <x:c r="B10" s="32" t="n">
-        <x:f>COUNTIFS($H$16:$H$36,"CLI model and effort documented; exact runtime unverified")+COUNTIFS($H$16:$H$36,"Profile documented; exact runtime unverified")</x:f>
+        <x:f>COUNTIFS($H$16:$H$40,"CLI model and effort documented; exact runtime unverified")+COUNTIFS($H$16:$H$40,"Profile documented; exact runtime unverified")</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="C10" s="24" t="str">
@@ -1254,15 +1452,15 @@
         <x:v>high</x:v>
       </x:c>
       <x:c r="E16" s="22" t="str">
-        <x:v>delivery manager: approved alternative with explicit handover when switching houses</x:v>
+        <x:v>delivery manager: mechanical coordination and continuity; route unresolved interpretation to an approved brain</x:v>
       </x:c>
       <x:c r="F16" s="34" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G16" s="173" t="str">
+      <x:c r="G16" s="233" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H16" s="175" t="str">
+      <x:c r="H16" s="235" t="str">
         <x:v>Profile documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I16" s="22" t="str">
@@ -1283,15 +1481,15 @@
         <x:v>high</x:v>
       </x:c>
       <x:c r="E17" s="24" t="str">
-        <x:v>delivery manager: approved alternative when starting with Sol high</x:v>
+        <x:v>delivery manager and default product/architecture brain</x:v>
       </x:c>
       <x:c r="F17" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G17" s="174" t="str">
+      <x:c r="G17" s="234" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H17" s="176" t="str">
+      <x:c r="H17" s="236" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I17" s="24" t="str">
@@ -1312,15 +1510,15 @@
         <x:v>medium</x:v>
       </x:c>
       <x:c r="E18" s="24" t="str">
-        <x:v>delivery manager</x:v>
+        <x:v>delivery manager and brain for unusually large cross-workstream ambiguity</x:v>
       </x:c>
       <x:c r="F18" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G18" s="174" t="str">
+      <x:c r="G18" s="234" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H18" s="176" t="str">
+      <x:c r="H18" s="236" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I18" s="24" t="str">
@@ -1341,15 +1539,15 @@
         <x:v>medium</x:v>
       </x:c>
       <x:c r="E19" s="24" t="str">
-        <x:v>lead: high ambiguity or cross-workstream architecture</x:v>
+        <x:v>brain lead: unusually large ambiguity or cross-workstream architecture</x:v>
       </x:c>
       <x:c r="F19" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G19" s="174" t="str">
+      <x:c r="G19" s="234" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H19" s="176" t="str">
+      <x:c r="H19" s="236" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I19" s="24" t="str">
@@ -1370,15 +1568,15 @@
         <x:v>medium</x:v>
       </x:c>
       <x:c r="E20" s="24" t="str">
-        <x:v>lead: bounded architecture and moderate coupling</x:v>
+        <x:v>mechanical workstream coordinator for settled contracts; no interpretive authority</x:v>
       </x:c>
       <x:c r="F20" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G20" s="174" t="str">
+      <x:c r="G20" s="234" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H20" s="176" t="str">
+      <x:c r="H20" s="236" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I20" s="24" t="str">
@@ -1399,15 +1597,15 @@
         <x:v>high</x:v>
       </x:c>
       <x:c r="E21" s="24" t="str">
-        <x:v>lead: consequential design and risk</x:v>
+        <x:v>default brain lead: product, architecture, consequence and tradeoff decisions</x:v>
       </x:c>
       <x:c r="F21" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G21" s="174" t="str">
+      <x:c r="G21" s="234" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H21" s="176" t="str">
+      <x:c r="H21" s="236" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I21" s="24" t="str">
@@ -1416,306 +1614,306 @@
     </x:row>
     <x:row r="22" ht="38" customHeight="1">
       <x:c r="A22" s="24" t="str">
-        <x:v>lead-terra-xhigh</x:v>
+        <x:v>reviewer-sol-high</x:v>
       </x:c>
       <x:c r="B22" s="24" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="C22" s="24" t="str">
-        <x:v>gpt-5.6-terra</x:v>
+        <x:v>gpt-5.6-sol</x:v>
       </x:c>
       <x:c r="D22" s="24" t="str">
-        <x:v>xhigh</x:v>
+        <x:v>high</x:v>
       </x:c>
       <x:c r="E22" s="24" t="str">
-        <x:v>lead: defined contracts and bounded workstream</x:v>
+        <x:v>independent semantic and risk review brain; no implementation or self-review</x:v>
       </x:c>
       <x:c r="F22" s="35" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="G22" s="174" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="G22" s="234" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H22" s="176" t="str">
+      <x:c r="H22" s="236" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I22" s="24" t="str">
-        <x:v>Supported by current tool metadata; routing uncalibrated</x:v>
+        <x:v>Sol high review found meaning-level defects in governed delivery; reviewer remains independent of writer and current-head bound</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="38" customHeight="1">
       <x:c r="A23" s="24" t="str">
-        <x:v>lead-terra-max</x:v>
+        <x:v>reviewer-astra-medium</x:v>
       </x:c>
       <x:c r="B23" s="24" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="C23" s="24" t="str">
-        <x:v>gpt-5.6-terra</x:v>
+        <x:v>gpt-6-astra</x:v>
       </x:c>
       <x:c r="D23" s="24" t="str">
-        <x:v>max</x:v>
+        <x:v>medium</x:v>
       </x:c>
       <x:c r="E23" s="24" t="str">
-        <x:v>lead: defined architecture with difficult integration</x:v>
+        <x:v>independent semantic review brain for unusually large cross-workstream scope; no implementation or self-review</x:v>
       </x:c>
       <x:c r="F23" s="35" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="G23" s="174" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="G23" s="234" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H23" s="176" t="str">
+      <x:c r="H23" s="236" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I23" s="24" t="str">
-        <x:v>Supported by current tool metadata; routing uncalibrated</x:v>
+        <x:v>Supported by current tool metadata; reviewer routing uncalibrated</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="38" customHeight="1">
       <x:c r="A24" s="24" t="str">
-        <x:v>worker-luna-xhigh</x:v>
+        <x:v>lead-terra-xhigh</x:v>
       </x:c>
       <x:c r="B24" s="24" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="C24" s="24" t="str">
-        <x:v>gpt-5.6-luna</x:v>
+        <x:v>gpt-5.6-terra</x:v>
       </x:c>
       <x:c r="D24" s="24" t="str">
         <x:v>xhigh</x:v>
       </x:c>
       <x:c r="E24" s="24" t="str">
-        <x:v>bounded leaf exploration or explicit small change</x:v>
+        <x:v>mechanical lead: defined contracts and bounded workstream; escalate interpretation</x:v>
       </x:c>
       <x:c r="F24" s="35" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="G24" s="174" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G24" s="234" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H24" s="176" t="str">
+      <x:c r="H24" s="236" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I24" s="24" t="str">
-        <x:v>Supported; lower effort forbidden by owner</x:v>
+        <x:v>Supported by current tool metadata; routing uncalibrated</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="38" customHeight="1">
       <x:c r="A25" s="24" t="str">
-        <x:v>worker-luna-max</x:v>
+        <x:v>lead-terra-max</x:v>
       </x:c>
       <x:c r="B25" s="24" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="C25" s="24" t="str">
-        <x:v>gpt-5.6-luna</x:v>
+        <x:v>gpt-5.6-terra</x:v>
       </x:c>
       <x:c r="D25" s="24" t="str">
         <x:v>max</x:v>
       </x:c>
       <x:c r="E25" s="24" t="str">
-        <x:v>bounded leaf with denser evidence</x:v>
+        <x:v>mechanical lead: difficult integration within defined architecture; escalate interpretation</x:v>
       </x:c>
       <x:c r="F25" s="35" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="G25" s="174" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G25" s="234" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H25" s="176" t="str">
+      <x:c r="H25" s="236" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I25" s="24" t="str">
-        <x:v>Supported; lower effort forbidden by owner</x:v>
+        <x:v>Supported by current tool metadata; routing uncalibrated</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="38" customHeight="1">
       <x:c r="A26" s="24" t="str">
-        <x:v>worker-terra-xhigh</x:v>
+        <x:v>worker-luna-xhigh</x:v>
       </x:c>
       <x:c r="B26" s="24" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="C26" s="24" t="str">
-        <x:v>gpt-5.6-terra</x:v>
+        <x:v>gpt-5.6-luna</x:v>
       </x:c>
       <x:c r="D26" s="24" t="str">
         <x:v>xhigh</x:v>
       </x:c>
       <x:c r="E26" s="24" t="str">
-        <x:v>bounded builder or independent verifier</x:v>
+        <x:v>bounded leaf exploration or explicit small change</x:v>
       </x:c>
       <x:c r="F26" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G26" s="174" t="str">
+      <x:c r="G26" s="234" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H26" s="176" t="str">
+      <x:c r="H26" s="236" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I26" s="24" t="str">
-        <x:v>Supported; role assignment separate from model</x:v>
+        <x:v>Supported; lower effort forbidden by owner</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="38" customHeight="1">
       <x:c r="A27" s="24" t="str">
-        <x:v>worker-muse-xhigh</x:v>
+        <x:v>worker-luna-max</x:v>
       </x:c>
       <x:c r="B27" s="24" t="str">
-        <x:v>OpenCode / Go pool</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="C27" s="24" t="str">
-        <x:v>opencode-go/muse-spark-1.3-contributor</x:v>
+        <x:v>gpt-5.6-luna</x:v>
       </x:c>
       <x:c r="D27" s="24" t="str">
-        <x:v>xhigh</x:v>
+        <x:v>max</x:v>
       </x:c>
       <x:c r="E27" s="24" t="str">
-        <x:v>preferred initial cheap leaf candidate</x:v>
+        <x:v>bounded leaf with denser evidence</x:v>
       </x:c>
       <x:c r="F27" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G27" s="174" t="str">
+      <x:c r="G27" s="234" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H27" s="177" t="str">
-        <x:v>Smoke-tested</x:v>
+      <x:c r="H27" s="236" t="str">
+        <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I27" s="24" t="str">
-        <x:v>CLI send/resume/recall smoke-tested; quality advantage is owner hypothesis</x:v>
+        <x:v>Supported; lower effort forbidden by owner</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="38" customHeight="1">
       <x:c r="A28" s="24" t="str">
-        <x:v>worker-grok-high</x:v>
+        <x:v>worker-terra-xhigh</x:v>
       </x:c>
       <x:c r="B28" s="24" t="str">
-        <x:v>Grok</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="C28" s="24" t="str">
-        <x:v>grok-4.6</x:v>
+        <x:v>gpt-5.6-terra</x:v>
       </x:c>
       <x:c r="D28" s="24" t="str">
-        <x:v>high</x:v>
+        <x:v>xhigh</x:v>
       </x:c>
       <x:c r="E28" s="24" t="str">
-        <x:v>primary low/mid complexity developer</x:v>
+        <x:v>bounded builder or independent verifier</x:v>
       </x:c>
       <x:c r="F28" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G28" s="174" t="str">
+      <x:c r="G28" s="234" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H28" s="176" t="str">
-        <x:v>CLI model and effort documented; exact runtime unverified</x:v>
+      <x:c r="H28" s="236" t="str">
+        <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I28" s="24" t="str">
-        <x:v>grok models lists grok-4.6; effort flags documented; exact profile smoke test pending</x:v>
+        <x:v>Supported; role assignment separate from model</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="38" customHeight="1">
       <x:c r="A29" s="24" t="str">
-        <x:v>worker-grok-xhigh</x:v>
+        <x:v>worker-muse-xhigh</x:v>
       </x:c>
       <x:c r="B29" s="24" t="str">
-        <x:v>Grok</x:v>
+        <x:v>OpenCode / Go pool</x:v>
       </x:c>
       <x:c r="C29" s="24" t="str">
-        <x:v>grok-4.6</x:v>
+        <x:v>opencode-go/muse-spark-1.3-contributor</x:v>
       </x:c>
       <x:c r="D29" s="24" t="str">
         <x:v>xhigh</x:v>
       </x:c>
       <x:c r="E29" s="24" t="str">
-        <x:v>primary upper-mid complexity developer</x:v>
+        <x:v>light mechanical and read/seek leaf: repository search, localization, evidence, narrow checks or small explicit edits</x:v>
       </x:c>
       <x:c r="F29" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G29" s="174" t="str">
+      <x:c r="G29" s="234" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H29" s="176" t="str">
-        <x:v>CLI model and effort documented; exact runtime unverified</x:v>
+      <x:c r="H29" s="237" t="str">
+        <x:v>Smoke-tested</x:v>
       </x:c>
       <x:c r="I29" s="24" t="str">
-        <x:v>grok models lists grok-4.6; effort flags documented; exact profile smoke test pending</x:v>
+        <x:v>CLI send/resume/recall smoke-tested; quality advantage is owner hypothesis</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="38" customHeight="1">
       <x:c r="A30" s="24" t="str">
-        <x:v>worker-opus-medium</x:v>
+        <x:v>worker-deepseek-flash-high</x:v>
       </x:c>
       <x:c r="B30" s="24" t="str">
-        <x:v>Claude</x:v>
+        <x:v>OpenCode / Go pool</x:v>
       </x:c>
       <x:c r="C30" s="24" t="str">
-        <x:v>claude-opus-5</x:v>
+        <x:v>opencode-go/deepseek-v4.1-flash</x:v>
       </x:c>
       <x:c r="D30" s="24" t="str">
-        <x:v>medium</x:v>
+        <x:v>high</x:v>
       </x:c>
       <x:c r="E30" s="24" t="str">
-        <x:v>primary low/mid and upper-mid complexity developer</x:v>
+        <x:v>preferred bounded implementation worker with clear acceptance and settled architecture</x:v>
       </x:c>
       <x:c r="F30" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G30" s="174" t="str">
+      <x:c r="G30" s="234" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H30" s="176" t="str">
-        <x:v>Profile documented; exact runtime unverified</x:v>
+      <x:c r="H30" s="236" t="str">
+        <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I30" s="24" t="str">
-        <x:v>Full model ID and effort documented; exact profile runtime identity and smoke test pending</x:v>
+        <x:v>Eleven governed DeepSeek Flash runs across two repositories; high is the approved default. Independent semantic review remains mandatory.</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="38" customHeight="1">
       <x:c r="A31" s="24" t="str">
-        <x:v>worker-opus-high</x:v>
+        <x:v>worker-deepseek-flash-max</x:v>
       </x:c>
       <x:c r="B31" s="24" t="str">
-        <x:v>Claude</x:v>
+        <x:v>OpenCode / Go pool</x:v>
       </x:c>
       <x:c r="C31" s="24" t="str">
-        <x:v>claude-opus-5</x:v>
+        <x:v>opencode-go/deepseek-v4.1-flash</x:v>
       </x:c>
       <x:c r="D31" s="24" t="str">
-        <x:v>high</x:v>
+        <x:v>max</x:v>
       </x:c>
       <x:c r="E31" s="24" t="str">
-        <x:v>primary high complexity developer</x:v>
+        <x:v>mechanical implementation of a novel public contract shape already settled by an approved brain</x:v>
       </x:c>
       <x:c r="F31" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G31" s="174" t="str">
+      <x:c r="G31" s="234" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H31" s="176" t="str">
-        <x:v>Profile documented; exact runtime unverified</x:v>
+      <x:c r="H31" s="236" t="str">
+        <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I31" s="24" t="str">
-        <x:v>Full model ID and effort documented; exact profile runtime identity and smoke test pending</x:v>
+        <x:v>One evaluated max assignment showed value on novel public identity work; current policy restricts max to mechanical implementation after a brain settles the shape. Independent semantic review remains mandatory.</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="38" customHeight="1">
       <x:c r="A32" s="24" t="str">
-        <x:v>worker-sol-medium</x:v>
+        <x:v>worker-grok-high</x:v>
       </x:c>
       <x:c r="B32" s="24" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Grok</x:v>
       </x:c>
       <x:c r="C32" s="24" t="str">
-        <x:v>gpt-5.6-sol</x:v>
+        <x:v>grok-4.6</x:v>
       </x:c>
       <x:c r="D32" s="24" t="str">
-        <x:v>medium</x:v>
+        <x:v>high</x:v>
       </x:c>
       <x:c r="E32" s="24" t="str">
         <x:v>primary low/mid complexity developer</x:v>
@@ -1723,129 +1921,245 @@
       <x:c r="F32" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G32" s="174" t="str">
+      <x:c r="G32" s="234" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H32" s="176" t="str">
-        <x:v>Supported by metadata; routing unverified</x:v>
+      <x:c r="H32" s="236" t="str">
+        <x:v>CLI model and effort documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I32" s="24" t="str">
-        <x:v>Current tool metadata supports profile; task-class performance uncalibrated</x:v>
+        <x:v>grok models lists grok-4.6; effort flags documented; exact profile smoke test pending</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="38" customHeight="1">
       <x:c r="A33" s="24" t="str">
-        <x:v>worker-sol-high</x:v>
+        <x:v>worker-grok-xhigh</x:v>
       </x:c>
       <x:c r="B33" s="24" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Grok</x:v>
       </x:c>
       <x:c r="C33" s="24" t="str">
-        <x:v>gpt-5.6-sol</x:v>
+        <x:v>grok-4.6</x:v>
       </x:c>
       <x:c r="D33" s="24" t="str">
-        <x:v>high</x:v>
+        <x:v>xhigh</x:v>
       </x:c>
       <x:c r="E33" s="24" t="str">
-        <x:v>primary high complexity developer</x:v>
+        <x:v>primary upper-mid complexity developer</x:v>
       </x:c>
       <x:c r="F33" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G33" s="174" t="str">
+      <x:c r="G33" s="234" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H33" s="176" t="str">
-        <x:v>Supported by metadata; routing unverified</x:v>
+      <x:c r="H33" s="236" t="str">
+        <x:v>CLI model and effort documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I33" s="24" t="str">
-        <x:v>Current tool metadata supports profile; task-class performance uncalibrated</x:v>
+        <x:v>grok models lists grok-4.6; effort flags documented; exact profile smoke test pending</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="38" customHeight="1">
       <x:c r="A34" s="24" t="str">
-        <x:v>worker-terra-max</x:v>
+        <x:v>worker-opus-medium</x:v>
       </x:c>
       <x:c r="B34" s="24" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Claude</x:v>
       </x:c>
       <x:c r="C34" s="24" t="str">
-        <x:v>gpt-5.6-terra</x:v>
+        <x:v>claude-opus-5</x:v>
       </x:c>
       <x:c r="D34" s="24" t="str">
-        <x:v>max</x:v>
+        <x:v>medium</x:v>
       </x:c>
       <x:c r="E34" s="24" t="str">
-        <x:v>demanding implementation with settled contracts and bounded scope</x:v>
+        <x:v>primary low/mid and upper-mid complexity developer</x:v>
       </x:c>
       <x:c r="F34" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G34" s="174" t="str">
+      <x:c r="G34" s="234" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H34" s="176" t="str">
-        <x:v>Supported by metadata; routing unverified</x:v>
+      <x:c r="H34" s="236" t="str">
+        <x:v>Profile documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I34" s="24" t="str">
-        <x:v>Current tool metadata supports profile; effort is not a substitute for resolving ambiguity</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35" ht="76" customHeight="1">
+        <x:v>Full model ID and effort documented; exact profile runtime identity and smoke test pending</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="38" customHeight="1">
       <x:c r="A35" s="24" t="str">
-        <x:v>brainstorm-fable-medium</x:v>
+        <x:v>worker-opus-high</x:v>
       </x:c>
       <x:c r="B35" s="24" t="str">
         <x:v>Claude</x:v>
       </x:c>
       <x:c r="C35" s="24" t="str">
-        <x:v>claude-fable-5-1</x:v>
+        <x:v>claude-opus-5</x:v>
       </x:c>
       <x:c r="D35" s="24" t="str">
-        <x:v>medium</x:v>
+        <x:v>high</x:v>
       </x:c>
       <x:c r="E35" s="24" t="str">
-        <x:v>new-product ideation and brainstorming</x:v>
+        <x:v>primary high complexity developer</x:v>
       </x:c>
       <x:c r="F35" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G35" s="174" t="str">
+      <x:c r="G35" s="234" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H35" s="176" t="str">
+      <x:c r="H35" s="236" t="str">
         <x:v>Profile documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I35" s="24" t="str">
-        <x:v>Official model/effort documentation; exact runtime and included-plan eligibility not verified</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="36" ht="76" customHeight="1">
+        <x:v>Full model ID and effort documented; exact profile runtime identity and smoke test pending</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="38" customHeight="1">
       <x:c r="A36" s="24" t="str">
-        <x:v>brainstorm-astra-medium</x:v>
+        <x:v>worker-sol-medium</x:v>
       </x:c>
       <x:c r="B36" s="24" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="C36" s="24" t="str">
-        <x:v>gpt-6-astra</x:v>
+        <x:v>gpt-5.6-sol</x:v>
       </x:c>
       <x:c r="D36" s="24" t="str">
         <x:v>medium</x:v>
       </x:c>
       <x:c r="E36" s="24" t="str">
-        <x:v>new-product ideation and brainstorming</x:v>
+        <x:v>primary low/mid complexity developer</x:v>
       </x:c>
       <x:c r="F36" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G36" s="174" t="str">
+      <x:c r="G36" s="234" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H36" s="176" t="str">
+      <x:c r="H36" s="236" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I36" s="24" t="str">
+        <x:v>Current tool metadata supports profile; task-class performance uncalibrated</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="38" customHeight="1">
+      <x:c r="A37" s="24" t="str">
+        <x:v>worker-sol-high</x:v>
+      </x:c>
+      <x:c r="B37" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="C37" s="24" t="str">
+        <x:v>gpt-5.6-sol</x:v>
+      </x:c>
+      <x:c r="D37" s="24" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="E37" s="24" t="str">
+        <x:v>primary high complexity developer</x:v>
+      </x:c>
+      <x:c r="F37" s="35" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="G37" s="234" t="str">
+        <x:v>Allowed fixed profile</x:v>
+      </x:c>
+      <x:c r="H37" s="236" t="str">
+        <x:v>Supported by metadata; routing unverified</x:v>
+      </x:c>
+      <x:c r="I37" s="24" t="str">
+        <x:v>Current tool metadata supports profile; task-class performance uncalibrated</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="38" customHeight="1">
+      <x:c r="A38" s="24" t="str">
+        <x:v>worker-terra-max</x:v>
+      </x:c>
+      <x:c r="B38" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="C38" s="24" t="str">
+        <x:v>gpt-5.6-terra</x:v>
+      </x:c>
+      <x:c r="D38" s="24" t="str">
+        <x:v>max</x:v>
+      </x:c>
+      <x:c r="E38" s="24" t="str">
+        <x:v>demanding implementation with settled contracts and bounded scope</x:v>
+      </x:c>
+      <x:c r="F38" s="35" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="G38" s="234" t="str">
+        <x:v>Allowed fixed profile</x:v>
+      </x:c>
+      <x:c r="H38" s="236" t="str">
+        <x:v>Supported by metadata; routing unverified</x:v>
+      </x:c>
+      <x:c r="I38" s="24" t="str">
+        <x:v>Current tool metadata supports profile; effort is not a substitute for resolving ambiguity</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="76" customHeight="1">
+      <x:c r="A39" s="24" t="str">
+        <x:v>brainstorm-fable-medium</x:v>
+      </x:c>
+      <x:c r="B39" s="24" t="str">
+        <x:v>Claude</x:v>
+      </x:c>
+      <x:c r="C39" s="24" t="str">
+        <x:v>claude-fable-5-1</x:v>
+      </x:c>
+      <x:c r="D39" s="24" t="str">
+        <x:v>medium</x:v>
+      </x:c>
+      <x:c r="E39" s="24" t="str">
+        <x:v>product-ideation brain; no implementation; included-plan/no-extra-cost preflight required</x:v>
+      </x:c>
+      <x:c r="F39" s="35" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="G39" s="234" t="str">
+        <x:v>Allowed fixed profile</x:v>
+      </x:c>
+      <x:c r="H39" s="236" t="str">
+        <x:v>Profile documented; exact runtime unverified</x:v>
+      </x:c>
+      <x:c r="I39" s="24" t="str">
+        <x:v>Official model/effort documentation; exact runtime and included-plan eligibility not verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="76" customHeight="1">
+      <x:c r="A40" s="24" t="str">
+        <x:v>brainstorm-astra-medium</x:v>
+      </x:c>
+      <x:c r="B40" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="C40" s="24" t="str">
+        <x:v>gpt-6-astra</x:v>
+      </x:c>
+      <x:c r="D40" s="24" t="str">
+        <x:v>medium</x:v>
+      </x:c>
+      <x:c r="E40" s="24" t="str">
+        <x:v>product-ideation brain for unusually large or cross-workstream concepts</x:v>
+      </x:c>
+      <x:c r="F40" s="35" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="G40" s="234" t="str">
+        <x:v>Allowed fixed profile</x:v>
+      </x:c>
+      <x:c r="H40" s="236" t="str">
+        <x:v>Supported by metadata; routing unverified</x:v>
+      </x:c>
+      <x:c r="I40" s="24" t="str">
         <x:v>Current tool metadata supports profile; no comparative ideation benchmark</x:v>
       </x:c>
     </x:row>
@@ -1883,14 +2197,14 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>Policy source: Interchange policy v0.4.0</x:v>
+        <x:v>Policy source: Interchange policy v0.6.0</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2" t="str">
         <x:v>Approved on</x:v>
       </x:c>
       <x:c r="D3" s="5" t="n">
-        <x:v>46274</x:v>
+        <x:v>46278</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -1943,193 +2257,211 @@
     </x:row>
     <x:row r="9" ht="46" customHeight="1">
       <x:c r="A9" s="24" t="str">
-        <x:v>One direct lookup</x:v>
+        <x:v>Product, behavior or architecture judgment</x:v>
       </x:c>
       <x:c r="B9" s="24" t="str">
-        <x:v>Local search/tool</x:v>
+        <x:v>lead-sol-high or dm-sol-high</x:v>
       </x:c>
       <x:c r="C9" s="24" t="str">
-        <x:v>Bounded explorer only if context merits it</x:v>
+        <x:v>lead-astra-medium or dm-astra-medium for unusually large cross-workstream ambiguity</x:v>
       </x:c>
       <x:c r="D9" s="24" t="str">
-        <x:v>Avoid dispatch and repeated context overhead</x:v>
+        <x:v>Only approved brain profiles interpret missing requirements, choose tradeoffs or settle contracts</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="46" customHeight="1">
       <x:c r="A10" s="24" t="str">
-        <x:v>Small bounded support task</x:v>
+        <x:v>One direct lookup</x:v>
       </x:c>
       <x:c r="B10" s="24" t="str">
-        <x:v>worker-muse-xhigh</x:v>
+        <x:v>Local search/tool when immediate; worker-muse-xhigh when parallel dispatch frees the brain or is faster overall</x:v>
       </x:c>
       <x:c r="C10" s="24" t="str">
-        <x:v>worker-luna-xhigh; worker-luna-max when evidence density warrants</x:v>
+        <x:v>worker-luna-xhigh for bounded read-only evidence when Muse is unavailable</x:v>
       </x:c>
       <x:c r="D10" s="24" t="str">
-        <x:v>Exploration, explicit small edits or test preparation; retain lower-cost leaf lane</x:v>
+        <x:v>Count startup, supervision and handback overhead; delegate when it improves accepted-result time or cost</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="46" customHeight="1">
       <x:c r="A11" s="24" t="str">
-        <x:v>Low/mid complexity development</x:v>
+        <x:v>Light mechanical and read/seek task</x:v>
       </x:c>
       <x:c r="B11" s="24" t="str">
-        <x:v>worker-grok-high; worker-opus-medium; worker-terra-xhigh; worker-sol-medium</x:v>
+        <x:v>worker-muse-xhigh</x:v>
       </x:c>
       <x:c r="C11" s="24" t="str">
-        <x:v>Another eligible profile from this pool</x:v>
+        <x:v>worker-luna-xhigh; worker-luna-max when evidence density warrants</x:v>
       </x:c>
       <x:c r="D11" s="24" t="str">
-        <x:v>Preferred pool, not fixed rank: clear acceptance, known patterns, bounded dependencies; choose fit then speed and available quota</x:v>
+        <x:v>Repository search, localization, evidence collection, narrow checks and small explicit edits; no interpretation</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="46" customHeight="1">
       <x:c r="A12" s="24" t="str">
-        <x:v>Upper-mid complexity development</x:v>
+        <x:v>Low/mid complexity development</x:v>
       </x:c>
       <x:c r="B12" s="24" t="str">
-        <x:v>worker-grok-xhigh; worker-opus-medium</x:v>
+        <x:v>worker-deepseek-flash-high; worker-grok-high; worker-opus-medium; worker-terra-xhigh; worker-sol-medium</x:v>
       </x:c>
       <x:c r="C12" s="24" t="str">
-        <x:v>worker-sol-high or worker-opus-high when ambiguity or consequence warrants escalation</x:v>
+        <x:v>Another eligible profile from this pool</x:v>
       </x:c>
       <x:c r="D12" s="24" t="str">
-        <x:v>Difficult implementation within settled architecture; two primary choices are not claimed equal in capability</x:v>
+        <x:v>Settled behavior, objective acceptance and bounded dependencies; ambiguity already resolved by a brain</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="46" customHeight="1">
       <x:c r="A13" s="24" t="str">
-        <x:v>High complexity development</x:v>
+        <x:v>Upper-mid complexity development</x:v>
       </x:c>
       <x:c r="B13" s="24" t="str">
-        <x:v>worker-sol-high; worker-opus-high</x:v>
+        <x:v>worker-deepseek-flash-high; worker-grok-xhigh; worker-opus-medium</x:v>
       </x:c>
       <x:c r="C13" s="24" t="str">
-        <x:v>Lead/manager resolves architecture or scope before further execution</x:v>
+        <x:v>lead-sol-high resolves ambiguity or consequence; then choose worker-sol-high, worker-opus-high or another qualified mechanical profile</x:v>
       </x:c>
       <x:c r="D13" s="24" t="str">
-        <x:v>Substantial reasoning, sensitive boundaries or coupled contracts; keep mandatory independent risk review</x:v>
+        <x:v>Difficult mechanical implementation within settled architecture; return tradeoffs instead of choosing</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="46" customHeight="1">
       <x:c r="A14" s="24" t="str">
-        <x:v>Demanding but well-defined implementation</x:v>
+        <x:v>High complexity development</x:v>
       </x:c>
       <x:c r="B14" s="24" t="str">
-        <x:v>worker-terra-max</x:v>
+        <x:v>lead-sol-high resolves judgment; worker-opus-high or another qualified mechanical profile executes settled packets</x:v>
       </x:c>
       <x:c r="C14" s="24" t="str">
-        <x:v>High-complexity pool if evidence shows a reasoning blocker</x:v>
+        <x:v>lead-astra-medium resolves unusually large cross-workstream ambiguity before mechanical execution</x:v>
       </x:c>
       <x:c r="D14" s="24" t="str">
-        <x:v>Dense implementation or integration with exact contracts and tests; never assign to outlast a loop</x:v>
+        <x:v>Separate consequential decisions from implementation; independent review remains mandatory</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="46" customHeight="1">
       <x:c r="A15" s="24" t="str">
-        <x:v>Workstream with fixed contracts</x:v>
+        <x:v>Demanding but well-defined implementation</x:v>
       </x:c>
       <x:c r="B15" s="24" t="str">
-        <x:v>lead-terra-xhigh</x:v>
+        <x:v>worker-terra-max; worker-deepseek-flash-high</x:v>
       </x:c>
       <x:c r="C15" s="24" t="str">
-        <x:v>lead-terra-max or lead-sol-medium</x:v>
+        <x:v>High-complexity pool if evidence shows a reasoning blocker; never DeepSeek V4 Pro</x:v>
       </x:c>
       <x:c r="D15" s="24" t="str">
-        <x:v>Lead authority is explicitly assigned; a worker on the same model remains a leaf</x:v>
+        <x:v>Dense mechanical implementation or integration with exact contracts and tests; never assign interpretation or use effort to outlast a loop</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="46" customHeight="1">
       <x:c r="A16" s="24" t="str">
-        <x:v>Consequential architecture or high coupling</x:v>
+        <x:v>Novel public contract implementation</x:v>
       </x:c>
       <x:c r="B16" s="24" t="str">
-        <x:v>lead-sol-high</x:v>
+        <x:v>lead-sol-high settles shape; worker-deepseek-flash-max implements the exact contract</x:v>
       </x:c>
       <x:c r="C16" s="24" t="str">
-        <x:v>lead-astra-medium</x:v>
+        <x:v>lead-astra-medium settles unusually large cross-workstream contract ambiguity before execution</x:v>
       </x:c>
       <x:c r="D16" s="24" t="str">
-        <x:v>Escalate ambiguity or consequence beyond owned workstream</x:v>
+        <x:v>DeepSeek max receives a decided shape and objective contract tests; it does not choose the public contract</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="46" customHeight="1">
       <x:c r="A17" s="24" t="str">
-        <x:v>Cross-workstream planning and decisions</x:v>
+        <x:v>Workstream with fixed contracts</x:v>
       </x:c>
       <x:c r="B17" s="24" t="str">
-        <x:v>dm-astra-medium</x:v>
+        <x:v>lead-terra-xhigh</x:v>
       </x:c>
       <x:c r="C17" s="24" t="str">
-        <x:v>dm-sol-high or dm-opus-high; use directly when already in that configuration; verify transport and handover for house switches</x:v>
+        <x:v>lead-terra-max or lead-sol-medium</x:v>
       </x:c>
       <x:c r="D17" s="24" t="str">
-        <x:v>Manager receives compact exceptions and evidence, not raw logs</x:v>
+        <x:v>Mechanical lead authority may coordinate and delegate settled packets; ambiguity returns to lead-sol-high or lead-astra-medium</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="46" customHeight="1">
       <x:c r="A18" s="24" t="str">
-        <x:v>Independent acceptance</x:v>
+        <x:v>Consequential architecture or high coupling</x:v>
       </x:c>
       <x:c r="B18" s="24" t="str">
-        <x:v>Separate qualified reviewer session</x:v>
+        <x:v>lead-sol-high</x:v>
       </x:c>
       <x:c r="C18" s="24" t="str">
-        <x:v>Another eligible house; same house allowed with reason</x:v>
+        <x:v>lead-astra-medium for unusually large cross-workstream ambiguity</x:v>
       </x:c>
       <x:c r="D18" s="24" t="str">
-        <x:v>Reviewer inspects actual head/artifacts and never fixes its own findings</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20"/>
-      <x:c r="B20"/>
-      <x:c r="C20"/>
-      <x:c r="D20"/>
+        <x:v>Approved brain resolves product, architecture, consequence and coupling before execution</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="46" customHeight="1">
+      <x:c r="A19" s="24" t="str">
+        <x:v>Cross-workstream planning and decisions</x:v>
+      </x:c>
+      <x:c r="B19" s="24" t="str">
+        <x:v>dm-sol-high</x:v>
+      </x:c>
+      <x:c r="C19" s="24" t="str">
+        <x:v>dm-astra-medium for unusually large ambiguity; dm-opus-high may coordinate but routes judgment to a brain</x:v>
+      </x:c>
+      <x:c r="D19" s="24" t="str">
+        <x:v>Manager receives compact exceptions and evidence; only an assigned brain resolves interpretation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="46" customHeight="1">
+      <x:c r="A20" s="24" t="str">
+        <x:v>Independent semantic or risk acceptance</x:v>
+      </x:c>
+      <x:c r="B20" s="24" t="str">
+        <x:v>reviewer-sol-high</x:v>
+      </x:c>
+      <x:c r="C20" s="24" t="str">
+        <x:v>reviewer-astra-medium for unusually large cross-workstream scope</x:v>
+      </x:c>
+      <x:c r="D20" s="24" t="str">
+        <x:v>Mechanical gate collection may be delegated, but acceptance judgment belongs to an independent brain on the exact head</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="180" t="str">
+      <x:c r="A21"/>
+      <x:c r="B21"/>
+      <x:c r="C21"/>
+      <x:c r="D21"/>
+    </x:row>
+    <x:row r="22" ht="42" customHeight="1">
+      <x:c r="A22"/>
+      <x:c r="B22"/>
+      <x:c r="C22"/>
+      <x:c r="D22"/>
+    </x:row>
+    <x:row r="23" ht="42" customHeight="1">
+      <x:c r="A23" s="240" t="str">
         <x:v>Selection rules</x:v>
       </x:c>
-      <x:c r="B21" s="181"/>
-      <x:c r="C21" s="181"/>
-      <x:c r="D21" s="182"/>
-    </x:row>
-    <x:row r="22" ht="42" customHeight="1">
-      <x:c r="A22" s="188" t="str">
+      <x:c r="B23" s="241"/>
+      <x:c r="C23" s="241"/>
+      <x:c r="D23" s="242"/>
+    </x:row>
+    <x:row r="24" ht="42" customHeight="1">
+      <x:c r="A24" s="248" t="str">
         <x:v>Approved selection rule</x:v>
       </x:c>
-      <x:c r="B22" s="189"/>
-      <x:c r="C22" s="189"/>
-      <x:c r="D22" s="190"/>
-    </x:row>
-    <x:row r="23" ht="42" customHeight="1">
-      <x:c r="A23" s="91" t="str">
+      <x:c r="B24" s="249"/>
+      <x:c r="C24" s="249"/>
+      <x:c r="D24" s="250"/>
+    </x:row>
+    <x:row r="25" ht="42" customHeight="1">
+      <x:c r="A25" s="91" t="str">
         <x:v>1. Only Codex, Grok CLI, Claude Code and OpenCode are active houses. Cursor removed from Interchange routing, not uninstalled.</x:v>
       </x:c>
-      <x:c r="B23" s="67"/>
-      <x:c r="C23" s="67"/>
-      <x:c r="D23" s="67"/>
-    </x:row>
-    <x:row r="24" ht="42" customHeight="1">
-      <x:c r="A24" s="92" t="str">
-        <x:v>2. Grok work uses Grok CLI only, model grok-4.6 with high or xhigh. No Cursor route.</x:v>
-      </x:c>
-      <x:c r="B24" s="69"/>
-      <x:c r="C24" s="69"/>
-      <x:c r="D24" s="69"/>
-    </x:row>
-    <x:row r="25" ht="42" customHeight="1">
-      <x:c r="A25" s="92" t="str">
-        <x:v>3. Claude development uses claude-opus-5 medium or high. Sonnet and automatic fallback to it are excluded.</x:v>
-      </x:c>
-      <x:c r="B25" s="69"/>
-      <x:c r="C25" s="69"/>
-      <x:c r="D25" s="69"/>
+      <x:c r="B25" s="67"/>
+      <x:c r="C25" s="67"/>
+      <x:c r="D25" s="67"/>
     </x:row>
     <x:row r="26" ht="42" customHeight="1">
       <x:c r="A26" s="92" t="str">
-        <x:v>4. Treat task bands as routing preferences, not benchmark rankings. Assess ambiguity, consequence, coupling and implementation difficulty separately.</x:v>
+        <x:v>2. Grok work uses Grok CLI only, model grok-4.6 with high or xhigh. No Cursor route.</x:v>
       </x:c>
       <x:c r="B26" s="69"/>
       <x:c r="C26" s="69"/>
@@ -2137,7 +2469,7 @@
     </x:row>
     <x:row r="27" ht="42" customHeight="1">
       <x:c r="A27" s="92" t="str">
-        <x:v>5. Within an eligible pool, use task-fit evidence first, then expected accepted-result latency and available account/pool quota. Pool order is not a ranking.</x:v>
+        <x:v>3. Claude development uses claude-opus-5 medium or high. Sonnet and automatic fallback to it are excluded.</x:v>
       </x:c>
       <x:c r="B27" s="69"/>
       <x:c r="C27" s="69"/>
@@ -2145,7 +2477,7 @@
     </x:row>
     <x:row r="28" ht="42" customHeight="1">
       <x:c r="A28" s="92" t="str">
-        <x:v>6. Use different houses for parallel independent jobs of similar nature when suitable; preserve cached context and session continuity when that is cheaper or faster.</x:v>
+        <x:v>4. Brain boundary: only assigned Sol high, Astra medium and Fable 5.1 medium brain profiles resolve product, behavior, architecture or tradeoff ambiguity. Fable is for product ideation; Astra is for unusually large cross-workstream ambiguity; Sol high is the default.</x:v>
       </x:c>
       <x:c r="B28" s="69"/>
       <x:c r="C28" s="69"/>
@@ -2153,7 +2485,7 @@
     </x:row>
     <x:row r="29" ht="42" customHeight="1">
       <x:c r="A29" s="92" t="str">
-        <x:v>7. More reasoning is not universally more intelligence or better value. Terra max handles difficult settled implementation, not unresolved product decisions.</x:v>
+        <x:v>5. Semantic and risk acceptance is a brain task: use an independent Sol high reviewer, or Astra medium for unusually large cross-workstream scope. Mechanical workers may collect gates but cannot issue acceptance judgment.</x:v>
       </x:c>
       <x:c r="B29" s="69"/>
       <x:c r="C29" s="69"/>
@@ -2161,7 +2493,7 @@
     </x:row>
     <x:row r="30" ht="42" customHeight="1">
       <x:c r="A30" s="92" t="str">
-        <x:v>8. No automatic repeated effort increases. Stop, diagnose or reassign under existing watchdog and recovery limits.</x:v>
+        <x:v>6. Coordination is not judgment authority. Opus delivery managers and mechanical leads may coordinate, monitor and integrate, but route unresolved interpretation to an approved brain.</x:v>
       </x:c>
       <x:c r="B30" s="69"/>
       <x:c r="C30" s="69"/>
@@ -2169,7 +2501,7 @@
     </x:row>
     <x:row r="31" ht="42" customHeight="1">
       <x:c r="A31" s="92" t="str">
-        <x:v>9. Do not send every tiny job to the primary developer pool. Muse/Luna remain eligible bounded support workers.</x:v>
+        <x:v>7. Mechanical packets contain settled behavior, objective acceptance, owned paths, allowed variance and an escalation condition. Workers return evidence and the smallest question when a choice requires interpretation.</x:v>
       </x:c>
       <x:c r="B31" s="69"/>
       <x:c r="C31" s="69"/>
@@ -2177,7 +2509,7 @@
     </x:row>
     <x:row r="32" ht="42" customHeight="1">
       <x:c r="A32" s="92" t="str">
-        <x:v>10. High consequence can require stronger review even for a small edit. Model choice never removes acceptance gates.</x:v>
+        <x:v>8. Use fast, low-cost mechanical workers when startup, supervision and integration overhead still improves accepted-result time or cost. Parallelize independent objectively testable packets after decisions, interfaces and write ownership are fixed.</x:v>
       </x:c>
       <x:c r="B32" s="69"/>
       <x:c r="C32" s="69"/>
@@ -2185,7 +2517,7 @@
     </x:row>
     <x:row r="33" ht="42" customHeight="1">
       <x:c r="A33" s="92" t="str">
-        <x:v>11. Verify effective model and effort at dispatch. Newly configured Grok/Opus combinations are not yet claimed smoke-tested; no unapproved substitution.</x:v>
+        <x:v>9. Muse Spark 1.3 is the preferred light mechanical and read/seek lane for repository search, file localization, evidence collection, narrow checks and small explicit edits.</x:v>
       </x:c>
       <x:c r="B33" s="69"/>
       <x:c r="C33" s="69"/>
@@ -2193,7 +2525,7 @@
     </x:row>
     <x:row r="34" ht="42" customHeight="1">
       <x:c r="A34" s="92" t="str">
-        <x:v>12. House exclusivity has two scopes. Astra at any effort reserves Codex globally and Fable 5.1 at any effort reserves Claude globally. Sol high or higher reserves Codex only for assignments under the same delivery manager; Opus high or higher reserves Claude only for assignments under the same delivery manager.</x:v>
+        <x:v>10. Do not fragment work when dispatch, context transfer or integration overhead would erase the expected speed or cost gain.</x:v>
       </x:c>
       <x:c r="B34" s="69"/>
       <x:c r="C34" s="69"/>
@@ -2201,7 +2533,7 @@
     </x:row>
     <x:row r="35" ht="42" customHeight="1">
       <x:c r="A35" s="92" t="str">
-        <x:v>13. New-product brainstorming may use Fable 5.1 medium or Astra medium. Both create global house reservations while active; prefer another eligible house or queue competing work.</x:v>
+        <x:v>11. More reasoning is not universally more intelligence or better value. Terra max handles difficult settled implementation, not unresolved product decisions.</x:v>
       </x:c>
       <x:c r="B35" s="69"/>
       <x:c r="C35" s="69"/>
@@ -2209,7 +2541,7 @@
     </x:row>
     <x:row r="36" ht="42" customHeight="1">
       <x:c r="A36" s="92" t="str">
-        <x:v>14. Fable model authorization does not permit paid usage credits or extra spending. Verify included allowance before any headless request.</x:v>
+        <x:v>12. No automatic repeated effort increases. Stop, diagnose or reassign under existing watchdog and recovery limits.</x:v>
       </x:c>
       <x:c r="B36" s="69"/>
       <x:c r="C36" s="69"/>
@@ -2217,7 +2549,7 @@
     </x:row>
     <x:row r="37" ht="42" customHeight="1">
       <x:c r="A37" s="92" t="str">
-        <x:v>15. The delivery manager keeps its turn active with a real bounded wait while workers run. It may finish only after terminal handbacks or explicit transfer to another live supervisor.</x:v>
+        <x:v>13. High consequence can require stronger review even for a small edit. Model choice never removes acceptance gates.</x:v>
       </x:c>
       <x:c r="B37" s="69"/>
       <x:c r="C37" s="69"/>
@@ -2225,7 +2557,7 @@
     </x:row>
     <x:row r="38" ht="42" customHeight="1">
       <x:c r="A38" s="92" t="str">
-        <x:v>16. External provider streams are drained outside manager context. Retrieve compact lifecycle changes and the mechanically extracted final assistant result, not accumulated raw output.</x:v>
+        <x:v>14. Verify effective model and effort at dispatch. Newly configured Grok/Opus combinations are not yet claimed smoke-tested; no unapproved substitution.</x:v>
       </x:c>
       <x:c r="B38" s="69"/>
       <x:c r="C38" s="69"/>
@@ -2233,7 +2565,7 @@
     </x:row>
     <x:row r="39" ht="42" customHeight="1">
       <x:c r="A39" s="92" t="str">
-        <x:v>17. A provider parent exit does not transfer writer ownership. Verify process tree, worktree command/CWD holders and provider background-agent registry before any replacement writer.</x:v>
+        <x:v>15. House exclusivity has two scopes. Astra at any effort reserves Codex globally and Fable 5.1 at any effort reserves Claude globally. Sol high or higher reserves Codex only for assignments under the same delivery manager; Opus high or higher reserves Claude only for assignments under the same delivery manager.</x:v>
       </x:c>
       <x:c r="B39" s="69"/>
       <x:c r="C39" s="69"/>
@@ -2241,7 +2573,7 @@
     </x:row>
     <x:row r="40" ht="42" customHeight="1">
       <x:c r="A40" s="92" t="str">
-        <x:v>18. Stop Claude after two consecutive no-progress auto-compactions; checkpoint and use one fresh narrow retry rather than resuming the thrashing session.</x:v>
+        <x:v>16. New-product brainstorming may use Fable 5.1 medium or Astra medium. Both create global house reservations while active; prefer another eligible house or queue competing work.</x:v>
       </x:c>
       <x:c r="B40" s="69"/>
       <x:c r="C40" s="69"/>
@@ -2249,16 +2581,78 @@
     </x:row>
     <x:row r="41" ht="42" customHeight="1">
       <x:c r="A41" s="92" t="str">
-        <x:v>19. Owner concurrency exceptions are finite and journalled after an occupancy probe; leads and managers cannot self-authorize them.</x:v>
+        <x:v>17. Fable model authorization does not permit paid usage credits or extra spending. Verify included allowance before any headless request.</x:v>
       </x:c>
       <x:c r="B41" s="69"/>
       <x:c r="C41" s="69"/>
       <x:c r="D41" s="69"/>
     </x:row>
+    <x:row r="42" ht="42" customHeight="1">
+      <x:c r="A42" s="92" t="str">
+        <x:v>18. The delivery manager keeps its turn active with a real bounded wait while workers run. It may finish only after terminal handbacks or explicit transfer to another live supervisor.</x:v>
+      </x:c>
+      <x:c r="B42" s="69"/>
+      <x:c r="C42" s="69"/>
+      <x:c r="D42" s="69"/>
+    </x:row>
+    <x:row r="43" ht="42" customHeight="1">
+      <x:c r="A43" s="92" t="str">
+        <x:v>19. External provider streams are drained outside manager context. Retrieve compact lifecycle changes and the mechanically extracted final assistant result, not accumulated raw output.</x:v>
+      </x:c>
+      <x:c r="B43" s="69"/>
+      <x:c r="C43" s="69"/>
+      <x:c r="D43" s="69"/>
+    </x:row>
+    <x:row r="44" ht="42" customHeight="1">
+      <x:c r="A44" s="92" t="str">
+        <x:v>20. A provider parent exit does not transfer writer ownership. Verify process tree, worktree command/CWD holders and provider background-agent registry before any replacement writer.</x:v>
+      </x:c>
+      <x:c r="B44" s="69"/>
+      <x:c r="C44" s="69"/>
+      <x:c r="D44" s="69"/>
+    </x:row>
+    <x:row r="45" ht="42" customHeight="1">
+      <x:c r="A45" s="92" t="str">
+        <x:v>21. Stop Claude after two consecutive no-progress auto-compactions; checkpoint and use one fresh narrow retry rather than resuming the thrashing session.</x:v>
+      </x:c>
+      <x:c r="B45" s="69"/>
+      <x:c r="C45" s="69"/>
+      <x:c r="D45" s="69"/>
+    </x:row>
+    <x:row r="46" ht="42" customHeight="1">
+      <x:c r="A46" s="92" t="str">
+        <x:v>22. Owner concurrency exceptions are finite and journalled after an occupancy probe; leads and managers cannot self-authorize them.</x:v>
+      </x:c>
+      <x:c r="B46" s="69"/>
+      <x:c r="C46" s="69"/>
+      <x:c r="D46" s="69"/>
+    </x:row>
+    <x:row r="47" ht="42" customHeight="1">
+      <x:c r="A47" s="92" t="str">
+        <x:v>23. DeepSeek V4.1 Flash uses the provider code opencode-go/deepseek-v4.1-flash. The human-readable name and provider code identify the same approved model. The provider renamed this code from opencode-go/deepseek-flash, which no longer appears in `opencode models`; the version now lives in the code itself.</x:v>
+      </x:c>
+      <x:c r="B47" s="69"/>
+      <x:c r="C47" s="69"/>
+      <x:c r="D47" s="69"/>
+    </x:row>
+    <x:row r="48" ht="42" customHeight="1">
+      <x:c r="A48" s="92" t="str">
+        <x:v>24. DeepSeek high is the default for bounded implementation. DeepSeek max mechanically implements novel public contract, identity, schema or serialization shapes only after an approved brain settles the shape and objective contract tests.</x:v>
+      </x:c>
+      <x:c r="B48" s="69"/>
+      <x:c r="C48" s="69"/>
+      <x:c r="D48" s="69"/>
+    </x:row>
+    <x:row r="49" ht="42" customHeight="1">
+      <x:c r="A49" s="92" t="str">
+        <x:v>25. DeepSeek V4 Pro, DeepSeek V4 Flash and the vision-exp variants are excluded: opencode-go/deepseek-v4-pro, opencode-go/deepseek-v4-flash and opencode-go/deepseek-v4-flash-vision-exp are DIFFERENT models, not fallbacks for V4.1 Flash. If opencode-go/deepseek-v4.1-flash is unavailable, stop and reroute to a different approved house; never substitute another DeepSeek model.</x:v>
+      </x:c>
+      <x:c r="B49" s="69"/>
+      <x:c r="C49" s="69"/>
+      <x:c r="D49" s="69"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A22:D22"/>
-    <x:mergeCell ref="A23:D23"/>
     <x:mergeCell ref="A24:D24"/>
     <x:mergeCell ref="A25:D25"/>
     <x:mergeCell ref="A26:D26"/>
@@ -2277,6 +2671,14 @@
     <x:mergeCell ref="A39:D39"/>
     <x:mergeCell ref="A40:D40"/>
     <x:mergeCell ref="A41:D41"/>
+    <x:mergeCell ref="A42:D42"/>
+    <x:mergeCell ref="A43:D43"/>
+    <x:mergeCell ref="A44:D44"/>
+    <x:mergeCell ref="A45:D45"/>
+    <x:mergeCell ref="A46:D46"/>
+    <x:mergeCell ref="A47:D47"/>
+    <x:mergeCell ref="A48:D48"/>
+    <x:mergeCell ref="A49:D49"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2308,13 +2710,13 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>Policy source: Interchange policy v0.4.0</x:v>
+        <x:v>Policy source: Interchange policy v0.6.0</x:v>
       </x:c>
       <x:c r="B3" s="2" t="str">
         <x:v>Approved on</x:v>
       </x:c>
       <x:c r="C3" s="5" t="n">
-        <x:v>46274</x:v>
+        <x:v>46278</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -2519,13 +2921,13 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>Policy source: Interchange policy v0.4.0</x:v>
+        <x:v>Policy source: Interchange policy v0.6.0</x:v>
       </x:c>
       <x:c r="B3" s="2" t="str">
         <x:v>Approved on</x:v>
       </x:c>
       <x:c r="C3" s="5" t="n">
-        <x:v>46274</x:v>
+        <x:v>46278</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -2595,7 +2997,7 @@
         <x:v>Spending</x:v>
       </x:c>
       <x:c r="B12" s="24" t="str">
-        <x:v>No extra purchases or automatic recharge; existing OpenCode Go allowance/balance may be used for Muse only</x:v>
+        <x:v>No extra purchases or automatic recharge; existing OpenCode Go allowance/balance may be used for approved Muse and DeepSeek Flash profiles; DeepSeek V4 Pro is excluded</x:v>
       </x:c>
       <x:c r="C12"/>
     </x:row>
@@ -2682,20 +3084,20 @@
       <x:c r="C22"/>
     </x:row>
     <x:row r="23" ht="26" customHeight="1">
-      <x:c r="A23" s="180" t="str">
+      <x:c r="A23" s="240" t="str">
         <x:v>Recovery playbook</x:v>
       </x:c>
-      <x:c r="B23" s="181"/>
-      <x:c r="C23" s="182"/>
+      <x:c r="B23" s="241"/>
+      <x:c r="C23" s="242"/>
     </x:row>
     <x:row r="24" ht="44" customHeight="1">
-      <x:c r="A24" s="188" t="str">
+      <x:c r="A24" s="248" t="str">
         <x:v>Failure</x:v>
       </x:c>
-      <x:c r="B24" s="189" t="str">
+      <x:c r="B24" s="249" t="str">
         <x:v>First action</x:v>
       </x:c>
-      <x:c r="C24" s="190" t="str">
+      <x:c r="C24" s="250" t="str">
         <x:v>Escalation</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
feat(interchange): conserve Codex capacity
</commit_message>
<xml_diff>
--- a/outputs/interchange-design/interchange.xlsx
+++ b/outputs/interchange-design/interchange.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profiles" sheetId="1" r:id="R54bb1c1b109c4a81"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Routing" sheetId="2" r:id="Ra5fa34cf7b594df6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monitoring" sheetId="3" r:id="R9861e40f1bfe4770"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Recovery" sheetId="4" r:id="Re075d54395954ed3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profiles" sheetId="1" r:id="Rd9241db062e94bfd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Routing" sheetId="2" r:id="Rae13d59e66494d0b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monitoring" sheetId="3" r:id="R2bda169c4e1245d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Recovery" sheetId="4" r:id="R3477effca99e4dce"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -55,7 +55,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="51">
+  <x:fills count="59">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -85,6 +85,46 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFCE4D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -380,7 +420,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="251">
+  <x:cellXfs count="287">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -990,6 +1030,86 @@
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="50" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="51" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="51" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="52" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="52" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="51" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="53" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="53" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="53" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="53" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="53" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="54" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="54" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="54" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="54" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="54" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="54" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="54" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="54" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="55" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="55" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="56" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="56" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="55" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="57" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="57" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="57" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="57" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="57" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="58" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="58" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="58" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="58" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="58" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="58" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="58" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="58" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1234,7 +1354,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>Policy source: Interchange policy v0.6.0</x:v>
+        <x:v>Policy source: Interchange policy v0.7.0</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -1457,10 +1577,10 @@
       <x:c r="F16" s="34" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G16" s="233" t="str">
+      <x:c r="G16" s="269" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H16" s="235" t="str">
+      <x:c r="H16" s="271" t="str">
         <x:v>Profile documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I16" s="22" t="str">
@@ -1486,10 +1606,10 @@
       <x:c r="F17" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G17" s="234" t="str">
+      <x:c r="G17" s="270" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H17" s="236" t="str">
+      <x:c r="H17" s="272" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I17" s="24" t="str">
@@ -1515,10 +1635,10 @@
       <x:c r="F18" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G18" s="234" t="str">
+      <x:c r="G18" s="270" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H18" s="236" t="str">
+      <x:c r="H18" s="272" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I18" s="24" t="str">
@@ -1544,10 +1664,10 @@
       <x:c r="F19" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G19" s="234" t="str">
+      <x:c r="G19" s="270" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H19" s="236" t="str">
+      <x:c r="H19" s="272" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I19" s="24" t="str">
@@ -1573,10 +1693,10 @@
       <x:c r="F20" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G20" s="234" t="str">
+      <x:c r="G20" s="270" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H20" s="236" t="str">
+      <x:c r="H20" s="272" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I20" s="24" t="str">
@@ -1602,10 +1722,10 @@
       <x:c r="F21" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G21" s="234" t="str">
+      <x:c r="G21" s="270" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H21" s="236" t="str">
+      <x:c r="H21" s="272" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I21" s="24" t="str">
@@ -1631,10 +1751,10 @@
       <x:c r="F22" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G22" s="234" t="str">
+      <x:c r="G22" s="270" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H22" s="236" t="str">
+      <x:c r="H22" s="272" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I22" s="24" t="str">
@@ -1660,10 +1780,10 @@
       <x:c r="F23" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G23" s="234" t="str">
+      <x:c r="G23" s="270" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H23" s="236" t="str">
+      <x:c r="H23" s="272" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I23" s="24" t="str">
@@ -1689,10 +1809,10 @@
       <x:c r="F24" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G24" s="234" t="str">
+      <x:c r="G24" s="270" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H24" s="236" t="str">
+      <x:c r="H24" s="272" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I24" s="24" t="str">
@@ -1718,10 +1838,10 @@
       <x:c r="F25" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G25" s="234" t="str">
+      <x:c r="G25" s="270" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H25" s="236" t="str">
+      <x:c r="H25" s="272" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I25" s="24" t="str">
@@ -1747,10 +1867,10 @@
       <x:c r="F26" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G26" s="234" t="str">
+      <x:c r="G26" s="270" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H26" s="236" t="str">
+      <x:c r="H26" s="272" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I26" s="24" t="str">
@@ -1776,10 +1896,10 @@
       <x:c r="F27" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G27" s="234" t="str">
+      <x:c r="G27" s="270" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H27" s="236" t="str">
+      <x:c r="H27" s="272" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I27" s="24" t="str">
@@ -1805,10 +1925,10 @@
       <x:c r="F28" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G28" s="234" t="str">
+      <x:c r="G28" s="270" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H28" s="236" t="str">
+      <x:c r="H28" s="272" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I28" s="24" t="str">
@@ -1834,10 +1954,10 @@
       <x:c r="F29" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G29" s="234" t="str">
+      <x:c r="G29" s="270" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H29" s="237" t="str">
+      <x:c r="H29" s="273" t="str">
         <x:v>Smoke-tested</x:v>
       </x:c>
       <x:c r="I29" s="24" t="str">
@@ -1863,10 +1983,10 @@
       <x:c r="F30" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G30" s="234" t="str">
+      <x:c r="G30" s="270" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H30" s="236" t="str">
+      <x:c r="H30" s="272" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I30" s="24" t="str">
@@ -1892,10 +2012,10 @@
       <x:c r="F31" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G31" s="234" t="str">
+      <x:c r="G31" s="270" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H31" s="236" t="str">
+      <x:c r="H31" s="272" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I31" s="24" t="str">
@@ -1921,10 +2041,10 @@
       <x:c r="F32" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G32" s="234" t="str">
+      <x:c r="G32" s="270" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H32" s="236" t="str">
+      <x:c r="H32" s="272" t="str">
         <x:v>CLI model and effort documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I32" s="24" t="str">
@@ -1950,10 +2070,10 @@
       <x:c r="F33" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G33" s="234" t="str">
+      <x:c r="G33" s="270" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H33" s="236" t="str">
+      <x:c r="H33" s="272" t="str">
         <x:v>CLI model and effort documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I33" s="24" t="str">
@@ -1979,10 +2099,10 @@
       <x:c r="F34" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G34" s="234" t="str">
+      <x:c r="G34" s="270" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H34" s="236" t="str">
+      <x:c r="H34" s="272" t="str">
         <x:v>Profile documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I34" s="24" t="str">
@@ -2008,10 +2128,10 @@
       <x:c r="F35" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G35" s="234" t="str">
+      <x:c r="G35" s="270" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H35" s="236" t="str">
+      <x:c r="H35" s="272" t="str">
         <x:v>Profile documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I35" s="24" t="str">
@@ -2037,10 +2157,10 @@
       <x:c r="F36" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G36" s="234" t="str">
+      <x:c r="G36" s="270" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H36" s="236" t="str">
+      <x:c r="H36" s="272" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I36" s="24" t="str">
@@ -2066,10 +2186,10 @@
       <x:c r="F37" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G37" s="234" t="str">
+      <x:c r="G37" s="270" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H37" s="236" t="str">
+      <x:c r="H37" s="272" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I37" s="24" t="str">
@@ -2095,10 +2215,10 @@
       <x:c r="F38" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G38" s="234" t="str">
+      <x:c r="G38" s="270" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H38" s="236" t="str">
+      <x:c r="H38" s="272" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I38" s="24" t="str">
@@ -2124,10 +2244,10 @@
       <x:c r="F39" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G39" s="234" t="str">
+      <x:c r="G39" s="270" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H39" s="236" t="str">
+      <x:c r="H39" s="272" t="str">
         <x:v>Profile documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I39" s="24" t="str">
@@ -2153,10 +2273,10 @@
       <x:c r="F40" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G40" s="234" t="str">
+      <x:c r="G40" s="270" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H40" s="236" t="str">
+      <x:c r="H40" s="272" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I40" s="24" t="str">
@@ -2197,7 +2317,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>Policy source: Interchange policy v0.6.0</x:v>
+        <x:v>Policy source: Interchange policy v0.7.0</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2" t="str">
@@ -2274,10 +2394,10 @@
         <x:v>One direct lookup</x:v>
       </x:c>
       <x:c r="B10" s="24" t="str">
-        <x:v>Local search/tool when immediate; worker-muse-xhigh when parallel dispatch frees the brain or is faster overall</x:v>
+        <x:v>Local search/tool when immediate; worker-muse-xhigh when delegation frees the Codex brain or is faster overall</x:v>
       </x:c>
       <x:c r="C10" s="24" t="str">
-        <x:v>worker-luna-xhigh for bounded read-only evidence when Muse is unavailable</x:v>
+        <x:v>Another external read-only mechanical profile; Codex worker only under a recorded mechanical allowance</x:v>
       </x:c>
       <x:c r="D10" s="24" t="str">
         <x:v>Count startup, supervision and handback overhead; delegate when it improves accepted-result time or cost</x:v>
@@ -2291,7 +2411,7 @@
         <x:v>worker-muse-xhigh</x:v>
       </x:c>
       <x:c r="C11" s="24" t="str">
-        <x:v>worker-luna-xhigh; worker-luna-max when evidence density warrants</x:v>
+        <x:v>Another external bounded worker; Luna xhigh/max only under a recorded Codex mechanical allowance</x:v>
       </x:c>
       <x:c r="D11" s="24" t="str">
         <x:v>Repository search, localization, evidence collection, narrow checks and small explicit edits; no interpretation</x:v>
@@ -2305,7 +2425,7 @@
         <x:v>worker-deepseek-flash-high; worker-grok-high; worker-opus-medium; worker-terra-xhigh; worker-sol-medium</x:v>
       </x:c>
       <x:c r="C12" s="24" t="str">
-        <x:v>Another eligible profile from this pool</x:v>
+        <x:v>Codex worker from this pool only under a recorded mechanical allowance and after external fit/availability check</x:v>
       </x:c>
       <x:c r="D12" s="24" t="str">
         <x:v>Settled behavior, objective acceptance and bounded dependencies; ambiguity already resolved by a brain</x:v>
@@ -2319,7 +2439,7 @@
         <x:v>worker-deepseek-flash-high; worker-grok-xhigh; worker-opus-medium</x:v>
       </x:c>
       <x:c r="C13" s="24" t="str">
-        <x:v>lead-sol-high resolves ambiguity or consequence; then choose worker-sol-high, worker-opus-high or another qualified mechanical profile</x:v>
+        <x:v>lead-sol-high resolves ambiguity; choose an external mechanical worker first, or a Codex worker under a recorded allowance</x:v>
       </x:c>
       <x:c r="D13" s="24" t="str">
         <x:v>Difficult mechanical implementation within settled architecture; return tradeoffs instead of choosing</x:v>
@@ -2330,10 +2450,10 @@
         <x:v>High complexity development</x:v>
       </x:c>
       <x:c r="B14" s="24" t="str">
-        <x:v>lead-sol-high resolves judgment; worker-opus-high or another qualified mechanical profile executes settled packets</x:v>
+        <x:v>lead-sol-high resolves judgment; worker-opus-high or another qualified external profile executes settled packets</x:v>
       </x:c>
       <x:c r="C14" s="24" t="str">
-        <x:v>lead-astra-medium resolves unusually large cross-workstream ambiguity before mechanical execution</x:v>
+        <x:v>lead-astra-medium resolves unusually large ambiguity; Codex mechanical worker requires a recorded allowance</x:v>
       </x:c>
       <x:c r="D14" s="24" t="str">
         <x:v>Separate consequential decisions from implementation; independent review remains mandatory</x:v>
@@ -2344,10 +2464,10 @@
         <x:v>Demanding but well-defined implementation</x:v>
       </x:c>
       <x:c r="B15" s="24" t="str">
-        <x:v>worker-terra-max; worker-deepseek-flash-high</x:v>
+        <x:v>worker-deepseek-flash-high; worker-opus-high</x:v>
       </x:c>
       <x:c r="C15" s="24" t="str">
-        <x:v>High-complexity pool if evidence shows a reasoning blocker; never DeepSeek V4 Pro</x:v>
+        <x:v>worker-terra-max only under a recorded Codex mechanical allowance; never DeepSeek V4 Pro</x:v>
       </x:c>
       <x:c r="D15" s="24" t="str">
         <x:v>Dense mechanical implementation or integration with exact contracts and tests; never assign interpretation or use effort to outlast a loop</x:v>
@@ -2372,13 +2492,13 @@
         <x:v>Workstream with fixed contracts</x:v>
       </x:c>
       <x:c r="B17" s="24" t="str">
-        <x:v>lead-terra-xhigh</x:v>
+        <x:v>Current delivery manager coordinates settled packets across external mechanical workers</x:v>
       </x:c>
       <x:c r="C17" s="24" t="str">
-        <x:v>lead-terra-max or lead-sol-medium</x:v>
+        <x:v>lead-terra-xhigh/max only under a recorded Codex mechanical allowance</x:v>
       </x:c>
       <x:c r="D17" s="24" t="str">
-        <x:v>Mechanical lead authority may coordinate and delegate settled packets; ambiguity returns to lead-sol-high or lead-astra-medium</x:v>
+        <x:v>Preserve Codex brain capacity; a mechanical lead coordinates only settled work and returns ambiguity to Sol high or Astra medium</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="46" customHeight="1">
@@ -2420,7 +2540,7 @@
         <x:v>reviewer-astra-medium for unusually large cross-workstream scope</x:v>
       </x:c>
       <x:c r="D20" s="24" t="str">
-        <x:v>Mechanical gate collection may be delegated, but acceptance judgment belongs to an independent brain on the exact head</x:v>
+        <x:v>Run gates mechanically; batch one independent brain review at a meaningful integrated chunk boundary and bind it to the exact head</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -2436,20 +2556,20 @@
       <x:c r="D22"/>
     </x:row>
     <x:row r="23" ht="42" customHeight="1">
-      <x:c r="A23" s="240" t="str">
+      <x:c r="A23" s="276" t="str">
         <x:v>Selection rules</x:v>
       </x:c>
-      <x:c r="B23" s="241"/>
-      <x:c r="C23" s="241"/>
-      <x:c r="D23" s="242"/>
+      <x:c r="B23" s="277"/>
+      <x:c r="C23" s="277"/>
+      <x:c r="D23" s="278"/>
     </x:row>
     <x:row r="24" ht="42" customHeight="1">
-      <x:c r="A24" s="248" t="str">
+      <x:c r="A24" s="284" t="str">
         <x:v>Approved selection rule</x:v>
       </x:c>
-      <x:c r="B24" s="249"/>
-      <x:c r="C24" s="249"/>
-      <x:c r="D24" s="250"/>
+      <x:c r="B24" s="285"/>
+      <x:c r="C24" s="285"/>
+      <x:c r="D24" s="286"/>
     </x:row>
     <x:row r="25" ht="42" customHeight="1">
       <x:c r="A25" s="91" t="str">
@@ -2509,7 +2629,7 @@
     </x:row>
     <x:row r="32" ht="42" customHeight="1">
       <x:c r="A32" s="92" t="str">
-        <x:v>8. Use fast, low-cost mechanical workers when startup, supervision and integration overhead still improves accepted-result time or cost. Parallelize independent objectively testable packets after decisions, interfaces and write ownership are fixed.</x:v>
+        <x:v>8. Owner may set Codex delegation or leading to zero for a delivery. This overrides any planned mechanical allowance and preserves only explicitly requested Codex brain/review use.</x:v>
       </x:c>
       <x:c r="B32" s="69"/>
       <x:c r="C32" s="69"/>
@@ -2517,7 +2637,7 @@
     </x:row>
     <x:row r="33" ht="42" customHeight="1">
       <x:c r="A33" s="92" t="str">
-        <x:v>9. Muse Spark 1.3 is the preferred light mechanical and read/seek lane for repository search, file localization, evidence collection, narrow checks and small explicit edits.</x:v>
+        <x:v>9. Codex capacity is reserved for product/architecture judgment, integration decisions and independent semantic/risk review across the full usage window. Model quality alone does not justify Codex mechanical execution.</x:v>
       </x:c>
       <x:c r="B33" s="69"/>
       <x:c r="C33" s="69"/>
@@ -2525,7 +2645,7 @@
     </x:row>
     <x:row r="34" ht="42" customHeight="1">
       <x:c r="A34" s="92" t="str">
-        <x:v>10. Do not fragment work when dispatch, context transfer or integration overhead would erase the expected speed or cost gain.</x:v>
+        <x:v>10. External houses are the default mechanical lane. A Codex mechanical worker needs a recorded delivery allowance and reason; absence of an allowance means zero Codex mechanical dispatch.</x:v>
       </x:c>
       <x:c r="B34" s="69"/>
       <x:c r="C34" s="69"/>
@@ -2533,7 +2653,7 @@
     </x:row>
     <x:row r="35" ht="42" customHeight="1">
       <x:c r="A35" s="92" t="str">
-        <x:v>11. More reasoning is not universally more intelligence or better value. Terra max handles difficult settled implementation, not unresolved product decisions.</x:v>
+        <x:v>11. Codex mechanical concurrency defaults to one. Parallel Codex mechanical workers require explicit owner authorization; use qualified external houses for parallel execution.</x:v>
       </x:c>
       <x:c r="B35" s="69"/>
       <x:c r="C35" s="69"/>
@@ -2541,7 +2661,7 @@
     </x:row>
     <x:row r="36" ht="42" customHeight="1">
       <x:c r="A36" s="92" t="str">
-        <x:v>12. No automatic repeated effort increases. Stop, diagnose or reassign under existing watchdog and recovery limits.</x:v>
+        <x:v>12. Batch Codex brain questions and integrated reviews. Send compact evidence and exceptions gathered by mechanical workers instead of using Codex for broad repository exploration.</x:v>
       </x:c>
       <x:c r="B36" s="69"/>
       <x:c r="C36" s="69"/>
@@ -2549,7 +2669,7 @@
     </x:row>
     <x:row r="37" ht="42" customHeight="1">
       <x:c r="A37" s="92" t="str">
-        <x:v>13. High consequence can require stronger review even for a small edit. Model choice never removes acceptance gates.</x:v>
+        <x:v>13. Run build, test and evidence collection mechanically. Use one Sol-high semantic/risk review per meaningful integrated chunk; new remedy commits still require exact-head re-review.</x:v>
       </x:c>
       <x:c r="B37" s="69"/>
       <x:c r="C37" s="69"/>
@@ -2557,7 +2677,7 @@
     </x:row>
     <x:row r="38" ht="42" customHeight="1">
       <x:c r="A38" s="92" t="str">
-        <x:v>14. Verify effective model and effort at dispatch. Newly configured Grok/Opus combinations are not yet claimed smoke-tested; no unapproved substitution.</x:v>
+        <x:v>14. Use fast, low-cost mechanical workers when startup, supervision and integration overhead still improves accepted-result time or cost. Parallelize independent objectively testable packets after decisions, interfaces and write ownership are fixed.</x:v>
       </x:c>
       <x:c r="B38" s="69"/>
       <x:c r="C38" s="69"/>
@@ -2565,7 +2685,7 @@
     </x:row>
     <x:row r="39" ht="42" customHeight="1">
       <x:c r="A39" s="92" t="str">
-        <x:v>15. House exclusivity has two scopes. Astra at any effort reserves Codex globally and Fable 5.1 at any effort reserves Claude globally. Sol high or higher reserves Codex only for assignments under the same delivery manager; Opus high or higher reserves Claude only for assignments under the same delivery manager.</x:v>
+        <x:v>15. Muse Spark 1.3 is the preferred light mechanical and read/seek lane for repository search, file localization, evidence collection, narrow checks and small explicit edits.</x:v>
       </x:c>
       <x:c r="B39" s="69"/>
       <x:c r="C39" s="69"/>
@@ -2573,7 +2693,7 @@
     </x:row>
     <x:row r="40" ht="42" customHeight="1">
       <x:c r="A40" s="92" t="str">
-        <x:v>16. New-product brainstorming may use Fable 5.1 medium or Astra medium. Both create global house reservations while active; prefer another eligible house or queue competing work.</x:v>
+        <x:v>16. Do not fragment work when dispatch, context transfer or integration overhead would erase the expected speed or cost gain.</x:v>
       </x:c>
       <x:c r="B40" s="69"/>
       <x:c r="C40" s="69"/>
@@ -2581,7 +2701,7 @@
     </x:row>
     <x:row r="41" ht="42" customHeight="1">
       <x:c r="A41" s="92" t="str">
-        <x:v>17. Fable model authorization does not permit paid usage credits or extra spending. Verify included allowance before any headless request.</x:v>
+        <x:v>17. More reasoning is not universally more intelligence or better value. Terra max handles difficult settled implementation, not unresolved product decisions.</x:v>
       </x:c>
       <x:c r="B41" s="69"/>
       <x:c r="C41" s="69"/>
@@ -2589,7 +2709,7 @@
     </x:row>
     <x:row r="42" ht="42" customHeight="1">
       <x:c r="A42" s="92" t="str">
-        <x:v>18. The delivery manager keeps its turn active with a real bounded wait while workers run. It may finish only after terminal handbacks or explicit transfer to another live supervisor.</x:v>
+        <x:v>18. No automatic repeated effort increases. Stop, diagnose or reassign under existing watchdog and recovery limits.</x:v>
       </x:c>
       <x:c r="B42" s="69"/>
       <x:c r="C42" s="69"/>
@@ -2597,7 +2717,7 @@
     </x:row>
     <x:row r="43" ht="42" customHeight="1">
       <x:c r="A43" s="92" t="str">
-        <x:v>19. External provider streams are drained outside manager context. Retrieve compact lifecycle changes and the mechanically extracted final assistant result, not accumulated raw output.</x:v>
+        <x:v>19. High consequence can require stronger review even for a small edit. Model choice never removes acceptance gates.</x:v>
       </x:c>
       <x:c r="B43" s="69"/>
       <x:c r="C43" s="69"/>
@@ -2605,7 +2725,7 @@
     </x:row>
     <x:row r="44" ht="42" customHeight="1">
       <x:c r="A44" s="92" t="str">
-        <x:v>20. A provider parent exit does not transfer writer ownership. Verify process tree, worktree command/CWD holders and provider background-agent registry before any replacement writer.</x:v>
+        <x:v>20. Verify effective model and effort at dispatch. Newly configured Grok/Opus combinations are not yet claimed smoke-tested; no unapproved substitution.</x:v>
       </x:c>
       <x:c r="B44" s="69"/>
       <x:c r="C44" s="69"/>
@@ -2613,7 +2733,7 @@
     </x:row>
     <x:row r="45" ht="42" customHeight="1">
       <x:c r="A45" s="92" t="str">
-        <x:v>21. Stop Claude after two consecutive no-progress auto-compactions; checkpoint and use one fresh narrow retry rather than resuming the thrashing session.</x:v>
+        <x:v>21. House exclusivity has two scopes. Astra at any effort reserves Codex globally and Fable 5.1 at any effort reserves Claude globally. Sol high or higher reserves Codex only for assignments under the same delivery manager; Opus high or higher reserves Claude only for assignments under the same delivery manager.</x:v>
       </x:c>
       <x:c r="B45" s="69"/>
       <x:c r="C45" s="69"/>
@@ -2621,7 +2741,7 @@
     </x:row>
     <x:row r="46" ht="42" customHeight="1">
       <x:c r="A46" s="92" t="str">
-        <x:v>22. Owner concurrency exceptions are finite and journalled after an occupancy probe; leads and managers cannot self-authorize them.</x:v>
+        <x:v>22. New-product brainstorming may use Fable 5.1 medium or Astra medium. Both create global house reservations while active; prefer another eligible house or queue competing work.</x:v>
       </x:c>
       <x:c r="B46" s="69"/>
       <x:c r="C46" s="69"/>
@@ -2629,7 +2749,7 @@
     </x:row>
     <x:row r="47" ht="42" customHeight="1">
       <x:c r="A47" s="92" t="str">
-        <x:v>23. DeepSeek V4.1 Flash uses the provider code opencode-go/deepseek-v4.1-flash. The human-readable name and provider code identify the same approved model. The provider renamed this code from opencode-go/deepseek-flash, which no longer appears in `opencode models`; the version now lives in the code itself.</x:v>
+        <x:v>23. Fable model authorization does not permit paid usage credits or extra spending. Verify included allowance before any headless request.</x:v>
       </x:c>
       <x:c r="B47" s="69"/>
       <x:c r="C47" s="69"/>
@@ -2637,7 +2757,7 @@
     </x:row>
     <x:row r="48" ht="42" customHeight="1">
       <x:c r="A48" s="92" t="str">
-        <x:v>24. DeepSeek high is the default for bounded implementation. DeepSeek max mechanically implements novel public contract, identity, schema or serialization shapes only after an approved brain settles the shape and objective contract tests.</x:v>
+        <x:v>24. The delivery manager keeps its turn active with a real bounded wait while workers run. It may finish only after terminal handbacks or explicit transfer to another live supervisor.</x:v>
       </x:c>
       <x:c r="B48" s="69"/>
       <x:c r="C48" s="69"/>
@@ -2645,11 +2765,59 @@
     </x:row>
     <x:row r="49" ht="42" customHeight="1">
       <x:c r="A49" s="92" t="str">
-        <x:v>25. DeepSeek V4 Pro, DeepSeek V4 Flash and the vision-exp variants are excluded: opencode-go/deepseek-v4-pro, opencode-go/deepseek-v4-flash and opencode-go/deepseek-v4-flash-vision-exp are DIFFERENT models, not fallbacks for V4.1 Flash. If opencode-go/deepseek-v4.1-flash is unavailable, stop and reroute to a different approved house; never substitute another DeepSeek model.</x:v>
+        <x:v>25. External provider streams are drained outside manager context. Retrieve compact lifecycle changes and the mechanically extracted final assistant result, not accumulated raw output.</x:v>
       </x:c>
       <x:c r="B49" s="69"/>
       <x:c r="C49" s="69"/>
       <x:c r="D49" s="69"/>
+    </x:row>
+    <x:row r="50" ht="42" customHeight="1">
+      <x:c r="A50" s="92" t="str">
+        <x:v>26. A provider parent exit does not transfer writer ownership. Verify process tree, worktree command/CWD holders and provider background-agent registry before any replacement writer.</x:v>
+      </x:c>
+      <x:c r="B50" s="69"/>
+      <x:c r="C50" s="69"/>
+      <x:c r="D50" s="69"/>
+    </x:row>
+    <x:row r="51" ht="42" customHeight="1">
+      <x:c r="A51" s="92" t="str">
+        <x:v>27. Stop Claude after two consecutive no-progress auto-compactions; checkpoint and use one fresh narrow retry rather than resuming the thrashing session.</x:v>
+      </x:c>
+      <x:c r="B51" s="69"/>
+      <x:c r="C51" s="69"/>
+      <x:c r="D51" s="69"/>
+    </x:row>
+    <x:row r="52" ht="42" customHeight="1">
+      <x:c r="A52" s="92" t="str">
+        <x:v>28. Owner concurrency exceptions are finite and journalled after an occupancy probe; leads and managers cannot self-authorize them.</x:v>
+      </x:c>
+      <x:c r="B52" s="69"/>
+      <x:c r="C52" s="69"/>
+      <x:c r="D52" s="69"/>
+    </x:row>
+    <x:row r="53" ht="42" customHeight="1">
+      <x:c r="A53" s="92" t="str">
+        <x:v>29. DeepSeek V4.1 Flash uses the provider code opencode-go/deepseek-v4.1-flash. The human-readable name and provider code identify the same approved model. The provider renamed this code from opencode-go/deepseek-flash, which no longer appears in `opencode models`; the version now lives in the code itself.</x:v>
+      </x:c>
+      <x:c r="B53" s="69"/>
+      <x:c r="C53" s="69"/>
+      <x:c r="D53" s="69"/>
+    </x:row>
+    <x:row r="54" ht="42" customHeight="1">
+      <x:c r="A54" s="92" t="str">
+        <x:v>30. DeepSeek high is the default for bounded implementation. DeepSeek max mechanically implements novel public contract, identity, schema or serialization shapes only after an approved brain settles the shape and objective contract tests.</x:v>
+      </x:c>
+      <x:c r="B54" s="69"/>
+      <x:c r="C54" s="69"/>
+      <x:c r="D54" s="69"/>
+    </x:row>
+    <x:row r="55" ht="42" customHeight="1">
+      <x:c r="A55" s="92" t="str">
+        <x:v>31. DeepSeek V4 Pro, DeepSeek V4 Flash and the vision-exp variants are excluded: opencode-go/deepseek-v4-pro, opencode-go/deepseek-v4-flash and opencode-go/deepseek-v4-flash-vision-exp are DIFFERENT models, not fallbacks for V4.1 Flash. If opencode-go/deepseek-v4.1-flash is unavailable, stop and reroute to a different approved house; never substitute another DeepSeek model.</x:v>
+      </x:c>
+      <x:c r="B55" s="69"/>
+      <x:c r="C55" s="69"/>
+      <x:c r="D55" s="69"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2679,6 +2847,12 @@
     <x:mergeCell ref="A47:D47"/>
     <x:mergeCell ref="A48:D48"/>
     <x:mergeCell ref="A49:D49"/>
+    <x:mergeCell ref="A50:D50"/>
+    <x:mergeCell ref="A51:D51"/>
+    <x:mergeCell ref="A52:D52"/>
+    <x:mergeCell ref="A53:D53"/>
+    <x:mergeCell ref="A54:D54"/>
+    <x:mergeCell ref="A55:D55"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2710,7 +2884,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>Policy source: Interchange policy v0.6.0</x:v>
+        <x:v>Policy source: Interchange policy v0.7.0</x:v>
       </x:c>
       <x:c r="B3" s="2" t="str">
         <x:v>Approved on</x:v>
@@ -2837,56 +3011,111 @@
     </x:row>
     <x:row r="16" ht="50" customHeight="1">
       <x:c r="A16" s="24" t="str">
-        <x:v>Usage</x:v>
+        <x:v>Owner zero-Codex override</x:v>
       </x:c>
       <x:c r="B16" s="24" t="str">
-        <x:v>Parse available CLI usage mechanically; unknown when absent</x:v>
+        <x:v>Explicit do-not-use-Codex-for-delegation-or-leading instruction</x:v>
       </x:c>
       <x:c r="C16" s="24" t="str">
-        <x:v>Store input/output/cache/reasoning separately; do not assume provider counters are additive</x:v>
+        <x:v>Set Codex mechanical worker and mechanical lead allowance to zero; retain only explicitly requested brain/review use</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="50" customHeight="1">
       <x:c r="A17" s="24" t="str">
-        <x:v>Supervision ownership</x:v>
+        <x:v>Codex capacity preflight</x:v>
       </x:c>
       <x:c r="B17" s="24" t="str">
-        <x:v>Manager turn remains active until terminal handback or explicit live-supervisor transfer</x:v>
+        <x:v>Fresh usage snapshot when available + declared brain/review reserve + explicit mechanical allowance</x:v>
       </x:c>
       <x:c r="C17" s="24" t="str">
-        <x:v>A wait timeout, session ID or future promise is not a continuation mechanism</x:v>
+        <x:v>No recorded allowance means zero new Codex mechanical workers; external houses are the default execution lane</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="50" customHeight="1">
       <x:c r="A18" s="24" t="str">
-        <x:v>Output isolation</x:v>
+        <x:v>Codex mechanical concurrency</x:v>
       </x:c>
       <x:c r="B18" s="24" t="str">
-        <x:v>Adapter drains provider streams outside manager context</x:v>
+        <x:v>At most 1 active by default</x:v>
       </x:c>
       <x:c r="C18" s="24" t="str">
-        <x:v>Manager receives lifecycle changes, final assistant result, usage, warnings and exit state only</x:v>
+        <x:v>Parallel Codex mechanical workers require explicit owner authorization; prefer external-house parallelism</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="50" customHeight="1">
       <x:c r="A19" s="24" t="str">
-        <x:v>Attempt ceilings</x:v>
+        <x:v>Codex early burn checkpoint</x:v>
       </x:c>
       <x:c r="B19" s="24" t="str">
-        <x:v>Finite wall-time and turn ceilings; token/cost ceilings where timely counters exist</x:v>
+        <x:v>Recheck after first mechanical checkpoint when usage is observable</x:v>
       </x:c>
       <x:c r="C19" s="24" t="str">
-        <x:v>Stop deterministic blockers; do not spend a ceiling rediscovering known failures</x:v>
+        <x:v>Freeze new Codex mechanical dispatch when burn exceeds allowance or threatens reserved brain/review capacity</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="50" customHeight="1">
       <x:c r="A20" s="24" t="str">
+        <x:v>Codex review batching</x:v>
+      </x:c>
+      <x:c r="B20" s="24" t="str">
+        <x:v>One semantic/risk reviewer per meaningful integrated chunk</x:v>
+      </x:c>
+      <x:c r="C20" s="24" t="str">
+        <x:v>Mechanical gates run outside Codex; remedy commits invalidate prior review and require exact-head re-review</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="50" customHeight="1">
+      <x:c r="A21" s="24" t="str">
+        <x:v>Usage</x:v>
+      </x:c>
+      <x:c r="B21" s="24" t="str">
+        <x:v>Parse available CLI usage mechanically; unknown when absent</x:v>
+      </x:c>
+      <x:c r="C21" s="24" t="str">
+        <x:v>Store input/output/cache/reasoning separately; do not assume provider counters are additive</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="50" customHeight="1">
+      <x:c r="A22" s="24" t="str">
+        <x:v>Supervision ownership</x:v>
+      </x:c>
+      <x:c r="B22" s="24" t="str">
+        <x:v>Manager turn remains active until terminal handback or explicit live-supervisor transfer</x:v>
+      </x:c>
+      <x:c r="C22" s="24" t="str">
+        <x:v>A wait timeout, session ID or future promise is not a continuation mechanism</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="50" customHeight="1">
+      <x:c r="A23" s="24" t="str">
+        <x:v>Output isolation</x:v>
+      </x:c>
+      <x:c r="B23" s="24" t="str">
+        <x:v>Adapter drains provider streams outside manager context</x:v>
+      </x:c>
+      <x:c r="C23" s="24" t="str">
+        <x:v>Manager receives lifecycle changes, final assistant result, usage, warnings and exit state only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="50" customHeight="1">
+      <x:c r="A24" s="24" t="str">
+        <x:v>Attempt ceilings</x:v>
+      </x:c>
+      <x:c r="B24" s="24" t="str">
+        <x:v>Finite wall-time and turn ceilings; token/cost ceilings where timely counters exist</x:v>
+      </x:c>
+      <x:c r="C24" s="24" t="str">
+        <x:v>Stop deterministic blockers; do not spend a ceiling rediscovering known failures</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="50" customHeight="1">
+      <x:c r="A25" s="24" t="str">
         <x:v>Claude compaction</x:v>
       </x:c>
-      <x:c r="B20" s="24" t="str">
+      <x:c r="B25" s="24" t="str">
         <x:v>Stop after 2 consecutive auto-compactions without artifact, evidence or gate progress</x:v>
       </x:c>
-      <x:c r="C20" s="24" t="str">
+      <x:c r="C25" s="24" t="str">
         <x:v>Classify autocompact_thrashing as context/transport failure; retry fresh and narrow, never resume that context</x:v>
       </x:c>
     </x:row>
@@ -2921,7 +3150,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>Policy source: Interchange policy v0.6.0</x:v>
+        <x:v>Policy source: Interchange policy v0.7.0</x:v>
       </x:c>
       <x:c r="B3" s="2" t="str">
         <x:v>Approved on</x:v>
@@ -3084,20 +3313,20 @@
       <x:c r="C22"/>
     </x:row>
     <x:row r="23" ht="26" customHeight="1">
-      <x:c r="A23" s="240" t="str">
+      <x:c r="A23" s="276" t="str">
         <x:v>Recovery playbook</x:v>
       </x:c>
-      <x:c r="B23" s="241"/>
-      <x:c r="C23" s="242"/>
+      <x:c r="B23" s="277"/>
+      <x:c r="C23" s="278"/>
     </x:row>
     <x:row r="24" ht="44" customHeight="1">
-      <x:c r="A24" s="248" t="str">
+      <x:c r="A24" s="284" t="str">
         <x:v>Failure</x:v>
       </x:c>
-      <x:c r="B24" s="249" t="str">
+      <x:c r="B24" s="285" t="str">
         <x:v>First action</x:v>
       </x:c>
-      <x:c r="C24" s="250" t="str">
+      <x:c r="C24" s="286" t="str">
         <x:v>Escalation</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
feat(interchange): gate Astra and Fable use
</commit_message>
<xml_diff>
--- a/outputs/interchange-design/interchange.xlsx
+++ b/outputs/interchange-design/interchange.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profiles" sheetId="1" r:id="Rd9241db062e94bfd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Routing" sheetId="2" r:id="Rae13d59e66494d0b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monitoring" sheetId="3" r:id="R2bda169c4e1245d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Recovery" sheetId="4" r:id="R3477effca99e4dce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profiles" sheetId="1" r:id="R801cbea57ead49c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Routing" sheetId="2" r:id="Rbe456525160944ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monitoring" sheetId="3" r:id="Rd03ae35d614a4084"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Recovery" sheetId="4" r:id="R78027977ff274756"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -55,7 +55,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="59">
+  <x:fills count="67">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -85,6 +85,46 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFCE4D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -420,7 +460,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="287">
+  <x:cellXfs count="323">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1110,6 +1150,86 @@
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="58" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="59" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="59" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="60" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="60" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="59" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="61" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="61" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="61" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="61" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="61" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="62" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="62" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="62" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="62" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="62" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="62" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="62" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="62" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="63" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="63" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="64" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="64" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="63" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="65" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="65" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="65" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="65" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="65" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="66" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="66" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="66" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="66" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="66" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="66" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="66" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="66" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1354,7 +1474,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>Policy source: Interchange policy v0.7.0</x:v>
+        <x:v>Policy source: Interchange policy v0.8.0</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -1577,10 +1697,10 @@
       <x:c r="F16" s="34" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G16" s="269" t="str">
+      <x:c r="G16" s="305" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H16" s="271" t="str">
+      <x:c r="H16" s="307" t="str">
         <x:v>Profile documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I16" s="22" t="str">
@@ -1606,10 +1726,10 @@
       <x:c r="F17" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G17" s="270" t="str">
+      <x:c r="G17" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H17" s="272" t="str">
+      <x:c r="H17" s="308" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I17" s="24" t="str">
@@ -1635,10 +1755,10 @@
       <x:c r="F18" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G18" s="270" t="str">
+      <x:c r="G18" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H18" s="272" t="str">
+      <x:c r="H18" s="308" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I18" s="24" t="str">
@@ -1664,10 +1784,10 @@
       <x:c r="F19" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G19" s="270" t="str">
+      <x:c r="G19" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H19" s="272" t="str">
+      <x:c r="H19" s="308" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I19" s="24" t="str">
@@ -1693,10 +1813,10 @@
       <x:c r="F20" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G20" s="270" t="str">
+      <x:c r="G20" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H20" s="272" t="str">
+      <x:c r="H20" s="308" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I20" s="24" t="str">
@@ -1722,10 +1842,10 @@
       <x:c r="F21" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G21" s="270" t="str">
+      <x:c r="G21" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H21" s="272" t="str">
+      <x:c r="H21" s="308" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I21" s="24" t="str">
@@ -1751,10 +1871,10 @@
       <x:c r="F22" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G22" s="270" t="str">
+      <x:c r="G22" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H22" s="272" t="str">
+      <x:c r="H22" s="308" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I22" s="24" t="str">
@@ -1780,10 +1900,10 @@
       <x:c r="F23" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G23" s="270" t="str">
+      <x:c r="G23" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H23" s="272" t="str">
+      <x:c r="H23" s="308" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I23" s="24" t="str">
@@ -1809,10 +1929,10 @@
       <x:c r="F24" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G24" s="270" t="str">
+      <x:c r="G24" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H24" s="272" t="str">
+      <x:c r="H24" s="308" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I24" s="24" t="str">
@@ -1838,10 +1958,10 @@
       <x:c r="F25" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G25" s="270" t="str">
+      <x:c r="G25" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H25" s="272" t="str">
+      <x:c r="H25" s="308" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I25" s="24" t="str">
@@ -1867,10 +1987,10 @@
       <x:c r="F26" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G26" s="270" t="str">
+      <x:c r="G26" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H26" s="272" t="str">
+      <x:c r="H26" s="308" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I26" s="24" t="str">
@@ -1896,10 +2016,10 @@
       <x:c r="F27" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G27" s="270" t="str">
+      <x:c r="G27" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H27" s="272" t="str">
+      <x:c r="H27" s="308" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I27" s="24" t="str">
@@ -1925,10 +2045,10 @@
       <x:c r="F28" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G28" s="270" t="str">
+      <x:c r="G28" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H28" s="272" t="str">
+      <x:c r="H28" s="308" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I28" s="24" t="str">
@@ -1954,10 +2074,10 @@
       <x:c r="F29" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G29" s="270" t="str">
+      <x:c r="G29" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H29" s="273" t="str">
+      <x:c r="H29" s="309" t="str">
         <x:v>Smoke-tested</x:v>
       </x:c>
       <x:c r="I29" s="24" t="str">
@@ -1983,10 +2103,10 @@
       <x:c r="F30" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G30" s="270" t="str">
+      <x:c r="G30" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H30" s="272" t="str">
+      <x:c r="H30" s="308" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I30" s="24" t="str">
@@ -2012,10 +2132,10 @@
       <x:c r="F31" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G31" s="270" t="str">
+      <x:c r="G31" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H31" s="272" t="str">
+      <x:c r="H31" s="308" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I31" s="24" t="str">
@@ -2041,10 +2161,10 @@
       <x:c r="F32" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G32" s="270" t="str">
+      <x:c r="G32" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H32" s="272" t="str">
+      <x:c r="H32" s="308" t="str">
         <x:v>CLI model and effort documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I32" s="24" t="str">
@@ -2070,10 +2190,10 @@
       <x:c r="F33" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G33" s="270" t="str">
+      <x:c r="G33" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H33" s="272" t="str">
+      <x:c r="H33" s="308" t="str">
         <x:v>CLI model and effort documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I33" s="24" t="str">
@@ -2099,10 +2219,10 @@
       <x:c r="F34" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G34" s="270" t="str">
+      <x:c r="G34" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H34" s="272" t="str">
+      <x:c r="H34" s="308" t="str">
         <x:v>Profile documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I34" s="24" t="str">
@@ -2128,10 +2248,10 @@
       <x:c r="F35" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G35" s="270" t="str">
+      <x:c r="G35" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H35" s="272" t="str">
+      <x:c r="H35" s="308" t="str">
         <x:v>Profile documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I35" s="24" t="str">
@@ -2157,10 +2277,10 @@
       <x:c r="F36" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G36" s="270" t="str">
+      <x:c r="G36" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H36" s="272" t="str">
+      <x:c r="H36" s="308" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I36" s="24" t="str">
@@ -2186,10 +2306,10 @@
       <x:c r="F37" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G37" s="270" t="str">
+      <x:c r="G37" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H37" s="272" t="str">
+      <x:c r="H37" s="308" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I37" s="24" t="str">
@@ -2215,10 +2335,10 @@
       <x:c r="F38" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G38" s="270" t="str">
+      <x:c r="G38" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H38" s="272" t="str">
+      <x:c r="H38" s="308" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I38" s="24" t="str">
@@ -2244,10 +2364,10 @@
       <x:c r="F39" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G39" s="270" t="str">
+      <x:c r="G39" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H39" s="272" t="str">
+      <x:c r="H39" s="308" t="str">
         <x:v>Profile documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I39" s="24" t="str">
@@ -2273,10 +2393,10 @@
       <x:c r="F40" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G40" s="270" t="str">
+      <x:c r="G40" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H40" s="272" t="str">
+      <x:c r="H40" s="308" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I40" s="24" t="str">
@@ -2317,7 +2437,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>Policy source: Interchange policy v0.7.0</x:v>
+        <x:v>Policy source: Interchange policy v0.8.0</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2" t="str">
@@ -2366,10 +2486,10 @@
         <x:v>New product idea and brainstorming</x:v>
       </x:c>
       <x:c r="B8" s="22" t="str">
-        <x:v>brainstorm-fable-medium; brainstorm-astra-medium</x:v>
+        <x:v>lead-sol-high or dm-sol-high</x:v>
       </x:c>
       <x:c r="C8" s="22" t="str">
-        <x:v>Eligible alternative respecting house exclusivity and no-extra-spend policy</x:v>
+        <x:v>brainstorm-fable-medium or brainstorm-astra-medium only after fresh owner authorization for that invocation and a concrete reason Sol high cannot fit; Fable also requires included-plan/no-extra-spend proof</x:v>
       </x:c>
       <x:c r="D8" s="22" t="str">
         <x:v>Explore users, problem, options, assumptions and validation; does not authorize implementation</x:v>
@@ -2383,7 +2503,7 @@
         <x:v>lead-sol-high or dm-sol-high</x:v>
       </x:c>
       <x:c r="C9" s="24" t="str">
-        <x:v>lead-astra-medium or dm-astra-medium for unusually large cross-workstream ambiguity</x:v>
+        <x:v>lead-astra-medium or dm-astra-medium for unusually large cross-workstream ambiguity; every Astra invocation requires fresh owner authorization and a concrete reason Sol high cannot fit</x:v>
       </x:c>
       <x:c r="D9" s="24" t="str">
         <x:v>Only approved brain profiles interpret missing requirements, choose tradeoffs or settle contracts</x:v>
@@ -2453,7 +2573,7 @@
         <x:v>lead-sol-high resolves judgment; worker-opus-high or another qualified external profile executes settled packets</x:v>
       </x:c>
       <x:c r="C14" s="24" t="str">
-        <x:v>lead-astra-medium resolves unusually large ambiguity; Codex mechanical worker requires a recorded allowance</x:v>
+        <x:v>lead-astra-medium resolves unusually large ambiguity; Codex mechanical worker requires a recorded allowance; every Astra invocation requires fresh owner authorization and a concrete reason Sol high cannot fit</x:v>
       </x:c>
       <x:c r="D14" s="24" t="str">
         <x:v>Separate consequential decisions from implementation; independent review remains mandatory</x:v>
@@ -2481,7 +2601,7 @@
         <x:v>lead-sol-high settles shape; worker-deepseek-flash-max implements the exact contract</x:v>
       </x:c>
       <x:c r="C16" s="24" t="str">
-        <x:v>lead-astra-medium settles unusually large cross-workstream contract ambiguity before execution</x:v>
+        <x:v>lead-astra-medium settles unusually large cross-workstream contract ambiguity before execution; every Astra invocation requires fresh owner authorization and a concrete reason Sol high cannot fit</x:v>
       </x:c>
       <x:c r="D16" s="24" t="str">
         <x:v>DeepSeek max receives a decided shape and objective contract tests; it does not choose the public contract</x:v>
@@ -2509,7 +2629,7 @@
         <x:v>lead-sol-high</x:v>
       </x:c>
       <x:c r="C18" s="24" t="str">
-        <x:v>lead-astra-medium for unusually large cross-workstream ambiguity</x:v>
+        <x:v>lead-astra-medium for unusually large cross-workstream ambiguity; every Astra invocation requires fresh owner authorization and a concrete reason Sol high cannot fit</x:v>
       </x:c>
       <x:c r="D18" s="24" t="str">
         <x:v>Approved brain resolves product, architecture, consequence and coupling before execution</x:v>
@@ -2523,7 +2643,7 @@
         <x:v>dm-sol-high</x:v>
       </x:c>
       <x:c r="C19" s="24" t="str">
-        <x:v>dm-astra-medium for unusually large ambiguity; dm-opus-high may coordinate but routes judgment to a brain</x:v>
+        <x:v>dm-astra-medium for unusually large ambiguity; dm-opus-high may coordinate but routes judgment to a brain; every Astra invocation requires fresh owner authorization and a concrete reason Sol high cannot fit</x:v>
       </x:c>
       <x:c r="D19" s="24" t="str">
         <x:v>Manager receives compact exceptions and evidence; only an assigned brain resolves interpretation</x:v>
@@ -2537,7 +2657,7 @@
         <x:v>reviewer-sol-high</x:v>
       </x:c>
       <x:c r="C20" s="24" t="str">
-        <x:v>reviewer-astra-medium for unusually large cross-workstream scope</x:v>
+        <x:v>reviewer-astra-medium for unusually large cross-workstream scope; every Astra invocation requires fresh owner authorization and a concrete reason Sol high cannot fit</x:v>
       </x:c>
       <x:c r="D20" s="24" t="str">
         <x:v>Run gates mechanically; batch one independent brain review at a meaningful integrated chunk boundary and bind it to the exact head</x:v>
@@ -2556,20 +2676,20 @@
       <x:c r="D22"/>
     </x:row>
     <x:row r="23" ht="42" customHeight="1">
-      <x:c r="A23" s="276" t="str">
+      <x:c r="A23" s="312" t="str">
         <x:v>Selection rules</x:v>
       </x:c>
-      <x:c r="B23" s="277"/>
-      <x:c r="C23" s="277"/>
-      <x:c r="D23" s="278"/>
+      <x:c r="B23" s="313"/>
+      <x:c r="C23" s="313"/>
+      <x:c r="D23" s="314"/>
     </x:row>
     <x:row r="24" ht="42" customHeight="1">
-      <x:c r="A24" s="284" t="str">
+      <x:c r="A24" s="320" t="str">
         <x:v>Approved selection rule</x:v>
       </x:c>
-      <x:c r="B24" s="285"/>
-      <x:c r="C24" s="285"/>
-      <x:c r="D24" s="286"/>
+      <x:c r="B24" s="321"/>
+      <x:c r="C24" s="321"/>
+      <x:c r="D24" s="322"/>
     </x:row>
     <x:row r="25" ht="42" customHeight="1">
       <x:c r="A25" s="91" t="str">
@@ -2605,7 +2725,7 @@
     </x:row>
     <x:row r="29" ht="42" customHeight="1">
       <x:c r="A29" s="92" t="str">
-        <x:v>5. Semantic and risk acceptance is a brain task: use an independent Sol high reviewer, or Astra medium for unusually large cross-workstream scope. Mechanical workers may collect gates but cannot issue acceptance judgment.</x:v>
+        <x:v>5. Semantic and risk acceptance is a brain task: use an independent Sol high reviewer by default. Astra medium is eligible only for unusually large cross-workstream scope after fresh invocation-specific owner authorization and a concrete reason Sol high cannot fit. Mechanical workers may collect gates but cannot issue acceptance judgment.</x:v>
       </x:c>
       <x:c r="B29" s="69"/>
       <x:c r="C29" s="69"/>
@@ -2741,7 +2861,7 @@
     </x:row>
     <x:row r="46" ht="42" customHeight="1">
       <x:c r="A46" s="92" t="str">
-        <x:v>22. New-product brainstorming may use Fable 5.1 medium or Astra medium. Both create global house reservations while active; prefer another eligible house or queue competing work.</x:v>
+        <x:v>22. New-product brainstorming uses Sol high by default. Fable 5.1 medium or Astra medium requires fresh invocation-specific owner authorization and a concrete reason Sol high cannot fit; Fable separately requires included-plan/no-extra-spend proof. Both create global house reservations while active.</x:v>
       </x:c>
       <x:c r="B46" s="69"/>
       <x:c r="C46" s="69"/>
@@ -2818,6 +2938,14 @@
       <x:c r="B55" s="69"/>
       <x:c r="C55" s="69"/>
       <x:c r="D55" s="69"/>
+    </x:row>
+    <x:row r="56" ht="42" customHeight="1">
+      <x:c r="A56" s="92" t="str">
+        <x:v>32. Every Astra or Fable invocation in any role requires fresh explicit owner authorization bound to that start, resume, retry or follow-up, plus a concrete reason gpt-5.6-sol high cannot fit. Prior authorization is never reusable; Fable also requires included-plan/no-extra-spend proof.</x:v>
+      </x:c>
+      <x:c r="B56" s="69"/>
+      <x:c r="C56" s="69"/>
+      <x:c r="D56" s="69"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2853,6 +2981,7 @@
     <x:mergeCell ref="A53:D53"/>
     <x:mergeCell ref="A54:D54"/>
     <x:mergeCell ref="A55:D55"/>
+    <x:mergeCell ref="A56:D56"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2884,7 +3013,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>Policy source: Interchange policy v0.7.0</x:v>
+        <x:v>Policy source: Interchange policy v0.8.0</x:v>
       </x:c>
       <x:c r="B3" s="2" t="str">
         <x:v>Approved on</x:v>
@@ -3117,6 +3246,39 @@
       </x:c>
       <x:c r="C25" s="24" t="str">
         <x:v>Classify autocompact_thrashing as context/transport failure; retry fresh and narrow, never resume that context</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="50" customHeight="1">
+      <x:c r="A26" s="24" t="str">
+        <x:v>Astra/Fable invocation authorization</x:v>
+      </x:c>
+      <x:c r="B26" s="24" t="str">
+        <x:v>Fresh explicit owner authorization for every start, resume, retry and follow-up</x:v>
+      </x:c>
+      <x:c r="C26" s="24" t="str">
+        <x:v>Bind approval to packet, attempt and invocation ID plus model/effort/role; manager or lead cannot self-authorize</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="50" customHeight="1">
+      <x:c r="A27" s="24" t="str">
+        <x:v>Sol-high non-fit reason</x:v>
+      </x:c>
+      <x:c r="B27" s="24" t="str">
+        <x:v>Concrete recorded reason gpt-5.6-sol high cannot fit</x:v>
+      </x:c>
+      <x:c r="C27" s="24" t="str">
+        <x:v>Vague preference or prior approval fails closed; use Sol high if it fits or wait for owner</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="50" customHeight="1">
+      <x:c r="A28" s="24" t="str">
+        <x:v>Astra/Fable authorization reuse</x:v>
+      </x:c>
+      <x:c r="B28" s="24" t="str">
+        <x:v>Forbidden</x:v>
+      </x:c>
+      <x:c r="C28" s="24" t="str">
+        <x:v>A completed, failed or suspended invocation consumes its authorization; the next invocation needs a new owner decision</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3150,7 +3312,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>Policy source: Interchange policy v0.7.0</x:v>
+        <x:v>Policy source: Interchange policy v0.8.0</x:v>
       </x:c>
       <x:c r="B3" s="2" t="str">
         <x:v>Approved on</x:v>
@@ -3313,20 +3475,20 @@
       <x:c r="C22"/>
     </x:row>
     <x:row r="23" ht="26" customHeight="1">
-      <x:c r="A23" s="276" t="str">
+      <x:c r="A23" s="312" t="str">
         <x:v>Recovery playbook</x:v>
       </x:c>
-      <x:c r="B23" s="277"/>
-      <x:c r="C23" s="278"/>
+      <x:c r="B23" s="313"/>
+      <x:c r="C23" s="314"/>
     </x:row>
     <x:row r="24" ht="44" customHeight="1">
-      <x:c r="A24" s="284" t="str">
+      <x:c r="A24" s="320" t="str">
         <x:v>Failure</x:v>
       </x:c>
-      <x:c r="B24" s="285" t="str">
+      <x:c r="B24" s="321" t="str">
         <x:v>First action</x:v>
       </x:c>
-      <x:c r="C24" s="286" t="str">
+      <x:c r="C24" s="322" t="str">
         <x:v>Escalation</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Conserve Codex capacity and gate exceptional brains (#5)
* feat(interchange): conserve Codex capacity

* feat(interchange): gate Astra and Fable use
</commit_message>
<xml_diff>
--- a/outputs/interchange-design/interchange.xlsx
+++ b/outputs/interchange-design/interchange.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profiles" sheetId="1" r:id="R54bb1c1b109c4a81"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Routing" sheetId="2" r:id="Ra5fa34cf7b594df6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monitoring" sheetId="3" r:id="R9861e40f1bfe4770"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Recovery" sheetId="4" r:id="Re075d54395954ed3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profiles" sheetId="1" r:id="R801cbea57ead49c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Routing" sheetId="2" r:id="Rbe456525160944ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monitoring" sheetId="3" r:id="Rd03ae35d614a4084"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Recovery" sheetId="4" r:id="R78027977ff274756"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -55,7 +55,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="51">
+  <x:fills count="67">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -85,6 +85,86 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFCE4D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -380,7 +460,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="251">
+  <x:cellXfs count="323">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -990,6 +1070,166 @@
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="50" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="51" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="51" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="52" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="52" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="51" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="53" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="53" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="53" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="53" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="53" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="54" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="54" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="54" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="54" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="54" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="54" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="54" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="54" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="55" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="55" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="56" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="56" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="55" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="57" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="57" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="57" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="57" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="57" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="58" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="58" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="58" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="58" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="58" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="58" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="58" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="58" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="59" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="59" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="60" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="60" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="59" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="61" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="61" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="61" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="61" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="61" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="62" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="62" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="62" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="62" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="62" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="62" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="62" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="62" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="63" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="63" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="64" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="64" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="63" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="65" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="65" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="65" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="65" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="65" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="66" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="66" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="66" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="66" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="66" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="66" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="66" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="66" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1234,7 +1474,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>Policy source: Interchange policy v0.6.0</x:v>
+        <x:v>Policy source: Interchange policy v0.8.0</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -1457,10 +1697,10 @@
       <x:c r="F16" s="34" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G16" s="233" t="str">
+      <x:c r="G16" s="305" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H16" s="235" t="str">
+      <x:c r="H16" s="307" t="str">
         <x:v>Profile documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I16" s="22" t="str">
@@ -1486,10 +1726,10 @@
       <x:c r="F17" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G17" s="234" t="str">
+      <x:c r="G17" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H17" s="236" t="str">
+      <x:c r="H17" s="308" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I17" s="24" t="str">
@@ -1515,10 +1755,10 @@
       <x:c r="F18" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G18" s="234" t="str">
+      <x:c r="G18" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H18" s="236" t="str">
+      <x:c r="H18" s="308" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I18" s="24" t="str">
@@ -1544,10 +1784,10 @@
       <x:c r="F19" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G19" s="234" t="str">
+      <x:c r="G19" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H19" s="236" t="str">
+      <x:c r="H19" s="308" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I19" s="24" t="str">
@@ -1573,10 +1813,10 @@
       <x:c r="F20" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G20" s="234" t="str">
+      <x:c r="G20" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H20" s="236" t="str">
+      <x:c r="H20" s="308" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I20" s="24" t="str">
@@ -1602,10 +1842,10 @@
       <x:c r="F21" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G21" s="234" t="str">
+      <x:c r="G21" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H21" s="236" t="str">
+      <x:c r="H21" s="308" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I21" s="24" t="str">
@@ -1631,10 +1871,10 @@
       <x:c r="F22" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G22" s="234" t="str">
+      <x:c r="G22" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H22" s="236" t="str">
+      <x:c r="H22" s="308" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I22" s="24" t="str">
@@ -1660,10 +1900,10 @@
       <x:c r="F23" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G23" s="234" t="str">
+      <x:c r="G23" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H23" s="236" t="str">
+      <x:c r="H23" s="308" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I23" s="24" t="str">
@@ -1689,10 +1929,10 @@
       <x:c r="F24" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G24" s="234" t="str">
+      <x:c r="G24" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H24" s="236" t="str">
+      <x:c r="H24" s="308" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I24" s="24" t="str">
@@ -1718,10 +1958,10 @@
       <x:c r="F25" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G25" s="234" t="str">
+      <x:c r="G25" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H25" s="236" t="str">
+      <x:c r="H25" s="308" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I25" s="24" t="str">
@@ -1747,10 +1987,10 @@
       <x:c r="F26" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G26" s="234" t="str">
+      <x:c r="G26" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H26" s="236" t="str">
+      <x:c r="H26" s="308" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I26" s="24" t="str">
@@ -1776,10 +2016,10 @@
       <x:c r="F27" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G27" s="234" t="str">
+      <x:c r="G27" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H27" s="236" t="str">
+      <x:c r="H27" s="308" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I27" s="24" t="str">
@@ -1805,10 +2045,10 @@
       <x:c r="F28" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G28" s="234" t="str">
+      <x:c r="G28" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H28" s="236" t="str">
+      <x:c r="H28" s="308" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I28" s="24" t="str">
@@ -1834,10 +2074,10 @@
       <x:c r="F29" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G29" s="234" t="str">
+      <x:c r="G29" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H29" s="237" t="str">
+      <x:c r="H29" s="309" t="str">
         <x:v>Smoke-tested</x:v>
       </x:c>
       <x:c r="I29" s="24" t="str">
@@ -1863,10 +2103,10 @@
       <x:c r="F30" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G30" s="234" t="str">
+      <x:c r="G30" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H30" s="236" t="str">
+      <x:c r="H30" s="308" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I30" s="24" t="str">
@@ -1892,10 +2132,10 @@
       <x:c r="F31" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G31" s="234" t="str">
+      <x:c r="G31" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H31" s="236" t="str">
+      <x:c r="H31" s="308" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I31" s="24" t="str">
@@ -1921,10 +2161,10 @@
       <x:c r="F32" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G32" s="234" t="str">
+      <x:c r="G32" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H32" s="236" t="str">
+      <x:c r="H32" s="308" t="str">
         <x:v>CLI model and effort documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I32" s="24" t="str">
@@ -1950,10 +2190,10 @@
       <x:c r="F33" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G33" s="234" t="str">
+      <x:c r="G33" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H33" s="236" t="str">
+      <x:c r="H33" s="308" t="str">
         <x:v>CLI model and effort documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I33" s="24" t="str">
@@ -1979,10 +2219,10 @@
       <x:c r="F34" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G34" s="234" t="str">
+      <x:c r="G34" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H34" s="236" t="str">
+      <x:c r="H34" s="308" t="str">
         <x:v>Profile documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I34" s="24" t="str">
@@ -2008,10 +2248,10 @@
       <x:c r="F35" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G35" s="234" t="str">
+      <x:c r="G35" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H35" s="236" t="str">
+      <x:c r="H35" s="308" t="str">
         <x:v>Profile documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I35" s="24" t="str">
@@ -2037,10 +2277,10 @@
       <x:c r="F36" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G36" s="234" t="str">
+      <x:c r="G36" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H36" s="236" t="str">
+      <x:c r="H36" s="308" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I36" s="24" t="str">
@@ -2066,10 +2306,10 @@
       <x:c r="F37" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G37" s="234" t="str">
+      <x:c r="G37" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H37" s="236" t="str">
+      <x:c r="H37" s="308" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I37" s="24" t="str">
@@ -2095,10 +2335,10 @@
       <x:c r="F38" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G38" s="234" t="str">
+      <x:c r="G38" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H38" s="236" t="str">
+      <x:c r="H38" s="308" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I38" s="24" t="str">
@@ -2124,10 +2364,10 @@
       <x:c r="F39" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G39" s="234" t="str">
+      <x:c r="G39" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H39" s="236" t="str">
+      <x:c r="H39" s="308" t="str">
         <x:v>Profile documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I39" s="24" t="str">
@@ -2153,10 +2393,10 @@
       <x:c r="F40" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G40" s="234" t="str">
+      <x:c r="G40" s="306" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H40" s="236" t="str">
+      <x:c r="H40" s="308" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I40" s="24" t="str">
@@ -2197,7 +2437,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>Policy source: Interchange policy v0.6.0</x:v>
+        <x:v>Policy source: Interchange policy v0.8.0</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2" t="str">
@@ -2246,10 +2486,10 @@
         <x:v>New product idea and brainstorming</x:v>
       </x:c>
       <x:c r="B8" s="22" t="str">
-        <x:v>brainstorm-fable-medium; brainstorm-astra-medium</x:v>
+        <x:v>lead-sol-high or dm-sol-high</x:v>
       </x:c>
       <x:c r="C8" s="22" t="str">
-        <x:v>Eligible alternative respecting house exclusivity and no-extra-spend policy</x:v>
+        <x:v>brainstorm-fable-medium or brainstorm-astra-medium only after fresh owner authorization for that invocation and a concrete reason Sol high cannot fit; Fable also requires included-plan/no-extra-spend proof</x:v>
       </x:c>
       <x:c r="D8" s="22" t="str">
         <x:v>Explore users, problem, options, assumptions and validation; does not authorize implementation</x:v>
@@ -2263,7 +2503,7 @@
         <x:v>lead-sol-high or dm-sol-high</x:v>
       </x:c>
       <x:c r="C9" s="24" t="str">
-        <x:v>lead-astra-medium or dm-astra-medium for unusually large cross-workstream ambiguity</x:v>
+        <x:v>lead-astra-medium or dm-astra-medium for unusually large cross-workstream ambiguity; every Astra invocation requires fresh owner authorization and a concrete reason Sol high cannot fit</x:v>
       </x:c>
       <x:c r="D9" s="24" t="str">
         <x:v>Only approved brain profiles interpret missing requirements, choose tradeoffs or settle contracts</x:v>
@@ -2274,10 +2514,10 @@
         <x:v>One direct lookup</x:v>
       </x:c>
       <x:c r="B10" s="24" t="str">
-        <x:v>Local search/tool when immediate; worker-muse-xhigh when parallel dispatch frees the brain or is faster overall</x:v>
+        <x:v>Local search/tool when immediate; worker-muse-xhigh when delegation frees the Codex brain or is faster overall</x:v>
       </x:c>
       <x:c r="C10" s="24" t="str">
-        <x:v>worker-luna-xhigh for bounded read-only evidence when Muse is unavailable</x:v>
+        <x:v>Another external read-only mechanical profile; Codex worker only under a recorded mechanical allowance</x:v>
       </x:c>
       <x:c r="D10" s="24" t="str">
         <x:v>Count startup, supervision and handback overhead; delegate when it improves accepted-result time or cost</x:v>
@@ -2291,7 +2531,7 @@
         <x:v>worker-muse-xhigh</x:v>
       </x:c>
       <x:c r="C11" s="24" t="str">
-        <x:v>worker-luna-xhigh; worker-luna-max when evidence density warrants</x:v>
+        <x:v>Another external bounded worker; Luna xhigh/max only under a recorded Codex mechanical allowance</x:v>
       </x:c>
       <x:c r="D11" s="24" t="str">
         <x:v>Repository search, localization, evidence collection, narrow checks and small explicit edits; no interpretation</x:v>
@@ -2305,7 +2545,7 @@
         <x:v>worker-deepseek-flash-high; worker-grok-high; worker-opus-medium; worker-terra-xhigh; worker-sol-medium</x:v>
       </x:c>
       <x:c r="C12" s="24" t="str">
-        <x:v>Another eligible profile from this pool</x:v>
+        <x:v>Codex worker from this pool only under a recorded mechanical allowance and after external fit/availability check</x:v>
       </x:c>
       <x:c r="D12" s="24" t="str">
         <x:v>Settled behavior, objective acceptance and bounded dependencies; ambiguity already resolved by a brain</x:v>
@@ -2319,7 +2559,7 @@
         <x:v>worker-deepseek-flash-high; worker-grok-xhigh; worker-opus-medium</x:v>
       </x:c>
       <x:c r="C13" s="24" t="str">
-        <x:v>lead-sol-high resolves ambiguity or consequence; then choose worker-sol-high, worker-opus-high or another qualified mechanical profile</x:v>
+        <x:v>lead-sol-high resolves ambiguity; choose an external mechanical worker first, or a Codex worker under a recorded allowance</x:v>
       </x:c>
       <x:c r="D13" s="24" t="str">
         <x:v>Difficult mechanical implementation within settled architecture; return tradeoffs instead of choosing</x:v>
@@ -2330,10 +2570,10 @@
         <x:v>High complexity development</x:v>
       </x:c>
       <x:c r="B14" s="24" t="str">
-        <x:v>lead-sol-high resolves judgment; worker-opus-high or another qualified mechanical profile executes settled packets</x:v>
+        <x:v>lead-sol-high resolves judgment; worker-opus-high or another qualified external profile executes settled packets</x:v>
       </x:c>
       <x:c r="C14" s="24" t="str">
-        <x:v>lead-astra-medium resolves unusually large cross-workstream ambiguity before mechanical execution</x:v>
+        <x:v>lead-astra-medium resolves unusually large ambiguity; Codex mechanical worker requires a recorded allowance; every Astra invocation requires fresh owner authorization and a concrete reason Sol high cannot fit</x:v>
       </x:c>
       <x:c r="D14" s="24" t="str">
         <x:v>Separate consequential decisions from implementation; independent review remains mandatory</x:v>
@@ -2344,10 +2584,10 @@
         <x:v>Demanding but well-defined implementation</x:v>
       </x:c>
       <x:c r="B15" s="24" t="str">
-        <x:v>worker-terra-max; worker-deepseek-flash-high</x:v>
+        <x:v>worker-deepseek-flash-high; worker-opus-high</x:v>
       </x:c>
       <x:c r="C15" s="24" t="str">
-        <x:v>High-complexity pool if evidence shows a reasoning blocker; never DeepSeek V4 Pro</x:v>
+        <x:v>worker-terra-max only under a recorded Codex mechanical allowance; never DeepSeek V4 Pro</x:v>
       </x:c>
       <x:c r="D15" s="24" t="str">
         <x:v>Dense mechanical implementation or integration with exact contracts and tests; never assign interpretation or use effort to outlast a loop</x:v>
@@ -2361,7 +2601,7 @@
         <x:v>lead-sol-high settles shape; worker-deepseek-flash-max implements the exact contract</x:v>
       </x:c>
       <x:c r="C16" s="24" t="str">
-        <x:v>lead-astra-medium settles unusually large cross-workstream contract ambiguity before execution</x:v>
+        <x:v>lead-astra-medium settles unusually large cross-workstream contract ambiguity before execution; every Astra invocation requires fresh owner authorization and a concrete reason Sol high cannot fit</x:v>
       </x:c>
       <x:c r="D16" s="24" t="str">
         <x:v>DeepSeek max receives a decided shape and objective contract tests; it does not choose the public contract</x:v>
@@ -2372,13 +2612,13 @@
         <x:v>Workstream with fixed contracts</x:v>
       </x:c>
       <x:c r="B17" s="24" t="str">
-        <x:v>lead-terra-xhigh</x:v>
+        <x:v>Current delivery manager coordinates settled packets across external mechanical workers</x:v>
       </x:c>
       <x:c r="C17" s="24" t="str">
-        <x:v>lead-terra-max or lead-sol-medium</x:v>
+        <x:v>lead-terra-xhigh/max only under a recorded Codex mechanical allowance</x:v>
       </x:c>
       <x:c r="D17" s="24" t="str">
-        <x:v>Mechanical lead authority may coordinate and delegate settled packets; ambiguity returns to lead-sol-high or lead-astra-medium</x:v>
+        <x:v>Preserve Codex brain capacity; a mechanical lead coordinates only settled work and returns ambiguity to Sol high or Astra medium</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="46" customHeight="1">
@@ -2389,7 +2629,7 @@
         <x:v>lead-sol-high</x:v>
       </x:c>
       <x:c r="C18" s="24" t="str">
-        <x:v>lead-astra-medium for unusually large cross-workstream ambiguity</x:v>
+        <x:v>lead-astra-medium for unusually large cross-workstream ambiguity; every Astra invocation requires fresh owner authorization and a concrete reason Sol high cannot fit</x:v>
       </x:c>
       <x:c r="D18" s="24" t="str">
         <x:v>Approved brain resolves product, architecture, consequence and coupling before execution</x:v>
@@ -2403,7 +2643,7 @@
         <x:v>dm-sol-high</x:v>
       </x:c>
       <x:c r="C19" s="24" t="str">
-        <x:v>dm-astra-medium for unusually large ambiguity; dm-opus-high may coordinate but routes judgment to a brain</x:v>
+        <x:v>dm-astra-medium for unusually large ambiguity; dm-opus-high may coordinate but routes judgment to a brain; every Astra invocation requires fresh owner authorization and a concrete reason Sol high cannot fit</x:v>
       </x:c>
       <x:c r="D19" s="24" t="str">
         <x:v>Manager receives compact exceptions and evidence; only an assigned brain resolves interpretation</x:v>
@@ -2417,10 +2657,10 @@
         <x:v>reviewer-sol-high</x:v>
       </x:c>
       <x:c r="C20" s="24" t="str">
-        <x:v>reviewer-astra-medium for unusually large cross-workstream scope</x:v>
+        <x:v>reviewer-astra-medium for unusually large cross-workstream scope; every Astra invocation requires fresh owner authorization and a concrete reason Sol high cannot fit</x:v>
       </x:c>
       <x:c r="D20" s="24" t="str">
-        <x:v>Mechanical gate collection may be delegated, but acceptance judgment belongs to an independent brain on the exact head</x:v>
+        <x:v>Run gates mechanically; batch one independent brain review at a meaningful integrated chunk boundary and bind it to the exact head</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -2436,20 +2676,20 @@
       <x:c r="D22"/>
     </x:row>
     <x:row r="23" ht="42" customHeight="1">
-      <x:c r="A23" s="240" t="str">
+      <x:c r="A23" s="312" t="str">
         <x:v>Selection rules</x:v>
       </x:c>
-      <x:c r="B23" s="241"/>
-      <x:c r="C23" s="241"/>
-      <x:c r="D23" s="242"/>
+      <x:c r="B23" s="313"/>
+      <x:c r="C23" s="313"/>
+      <x:c r="D23" s="314"/>
     </x:row>
     <x:row r="24" ht="42" customHeight="1">
-      <x:c r="A24" s="248" t="str">
+      <x:c r="A24" s="320" t="str">
         <x:v>Approved selection rule</x:v>
       </x:c>
-      <x:c r="B24" s="249"/>
-      <x:c r="C24" s="249"/>
-      <x:c r="D24" s="250"/>
+      <x:c r="B24" s="321"/>
+      <x:c r="C24" s="321"/>
+      <x:c r="D24" s="322"/>
     </x:row>
     <x:row r="25" ht="42" customHeight="1">
       <x:c r="A25" s="91" t="str">
@@ -2485,7 +2725,7 @@
     </x:row>
     <x:row r="29" ht="42" customHeight="1">
       <x:c r="A29" s="92" t="str">
-        <x:v>5. Semantic and risk acceptance is a brain task: use an independent Sol high reviewer, or Astra medium for unusually large cross-workstream scope. Mechanical workers may collect gates but cannot issue acceptance judgment.</x:v>
+        <x:v>5. Semantic and risk acceptance is a brain task: use an independent Sol high reviewer by default. Astra medium is eligible only for unusually large cross-workstream scope after fresh invocation-specific owner authorization and a concrete reason Sol high cannot fit. Mechanical workers may collect gates but cannot issue acceptance judgment.</x:v>
       </x:c>
       <x:c r="B29" s="69"/>
       <x:c r="C29" s="69"/>
@@ -2509,7 +2749,7 @@
     </x:row>
     <x:row r="32" ht="42" customHeight="1">
       <x:c r="A32" s="92" t="str">
-        <x:v>8. Use fast, low-cost mechanical workers when startup, supervision and integration overhead still improves accepted-result time or cost. Parallelize independent objectively testable packets after decisions, interfaces and write ownership are fixed.</x:v>
+        <x:v>8. Owner may set Codex delegation or leading to zero for a delivery. This overrides any planned mechanical allowance and preserves only explicitly requested Codex brain/review use.</x:v>
       </x:c>
       <x:c r="B32" s="69"/>
       <x:c r="C32" s="69"/>
@@ -2517,7 +2757,7 @@
     </x:row>
     <x:row r="33" ht="42" customHeight="1">
       <x:c r="A33" s="92" t="str">
-        <x:v>9. Muse Spark 1.3 is the preferred light mechanical and read/seek lane for repository search, file localization, evidence collection, narrow checks and small explicit edits.</x:v>
+        <x:v>9. Codex capacity is reserved for product/architecture judgment, integration decisions and independent semantic/risk review across the full usage window. Model quality alone does not justify Codex mechanical execution.</x:v>
       </x:c>
       <x:c r="B33" s="69"/>
       <x:c r="C33" s="69"/>
@@ -2525,7 +2765,7 @@
     </x:row>
     <x:row r="34" ht="42" customHeight="1">
       <x:c r="A34" s="92" t="str">
-        <x:v>10. Do not fragment work when dispatch, context transfer or integration overhead would erase the expected speed or cost gain.</x:v>
+        <x:v>10. External houses are the default mechanical lane. A Codex mechanical worker needs a recorded delivery allowance and reason; absence of an allowance means zero Codex mechanical dispatch.</x:v>
       </x:c>
       <x:c r="B34" s="69"/>
       <x:c r="C34" s="69"/>
@@ -2533,7 +2773,7 @@
     </x:row>
     <x:row r="35" ht="42" customHeight="1">
       <x:c r="A35" s="92" t="str">
-        <x:v>11. More reasoning is not universally more intelligence or better value. Terra max handles difficult settled implementation, not unresolved product decisions.</x:v>
+        <x:v>11. Codex mechanical concurrency defaults to one. Parallel Codex mechanical workers require explicit owner authorization; use qualified external houses for parallel execution.</x:v>
       </x:c>
       <x:c r="B35" s="69"/>
       <x:c r="C35" s="69"/>
@@ -2541,7 +2781,7 @@
     </x:row>
     <x:row r="36" ht="42" customHeight="1">
       <x:c r="A36" s="92" t="str">
-        <x:v>12. No automatic repeated effort increases. Stop, diagnose or reassign under existing watchdog and recovery limits.</x:v>
+        <x:v>12. Batch Codex brain questions and integrated reviews. Send compact evidence and exceptions gathered by mechanical workers instead of using Codex for broad repository exploration.</x:v>
       </x:c>
       <x:c r="B36" s="69"/>
       <x:c r="C36" s="69"/>
@@ -2549,7 +2789,7 @@
     </x:row>
     <x:row r="37" ht="42" customHeight="1">
       <x:c r="A37" s="92" t="str">
-        <x:v>13. High consequence can require stronger review even for a small edit. Model choice never removes acceptance gates.</x:v>
+        <x:v>13. Run build, test and evidence collection mechanically. Use one Sol-high semantic/risk review per meaningful integrated chunk; new remedy commits still require exact-head re-review.</x:v>
       </x:c>
       <x:c r="B37" s="69"/>
       <x:c r="C37" s="69"/>
@@ -2557,7 +2797,7 @@
     </x:row>
     <x:row r="38" ht="42" customHeight="1">
       <x:c r="A38" s="92" t="str">
-        <x:v>14. Verify effective model and effort at dispatch. Newly configured Grok/Opus combinations are not yet claimed smoke-tested; no unapproved substitution.</x:v>
+        <x:v>14. Use fast, low-cost mechanical workers when startup, supervision and integration overhead still improves accepted-result time or cost. Parallelize independent objectively testable packets after decisions, interfaces and write ownership are fixed.</x:v>
       </x:c>
       <x:c r="B38" s="69"/>
       <x:c r="C38" s="69"/>
@@ -2565,7 +2805,7 @@
     </x:row>
     <x:row r="39" ht="42" customHeight="1">
       <x:c r="A39" s="92" t="str">
-        <x:v>15. House exclusivity has two scopes. Astra at any effort reserves Codex globally and Fable 5.1 at any effort reserves Claude globally. Sol high or higher reserves Codex only for assignments under the same delivery manager; Opus high or higher reserves Claude only for assignments under the same delivery manager.</x:v>
+        <x:v>15. Muse Spark 1.3 is the preferred light mechanical and read/seek lane for repository search, file localization, evidence collection, narrow checks and small explicit edits.</x:v>
       </x:c>
       <x:c r="B39" s="69"/>
       <x:c r="C39" s="69"/>
@@ -2573,7 +2813,7 @@
     </x:row>
     <x:row r="40" ht="42" customHeight="1">
       <x:c r="A40" s="92" t="str">
-        <x:v>16. New-product brainstorming may use Fable 5.1 medium or Astra medium. Both create global house reservations while active; prefer another eligible house or queue competing work.</x:v>
+        <x:v>16. Do not fragment work when dispatch, context transfer or integration overhead would erase the expected speed or cost gain.</x:v>
       </x:c>
       <x:c r="B40" s="69"/>
       <x:c r="C40" s="69"/>
@@ -2581,7 +2821,7 @@
     </x:row>
     <x:row r="41" ht="42" customHeight="1">
       <x:c r="A41" s="92" t="str">
-        <x:v>17. Fable model authorization does not permit paid usage credits or extra spending. Verify included allowance before any headless request.</x:v>
+        <x:v>17. More reasoning is not universally more intelligence or better value. Terra max handles difficult settled implementation, not unresolved product decisions.</x:v>
       </x:c>
       <x:c r="B41" s="69"/>
       <x:c r="C41" s="69"/>
@@ -2589,7 +2829,7 @@
     </x:row>
     <x:row r="42" ht="42" customHeight="1">
       <x:c r="A42" s="92" t="str">
-        <x:v>18. The delivery manager keeps its turn active with a real bounded wait while workers run. It may finish only after terminal handbacks or explicit transfer to another live supervisor.</x:v>
+        <x:v>18. No automatic repeated effort increases. Stop, diagnose or reassign under existing watchdog and recovery limits.</x:v>
       </x:c>
       <x:c r="B42" s="69"/>
       <x:c r="C42" s="69"/>
@@ -2597,7 +2837,7 @@
     </x:row>
     <x:row r="43" ht="42" customHeight="1">
       <x:c r="A43" s="92" t="str">
-        <x:v>19. External provider streams are drained outside manager context. Retrieve compact lifecycle changes and the mechanically extracted final assistant result, not accumulated raw output.</x:v>
+        <x:v>19. High consequence can require stronger review even for a small edit. Model choice never removes acceptance gates.</x:v>
       </x:c>
       <x:c r="B43" s="69"/>
       <x:c r="C43" s="69"/>
@@ -2605,7 +2845,7 @@
     </x:row>
     <x:row r="44" ht="42" customHeight="1">
       <x:c r="A44" s="92" t="str">
-        <x:v>20. A provider parent exit does not transfer writer ownership. Verify process tree, worktree command/CWD holders and provider background-agent registry before any replacement writer.</x:v>
+        <x:v>20. Verify effective model and effort at dispatch. Newly configured Grok/Opus combinations are not yet claimed smoke-tested; no unapproved substitution.</x:v>
       </x:c>
       <x:c r="B44" s="69"/>
       <x:c r="C44" s="69"/>
@@ -2613,7 +2853,7 @@
     </x:row>
     <x:row r="45" ht="42" customHeight="1">
       <x:c r="A45" s="92" t="str">
-        <x:v>21. Stop Claude after two consecutive no-progress auto-compactions; checkpoint and use one fresh narrow retry rather than resuming the thrashing session.</x:v>
+        <x:v>21. House exclusivity has two scopes. Astra at any effort reserves Codex globally and Fable 5.1 at any effort reserves Claude globally. Sol high or higher reserves Codex only for assignments under the same delivery manager; Opus high or higher reserves Claude only for assignments under the same delivery manager.</x:v>
       </x:c>
       <x:c r="B45" s="69"/>
       <x:c r="C45" s="69"/>
@@ -2621,7 +2861,7 @@
     </x:row>
     <x:row r="46" ht="42" customHeight="1">
       <x:c r="A46" s="92" t="str">
-        <x:v>22. Owner concurrency exceptions are finite and journalled after an occupancy probe; leads and managers cannot self-authorize them.</x:v>
+        <x:v>22. New-product brainstorming uses Sol high by default. Fable 5.1 medium or Astra medium requires fresh invocation-specific owner authorization and a concrete reason Sol high cannot fit; Fable separately requires included-plan/no-extra-spend proof. Both create global house reservations while active.</x:v>
       </x:c>
       <x:c r="B46" s="69"/>
       <x:c r="C46" s="69"/>
@@ -2629,7 +2869,7 @@
     </x:row>
     <x:row r="47" ht="42" customHeight="1">
       <x:c r="A47" s="92" t="str">
-        <x:v>23. DeepSeek V4.1 Flash uses the provider code opencode-go/deepseek-v4.1-flash. The human-readable name and provider code identify the same approved model. The provider renamed this code from opencode-go/deepseek-flash, which no longer appears in `opencode models`; the version now lives in the code itself.</x:v>
+        <x:v>23. Fable model authorization does not permit paid usage credits or extra spending. Verify included allowance before any headless request.</x:v>
       </x:c>
       <x:c r="B47" s="69"/>
       <x:c r="C47" s="69"/>
@@ -2637,7 +2877,7 @@
     </x:row>
     <x:row r="48" ht="42" customHeight="1">
       <x:c r="A48" s="92" t="str">
-        <x:v>24. DeepSeek high is the default for bounded implementation. DeepSeek max mechanically implements novel public contract, identity, schema or serialization shapes only after an approved brain settles the shape and objective contract tests.</x:v>
+        <x:v>24. The delivery manager keeps its turn active with a real bounded wait while workers run. It may finish only after terminal handbacks or explicit transfer to another live supervisor.</x:v>
       </x:c>
       <x:c r="B48" s="69"/>
       <x:c r="C48" s="69"/>
@@ -2645,11 +2885,67 @@
     </x:row>
     <x:row r="49" ht="42" customHeight="1">
       <x:c r="A49" s="92" t="str">
-        <x:v>25. DeepSeek V4 Pro, DeepSeek V4 Flash and the vision-exp variants are excluded: opencode-go/deepseek-v4-pro, opencode-go/deepseek-v4-flash and opencode-go/deepseek-v4-flash-vision-exp are DIFFERENT models, not fallbacks for V4.1 Flash. If opencode-go/deepseek-v4.1-flash is unavailable, stop and reroute to a different approved house; never substitute another DeepSeek model.</x:v>
+        <x:v>25. External provider streams are drained outside manager context. Retrieve compact lifecycle changes and the mechanically extracted final assistant result, not accumulated raw output.</x:v>
       </x:c>
       <x:c r="B49" s="69"/>
       <x:c r="C49" s="69"/>
       <x:c r="D49" s="69"/>
+    </x:row>
+    <x:row r="50" ht="42" customHeight="1">
+      <x:c r="A50" s="92" t="str">
+        <x:v>26. A provider parent exit does not transfer writer ownership. Verify process tree, worktree command/CWD holders and provider background-agent registry before any replacement writer.</x:v>
+      </x:c>
+      <x:c r="B50" s="69"/>
+      <x:c r="C50" s="69"/>
+      <x:c r="D50" s="69"/>
+    </x:row>
+    <x:row r="51" ht="42" customHeight="1">
+      <x:c r="A51" s="92" t="str">
+        <x:v>27. Stop Claude after two consecutive no-progress auto-compactions; checkpoint and use one fresh narrow retry rather than resuming the thrashing session.</x:v>
+      </x:c>
+      <x:c r="B51" s="69"/>
+      <x:c r="C51" s="69"/>
+      <x:c r="D51" s="69"/>
+    </x:row>
+    <x:row r="52" ht="42" customHeight="1">
+      <x:c r="A52" s="92" t="str">
+        <x:v>28. Owner concurrency exceptions are finite and journalled after an occupancy probe; leads and managers cannot self-authorize them.</x:v>
+      </x:c>
+      <x:c r="B52" s="69"/>
+      <x:c r="C52" s="69"/>
+      <x:c r="D52" s="69"/>
+    </x:row>
+    <x:row r="53" ht="42" customHeight="1">
+      <x:c r="A53" s="92" t="str">
+        <x:v>29. DeepSeek V4.1 Flash uses the provider code opencode-go/deepseek-v4.1-flash. The human-readable name and provider code identify the same approved model. The provider renamed this code from opencode-go/deepseek-flash, which no longer appears in `opencode models`; the version now lives in the code itself.</x:v>
+      </x:c>
+      <x:c r="B53" s="69"/>
+      <x:c r="C53" s="69"/>
+      <x:c r="D53" s="69"/>
+    </x:row>
+    <x:row r="54" ht="42" customHeight="1">
+      <x:c r="A54" s="92" t="str">
+        <x:v>30. DeepSeek high is the default for bounded implementation. DeepSeek max mechanically implements novel public contract, identity, schema or serialization shapes only after an approved brain settles the shape and objective contract tests.</x:v>
+      </x:c>
+      <x:c r="B54" s="69"/>
+      <x:c r="C54" s="69"/>
+      <x:c r="D54" s="69"/>
+    </x:row>
+    <x:row r="55" ht="42" customHeight="1">
+      <x:c r="A55" s="92" t="str">
+        <x:v>31. DeepSeek V4 Pro, DeepSeek V4 Flash and the vision-exp variants are excluded: opencode-go/deepseek-v4-pro, opencode-go/deepseek-v4-flash and opencode-go/deepseek-v4-flash-vision-exp are DIFFERENT models, not fallbacks for V4.1 Flash. If opencode-go/deepseek-v4.1-flash is unavailable, stop and reroute to a different approved house; never substitute another DeepSeek model.</x:v>
+      </x:c>
+      <x:c r="B55" s="69"/>
+      <x:c r="C55" s="69"/>
+      <x:c r="D55" s="69"/>
+    </x:row>
+    <x:row r="56" ht="42" customHeight="1">
+      <x:c r="A56" s="92" t="str">
+        <x:v>32. Every Astra or Fable invocation in any role requires fresh explicit owner authorization bound to that start, resume, retry or follow-up, plus a concrete reason gpt-5.6-sol high cannot fit. Prior authorization is never reusable; Fable also requires included-plan/no-extra-spend proof.</x:v>
+      </x:c>
+      <x:c r="B56" s="69"/>
+      <x:c r="C56" s="69"/>
+      <x:c r="D56" s="69"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2679,6 +2975,13 @@
     <x:mergeCell ref="A47:D47"/>
     <x:mergeCell ref="A48:D48"/>
     <x:mergeCell ref="A49:D49"/>
+    <x:mergeCell ref="A50:D50"/>
+    <x:mergeCell ref="A51:D51"/>
+    <x:mergeCell ref="A52:D52"/>
+    <x:mergeCell ref="A53:D53"/>
+    <x:mergeCell ref="A54:D54"/>
+    <x:mergeCell ref="A55:D55"/>
+    <x:mergeCell ref="A56:D56"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2710,7 +3013,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>Policy source: Interchange policy v0.6.0</x:v>
+        <x:v>Policy source: Interchange policy v0.8.0</x:v>
       </x:c>
       <x:c r="B3" s="2" t="str">
         <x:v>Approved on</x:v>
@@ -2837,57 +3140,145 @@
     </x:row>
     <x:row r="16" ht="50" customHeight="1">
       <x:c r="A16" s="24" t="str">
-        <x:v>Usage</x:v>
+        <x:v>Owner zero-Codex override</x:v>
       </x:c>
       <x:c r="B16" s="24" t="str">
-        <x:v>Parse available CLI usage mechanically; unknown when absent</x:v>
+        <x:v>Explicit do-not-use-Codex-for-delegation-or-leading instruction</x:v>
       </x:c>
       <x:c r="C16" s="24" t="str">
-        <x:v>Store input/output/cache/reasoning separately; do not assume provider counters are additive</x:v>
+        <x:v>Set Codex mechanical worker and mechanical lead allowance to zero; retain only explicitly requested brain/review use</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="50" customHeight="1">
       <x:c r="A17" s="24" t="str">
-        <x:v>Supervision ownership</x:v>
+        <x:v>Codex capacity preflight</x:v>
       </x:c>
       <x:c r="B17" s="24" t="str">
-        <x:v>Manager turn remains active until terminal handback or explicit live-supervisor transfer</x:v>
+        <x:v>Fresh usage snapshot when available + declared brain/review reserve + explicit mechanical allowance</x:v>
       </x:c>
       <x:c r="C17" s="24" t="str">
-        <x:v>A wait timeout, session ID or future promise is not a continuation mechanism</x:v>
+        <x:v>No recorded allowance means zero new Codex mechanical workers; external houses are the default execution lane</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="50" customHeight="1">
       <x:c r="A18" s="24" t="str">
-        <x:v>Output isolation</x:v>
+        <x:v>Codex mechanical concurrency</x:v>
       </x:c>
       <x:c r="B18" s="24" t="str">
-        <x:v>Adapter drains provider streams outside manager context</x:v>
+        <x:v>At most 1 active by default</x:v>
       </x:c>
       <x:c r="C18" s="24" t="str">
-        <x:v>Manager receives lifecycle changes, final assistant result, usage, warnings and exit state only</x:v>
+        <x:v>Parallel Codex mechanical workers require explicit owner authorization; prefer external-house parallelism</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="50" customHeight="1">
       <x:c r="A19" s="24" t="str">
-        <x:v>Attempt ceilings</x:v>
+        <x:v>Codex early burn checkpoint</x:v>
       </x:c>
       <x:c r="B19" s="24" t="str">
-        <x:v>Finite wall-time and turn ceilings; token/cost ceilings where timely counters exist</x:v>
+        <x:v>Recheck after first mechanical checkpoint when usage is observable</x:v>
       </x:c>
       <x:c r="C19" s="24" t="str">
-        <x:v>Stop deterministic blockers; do not spend a ceiling rediscovering known failures</x:v>
+        <x:v>Freeze new Codex mechanical dispatch when burn exceeds allowance or threatens reserved brain/review capacity</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="50" customHeight="1">
       <x:c r="A20" s="24" t="str">
+        <x:v>Codex review batching</x:v>
+      </x:c>
+      <x:c r="B20" s="24" t="str">
+        <x:v>One semantic/risk reviewer per meaningful integrated chunk</x:v>
+      </x:c>
+      <x:c r="C20" s="24" t="str">
+        <x:v>Mechanical gates run outside Codex; remedy commits invalidate prior review and require exact-head re-review</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="50" customHeight="1">
+      <x:c r="A21" s="24" t="str">
+        <x:v>Usage</x:v>
+      </x:c>
+      <x:c r="B21" s="24" t="str">
+        <x:v>Parse available CLI usage mechanically; unknown when absent</x:v>
+      </x:c>
+      <x:c r="C21" s="24" t="str">
+        <x:v>Store input/output/cache/reasoning separately; do not assume provider counters are additive</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="50" customHeight="1">
+      <x:c r="A22" s="24" t="str">
+        <x:v>Supervision ownership</x:v>
+      </x:c>
+      <x:c r="B22" s="24" t="str">
+        <x:v>Manager turn remains active until terminal handback or explicit live-supervisor transfer</x:v>
+      </x:c>
+      <x:c r="C22" s="24" t="str">
+        <x:v>A wait timeout, session ID or future promise is not a continuation mechanism</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="50" customHeight="1">
+      <x:c r="A23" s="24" t="str">
+        <x:v>Output isolation</x:v>
+      </x:c>
+      <x:c r="B23" s="24" t="str">
+        <x:v>Adapter drains provider streams outside manager context</x:v>
+      </x:c>
+      <x:c r="C23" s="24" t="str">
+        <x:v>Manager receives lifecycle changes, final assistant result, usage, warnings and exit state only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="50" customHeight="1">
+      <x:c r="A24" s="24" t="str">
+        <x:v>Attempt ceilings</x:v>
+      </x:c>
+      <x:c r="B24" s="24" t="str">
+        <x:v>Finite wall-time and turn ceilings; token/cost ceilings where timely counters exist</x:v>
+      </x:c>
+      <x:c r="C24" s="24" t="str">
+        <x:v>Stop deterministic blockers; do not spend a ceiling rediscovering known failures</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="50" customHeight="1">
+      <x:c r="A25" s="24" t="str">
         <x:v>Claude compaction</x:v>
       </x:c>
-      <x:c r="B20" s="24" t="str">
+      <x:c r="B25" s="24" t="str">
         <x:v>Stop after 2 consecutive auto-compactions without artifact, evidence or gate progress</x:v>
       </x:c>
-      <x:c r="C20" s="24" t="str">
+      <x:c r="C25" s="24" t="str">
         <x:v>Classify autocompact_thrashing as context/transport failure; retry fresh and narrow, never resume that context</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="50" customHeight="1">
+      <x:c r="A26" s="24" t="str">
+        <x:v>Astra/Fable invocation authorization</x:v>
+      </x:c>
+      <x:c r="B26" s="24" t="str">
+        <x:v>Fresh explicit owner authorization for every start, resume, retry and follow-up</x:v>
+      </x:c>
+      <x:c r="C26" s="24" t="str">
+        <x:v>Bind approval to packet, attempt and invocation ID plus model/effort/role; manager or lead cannot self-authorize</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="50" customHeight="1">
+      <x:c r="A27" s="24" t="str">
+        <x:v>Sol-high non-fit reason</x:v>
+      </x:c>
+      <x:c r="B27" s="24" t="str">
+        <x:v>Concrete recorded reason gpt-5.6-sol high cannot fit</x:v>
+      </x:c>
+      <x:c r="C27" s="24" t="str">
+        <x:v>Vague preference or prior approval fails closed; use Sol high if it fits or wait for owner</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="50" customHeight="1">
+      <x:c r="A28" s="24" t="str">
+        <x:v>Astra/Fable authorization reuse</x:v>
+      </x:c>
+      <x:c r="B28" s="24" t="str">
+        <x:v>Forbidden</x:v>
+      </x:c>
+      <x:c r="C28" s="24" t="str">
+        <x:v>A completed, failed or suspended invocation consumes its authorization; the next invocation needs a new owner decision</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2921,7 +3312,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>Policy source: Interchange policy v0.6.0</x:v>
+        <x:v>Policy source: Interchange policy v0.8.0</x:v>
       </x:c>
       <x:c r="B3" s="2" t="str">
         <x:v>Approved on</x:v>
@@ -3084,20 +3475,20 @@
       <x:c r="C22"/>
     </x:row>
     <x:row r="23" ht="26" customHeight="1">
-      <x:c r="A23" s="240" t="str">
+      <x:c r="A23" s="312" t="str">
         <x:v>Recovery playbook</x:v>
       </x:c>
-      <x:c r="B23" s="241"/>
-      <x:c r="C23" s="242"/>
+      <x:c r="B23" s="313"/>
+      <x:c r="C23" s="314"/>
     </x:row>
     <x:row r="24" ht="44" customHeight="1">
-      <x:c r="A24" s="248" t="str">
+      <x:c r="A24" s="320" t="str">
         <x:v>Failure</x:v>
       </x:c>
-      <x:c r="B24" s="249" t="str">
+      <x:c r="B24" s="321" t="str">
         <x:v>First action</x:v>
       </x:c>
-      <x:c r="C24" s="250" t="str">
+      <x:c r="C24" s="322" t="str">
         <x:v>Escalation</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
feat(interchange): define capacity tiers
</commit_message>
<xml_diff>
--- a/outputs/interchange-design/interchange.xlsx
+++ b/outputs/interchange-design/interchange.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profiles" sheetId="1" r:id="R801cbea57ead49c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Routing" sheetId="2" r:id="Rbe456525160944ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monitoring" sheetId="3" r:id="Rd03ae35d614a4084"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Recovery" sheetId="4" r:id="R78027977ff274756"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profiles" sheetId="1" r:id="R6e388f50fc5a4db4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Routing" sheetId="2" r:id="Rf8dca8fa3cb84187"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monitoring" sheetId="3" r:id="R99f2394bd14f4cb9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Recovery" sheetId="4" r:id="R51e7c5e621e944f0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -55,7 +55,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="67">
+  <x:fills count="79">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -85,6 +85,66 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFCE4D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -460,7 +520,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="323">
+  <x:cellXfs count="377">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1230,6 +1290,126 @@
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="66" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="67" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="67" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="68" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="68" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="67" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="69" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="69" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="69" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="69" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="69" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="70" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="70" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="70" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="70" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="70" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="70" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="70" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="70" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="71" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="71" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="72" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="72" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="71" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="73" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="73" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="73" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="73" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="73" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="74" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="74" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="74" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="74" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="74" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="74" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="74" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="74" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="75" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="75" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="76" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="76" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="75" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="77" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="77" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="77" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="77" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="77" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="78" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="78" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="78" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="78" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="78" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="78" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="78" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="78" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1474,7 +1654,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>Policy source: Interchange policy v0.8.0</x:v>
+        <x:v>Policy source: Interchange policy v0.9.0</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -1697,10 +1877,10 @@
       <x:c r="F16" s="34" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G16" s="305" t="str">
+      <x:c r="G16" s="359" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H16" s="307" t="str">
+      <x:c r="H16" s="361" t="str">
         <x:v>Profile documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I16" s="22" t="str">
@@ -1726,10 +1906,10 @@
       <x:c r="F17" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G17" s="306" t="str">
+      <x:c r="G17" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H17" s="308" t="str">
+      <x:c r="H17" s="362" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I17" s="24" t="str">
@@ -1755,10 +1935,10 @@
       <x:c r="F18" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G18" s="306" t="str">
+      <x:c r="G18" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H18" s="308" t="str">
+      <x:c r="H18" s="362" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I18" s="24" t="str">
@@ -1784,10 +1964,10 @@
       <x:c r="F19" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G19" s="306" t="str">
+      <x:c r="G19" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H19" s="308" t="str">
+      <x:c r="H19" s="362" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I19" s="24" t="str">
@@ -1813,10 +1993,10 @@
       <x:c r="F20" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G20" s="306" t="str">
+      <x:c r="G20" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H20" s="308" t="str">
+      <x:c r="H20" s="362" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I20" s="24" t="str">
@@ -1842,10 +2022,10 @@
       <x:c r="F21" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G21" s="306" t="str">
+      <x:c r="G21" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H21" s="308" t="str">
+      <x:c r="H21" s="362" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I21" s="24" t="str">
@@ -1871,10 +2051,10 @@
       <x:c r="F22" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G22" s="306" t="str">
+      <x:c r="G22" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H22" s="308" t="str">
+      <x:c r="H22" s="362" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I22" s="24" t="str">
@@ -1900,10 +2080,10 @@
       <x:c r="F23" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G23" s="306" t="str">
+      <x:c r="G23" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H23" s="308" t="str">
+      <x:c r="H23" s="362" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I23" s="24" t="str">
@@ -1929,10 +2109,10 @@
       <x:c r="F24" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G24" s="306" t="str">
+      <x:c r="G24" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H24" s="308" t="str">
+      <x:c r="H24" s="362" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I24" s="24" t="str">
@@ -1958,10 +2138,10 @@
       <x:c r="F25" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G25" s="306" t="str">
+      <x:c r="G25" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H25" s="308" t="str">
+      <x:c r="H25" s="362" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I25" s="24" t="str">
@@ -1987,10 +2167,10 @@
       <x:c r="F26" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G26" s="306" t="str">
+      <x:c r="G26" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H26" s="308" t="str">
+      <x:c r="H26" s="362" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I26" s="24" t="str">
@@ -2016,10 +2196,10 @@
       <x:c r="F27" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G27" s="306" t="str">
+      <x:c r="G27" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H27" s="308" t="str">
+      <x:c r="H27" s="362" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I27" s="24" t="str">
@@ -2045,10 +2225,10 @@
       <x:c r="F28" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G28" s="306" t="str">
+      <x:c r="G28" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H28" s="308" t="str">
+      <x:c r="H28" s="362" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I28" s="24" t="str">
@@ -2074,10 +2254,10 @@
       <x:c r="F29" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G29" s="306" t="str">
+      <x:c r="G29" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H29" s="309" t="str">
+      <x:c r="H29" s="363" t="str">
         <x:v>Smoke-tested</x:v>
       </x:c>
       <x:c r="I29" s="24" t="str">
@@ -2103,10 +2283,10 @@
       <x:c r="F30" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G30" s="306" t="str">
+      <x:c r="G30" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H30" s="308" t="str">
+      <x:c r="H30" s="362" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I30" s="24" t="str">
@@ -2132,10 +2312,10 @@
       <x:c r="F31" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G31" s="306" t="str">
+      <x:c r="G31" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H31" s="308" t="str">
+      <x:c r="H31" s="362" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I31" s="24" t="str">
@@ -2161,10 +2341,10 @@
       <x:c r="F32" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G32" s="306" t="str">
+      <x:c r="G32" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H32" s="308" t="str">
+      <x:c r="H32" s="362" t="str">
         <x:v>CLI model and effort documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I32" s="24" t="str">
@@ -2190,10 +2370,10 @@
       <x:c r="F33" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G33" s="306" t="str">
+      <x:c r="G33" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H33" s="308" t="str">
+      <x:c r="H33" s="362" t="str">
         <x:v>CLI model and effort documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I33" s="24" t="str">
@@ -2219,10 +2399,10 @@
       <x:c r="F34" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G34" s="306" t="str">
+      <x:c r="G34" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H34" s="308" t="str">
+      <x:c r="H34" s="362" t="str">
         <x:v>Profile documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I34" s="24" t="str">
@@ -2248,10 +2428,10 @@
       <x:c r="F35" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G35" s="306" t="str">
+      <x:c r="G35" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H35" s="308" t="str">
+      <x:c r="H35" s="362" t="str">
         <x:v>Profile documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I35" s="24" t="str">
@@ -2277,10 +2457,10 @@
       <x:c r="F36" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G36" s="306" t="str">
+      <x:c r="G36" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H36" s="308" t="str">
+      <x:c r="H36" s="362" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I36" s="24" t="str">
@@ -2306,10 +2486,10 @@
       <x:c r="F37" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G37" s="306" t="str">
+      <x:c r="G37" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H37" s="308" t="str">
+      <x:c r="H37" s="362" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I37" s="24" t="str">
@@ -2335,10 +2515,10 @@
       <x:c r="F38" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G38" s="306" t="str">
+      <x:c r="G38" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H38" s="308" t="str">
+      <x:c r="H38" s="362" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I38" s="24" t="str">
@@ -2364,10 +2544,10 @@
       <x:c r="F39" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G39" s="306" t="str">
+      <x:c r="G39" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H39" s="308" t="str">
+      <x:c r="H39" s="362" t="str">
         <x:v>Profile documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I39" s="24" t="str">
@@ -2393,10 +2573,10 @@
       <x:c r="F40" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G40" s="306" t="str">
+      <x:c r="G40" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H40" s="308" t="str">
+      <x:c r="H40" s="362" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I40" s="24" t="str">
@@ -2437,7 +2617,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>Policy source: Interchange policy v0.8.0</x:v>
+        <x:v>Policy source: Interchange policy v0.9.0</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2" t="str">
@@ -2517,7 +2697,7 @@
         <x:v>Local search/tool when immediate; worker-muse-xhigh when delegation frees the Codex brain or is faster overall</x:v>
       </x:c>
       <x:c r="C10" s="24" t="str">
-        <x:v>Another external read-only mechanical profile; Codex worker only under a recorded mechanical allowance</x:v>
+        <x:v>worker-luna-xhigh or worker-luna-max or another bounded read-only profile; Luna needs no balancing allowance</x:v>
       </x:c>
       <x:c r="D10" s="24" t="str">
         <x:v>Count startup, supervision and handback overhead; delegate when it improves accepted-result time or cost</x:v>
@@ -2531,7 +2711,7 @@
         <x:v>worker-muse-xhigh</x:v>
       </x:c>
       <x:c r="C11" s="24" t="str">
-        <x:v>Another external bounded worker; Luna xhigh/max only under a recorded Codex mechanical allowance</x:v>
+        <x:v>worker-luna-xhigh or worker-luna-max or another bounded worker; Luna, Muse and DeepSeek need no balancing allowance</x:v>
       </x:c>
       <x:c r="D11" s="24" t="str">
         <x:v>Repository search, localization, evidence collection, narrow checks and small explicit edits; no interpretation</x:v>
@@ -2545,7 +2725,7 @@
         <x:v>worker-deepseek-flash-high; worker-grok-high; worker-opus-medium; worker-terra-xhigh; worker-sol-medium</x:v>
       </x:c>
       <x:c r="C12" s="24" t="str">
-        <x:v>Codex worker from this pool only under a recorded mechanical allowance and after external fit/availability check</x:v>
+        <x:v>Prefer unrestricted DeepSeek/Muse/Luna when task-fit; Terra/Sol require measured Codex allowance and Claude Code remains moderate/balanced</x:v>
       </x:c>
       <x:c r="D12" s="24" t="str">
         <x:v>Settled behavior, objective acceptance and bounded dependencies; ambiguity already resolved by a brain</x:v>
@@ -2573,7 +2753,7 @@
         <x:v>lead-sol-high resolves judgment; worker-opus-high or another qualified external profile executes settled packets</x:v>
       </x:c>
       <x:c r="C14" s="24" t="str">
-        <x:v>lead-astra-medium resolves unusually large ambiguity; Codex mechanical worker requires a recorded allowance; every Astra invocation requires fresh owner authorization and a concrete reason Sol high cannot fit</x:v>
+        <x:v>lead-astra-medium resolves unusually large ambiguity; Terra/Sol mechanical worker requires a recorded allowance; every Astra invocation requires fresh owner authorization and a concrete reason Sol high cannot fit</x:v>
       </x:c>
       <x:c r="D14" s="24" t="str">
         <x:v>Separate consequential decisions from implementation; independent review remains mandatory</x:v>
@@ -2587,7 +2767,7 @@
         <x:v>worker-deepseek-flash-high; worker-opus-high</x:v>
       </x:c>
       <x:c r="C15" s="24" t="str">
-        <x:v>worker-terra-max only under a recorded Codex mechanical allowance; never DeepSeek V4 Pro</x:v>
+        <x:v>worker-terra-max only under a recorded Terra/Sol mechanical allowance; never DeepSeek V4 Pro</x:v>
       </x:c>
       <x:c r="D15" s="24" t="str">
         <x:v>Dense mechanical implementation or integration with exact contracts and tests; never assign interpretation or use effort to outlast a loop</x:v>
@@ -2615,7 +2795,7 @@
         <x:v>Current delivery manager coordinates settled packets across external mechanical workers</x:v>
       </x:c>
       <x:c r="C17" s="24" t="str">
-        <x:v>lead-terra-xhigh/max only under a recorded Codex mechanical allowance</x:v>
+        <x:v>lead-terra-xhigh/max only under a recorded Terra/Sol mechanical allowance</x:v>
       </x:c>
       <x:c r="D17" s="24" t="str">
         <x:v>Preserve Codex brain capacity; a mechanical lead coordinates only settled work and returns ambiguity to Sol high or Astra medium</x:v>
@@ -2676,20 +2856,20 @@
       <x:c r="D22"/>
     </x:row>
     <x:row r="23" ht="42" customHeight="1">
-      <x:c r="A23" s="312" t="str">
+      <x:c r="A23" s="366" t="str">
         <x:v>Selection rules</x:v>
       </x:c>
-      <x:c r="B23" s="313"/>
-      <x:c r="C23" s="313"/>
-      <x:c r="D23" s="314"/>
+      <x:c r="B23" s="367"/>
+      <x:c r="C23" s="367"/>
+      <x:c r="D23" s="368"/>
     </x:row>
     <x:row r="24" ht="42" customHeight="1">
-      <x:c r="A24" s="320" t="str">
+      <x:c r="A24" s="374" t="str">
         <x:v>Approved selection rule</x:v>
       </x:c>
-      <x:c r="B24" s="321"/>
-      <x:c r="C24" s="321"/>
-      <x:c r="D24" s="322"/>
+      <x:c r="B24" s="375"/>
+      <x:c r="C24" s="375"/>
+      <x:c r="D24" s="376"/>
     </x:row>
     <x:row r="25" ht="42" customHeight="1">
       <x:c r="A25" s="91" t="str">
@@ -2757,7 +2937,7 @@
     </x:row>
     <x:row r="33" ht="42" customHeight="1">
       <x:c r="A33" s="92" t="str">
-        <x:v>9. Codex capacity is reserved for product/architecture judgment, integration decisions and independent semantic/risk review across the full usage window. Model quality alone does not justify Codex mechanical execution.</x:v>
+        <x:v>9. Sol, Terra and Claude Code are moderate, balanced capacity. Preserve Sol for judgment, integration and independent semantic/risk review; use unrestricted Luna, DeepSeek and Muse for suitable mechanical work and balance premium work across Claude/Codex when fit is comparable.</x:v>
       </x:c>
       <x:c r="B33" s="69"/>
       <x:c r="C33" s="69"/>
@@ -2765,7 +2945,7 @@
     </x:row>
     <x:row r="34" ht="42" customHeight="1">
       <x:c r="A34" s="92" t="str">
-        <x:v>10. External houses are the default mechanical lane. A Codex mechanical worker needs a recorded delivery allowance and reason; absence of an allowance means zero Codex mechanical dispatch.</x:v>
+        <x:v>10. Luna xhigh/max, DeepSeek V4.1 Flash and Muse Spark 1.3 are the unrestricted mechanical tier. They require no balancing allowance and have no Interchange concurrency cap when packets are independent and non-overlapping.</x:v>
       </x:c>
       <x:c r="B34" s="69"/>
       <x:c r="C34" s="69"/>
@@ -2773,7 +2953,7 @@
     </x:row>
     <x:row r="35" ht="42" customHeight="1">
       <x:c r="A35" s="92" t="str">
-        <x:v>11. Codex mechanical concurrency defaults to one. Parallel Codex mechanical workers require explicit owner authorization; use qualified external houses for parallel execution.</x:v>
+        <x:v>11. Terra/Sol mechanical concurrency defaults to one and requires a recorded allowance; parallel Terra/Sol workers require explicit owner authorization. Luna is exempt unless Astra exclusivity or an owner zero-Codex override applies.</x:v>
       </x:c>
       <x:c r="B35" s="69"/>
       <x:c r="C35" s="69"/>
@@ -2853,7 +3033,7 @@
     </x:row>
     <x:row r="45" ht="42" customHeight="1">
       <x:c r="A45" s="92" t="str">
-        <x:v>21. House exclusivity has two scopes. Astra at any effort reserves Codex globally and Fable 5.1 at any effort reserves Claude globally. Sol high or higher reserves Codex only for assignments under the same delivery manager; Opus high or higher reserves Claude only for assignments under the same delivery manager.</x:v>
+        <x:v>21. House exclusivity has two scopes. Astra at any effort reserves Codex globally and Fable 5.1 at any effort reserves Claude globally. Sol high or higher reserves Codex under the same delivery manager except unrestricted Luna xhigh/max mechanical leaves; Opus high or higher reserves Claude under the same delivery manager without that exception.</x:v>
       </x:c>
       <x:c r="B45" s="69"/>
       <x:c r="C45" s="69"/>
@@ -2946,6 +3126,22 @@
       <x:c r="B56" s="69"/>
       <x:c r="C56" s="69"/>
       <x:c r="D56" s="69"/>
+    </x:row>
+    <x:row r="57" ht="42" customHeight="1">
+      <x:c r="A57" s="92" t="str">
+        <x:v>33. Unrestricted does not mean ungoverned: Luna, DeepSeek and Muse still require bounded mechanical packets, non-overlapping ownership, watchdogs, valid completion and independent acceptance. Do not duplicate work merely because capacity is available.</x:v>
+      </x:c>
+      <x:c r="B57" s="69"/>
+      <x:c r="C57" s="69"/>
+      <x:c r="D57" s="69"/>
+    </x:row>
+    <x:row r="58" ht="42" customHeight="1">
+      <x:c r="A58" s="92" t="str">
+        <x:v>34. Grok retains its approved task-fit routing but is not part of the unrestricted tier or the new Terra/Sol/Claude balancing rule.</x:v>
+      </x:c>
+      <x:c r="B58" s="69"/>
+      <x:c r="C58" s="69"/>
+      <x:c r="D58" s="69"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2982,6 +3178,8 @@
     <x:mergeCell ref="A54:D54"/>
     <x:mergeCell ref="A55:D55"/>
     <x:mergeCell ref="A56:D56"/>
+    <x:mergeCell ref="A57:D57"/>
+    <x:mergeCell ref="A58:D58"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -3013,7 +3211,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>Policy source: Interchange policy v0.8.0</x:v>
+        <x:v>Policy source: Interchange policy v0.9.0</x:v>
       </x:c>
       <x:c r="B3" s="2" t="str">
         <x:v>Approved on</x:v>
@@ -3146,40 +3344,40 @@
         <x:v>Explicit do-not-use-Codex-for-delegation-or-leading instruction</x:v>
       </x:c>
       <x:c r="C16" s="24" t="str">
-        <x:v>Set Codex mechanical worker and mechanical lead allowance to zero; retain only explicitly requested brain/review use</x:v>
+        <x:v>Set every Codex mechanical worker and lead allocation, including Luna, to zero; retain only explicitly requested brain/review use</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="50" customHeight="1">
       <x:c r="A17" s="24" t="str">
-        <x:v>Codex capacity preflight</x:v>
+        <x:v>Terra/Sol capacity preflight</x:v>
       </x:c>
       <x:c r="B17" s="24" t="str">
-        <x:v>Fresh usage snapshot when available + declared brain/review reserve + explicit mechanical allowance</x:v>
+        <x:v>Fresh usage snapshot when available + declared brain/review reserve + explicit Terra/Sol mechanical allowance</x:v>
       </x:c>
       <x:c r="C17" s="24" t="str">
-        <x:v>No recorded allowance means zero new Codex mechanical workers; external houses are the default execution lane</x:v>
+        <x:v>No recorded allowance means zero new Terra/Sol mechanical workers; Luna is exempt unless Astra exclusivity or an owner zero-Codex override applies</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="50" customHeight="1">
       <x:c r="A18" s="24" t="str">
-        <x:v>Codex mechanical concurrency</x:v>
+        <x:v>Terra/Sol mechanical concurrency</x:v>
       </x:c>
       <x:c r="B18" s="24" t="str">
         <x:v>At most 1 active by default</x:v>
       </x:c>
       <x:c r="C18" s="24" t="str">
-        <x:v>Parallel Codex mechanical workers require explicit owner authorization; prefer external-house parallelism</x:v>
+        <x:v>Parallel Terra/Sol mechanical workers require explicit owner authorization; Luna is unrestricted by this cap</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="50" customHeight="1">
       <x:c r="A19" s="24" t="str">
-        <x:v>Codex early burn checkpoint</x:v>
+        <x:v>Terra/Sol early burn checkpoint</x:v>
       </x:c>
       <x:c r="B19" s="24" t="str">
-        <x:v>Recheck after first mechanical checkpoint when usage is observable</x:v>
+        <x:v>Recheck after first Terra/Sol mechanical checkpoint when usage is observable</x:v>
       </x:c>
       <x:c r="C19" s="24" t="str">
-        <x:v>Freeze new Codex mechanical dispatch when burn exceeds allowance or threatens reserved brain/review capacity</x:v>
+        <x:v>Freeze new Terra/Sol mechanical dispatch when burn exceeds allowance or threatens reserved brain/review capacity</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="50" customHeight="1">
@@ -3279,6 +3477,39 @@
       </x:c>
       <x:c r="C28" s="24" t="str">
         <x:v>A completed, failed or suspended invocation consumes its authorization; the next invocation needs a new owner decision</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="50" customHeight="1">
+      <x:c r="A29" s="24" t="str">
+        <x:v>Unrestricted mechanical tier</x:v>
+      </x:c>
+      <x:c r="B29" s="24" t="str">
+        <x:v>Luna xhigh/max, DeepSeek V4.1 Flash high/max, Muse Spark 1.3 xhigh</x:v>
+      </x:c>
+      <x:c r="C29" s="24" t="str">
+        <x:v>No balancing prerequisite or Interchange concurrency cap; three, four, five or more may run when assignments are useful, independent and non-overlapping</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="50" customHeight="1">
+      <x:c r="A30" s="24" t="str">
+        <x:v>Unrestricted-tier safeguards</x:v>
+      </x:c>
+      <x:c r="B30" s="24" t="str">
+        <x:v>Normal ownership, watchdog, completion and independent-acceptance rules remain</x:v>
+      </x:c>
+      <x:c r="C30" s="24" t="str">
+        <x:v>Free use never permits duplicate writers, overlapping paths, interpretation, unbounded loops or extra spending</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="50" customHeight="1">
+      <x:c r="A31" s="24" t="str">
+        <x:v>Moderate balanced tier</x:v>
+      </x:c>
+      <x:c r="B31" s="24" t="str">
+        <x:v>Terra, Sol and Claude Code</x:v>
+      </x:c>
+      <x:c r="C31" s="24" t="str">
+        <x:v>Plan and observe usage, protect brain/review capacity, avoid unnecessary concentration and balance across Claude/Codex when task fit is comparable; no forced alternation</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3312,7 +3543,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>Policy source: Interchange policy v0.8.0</x:v>
+        <x:v>Policy source: Interchange policy v0.9.0</x:v>
       </x:c>
       <x:c r="B3" s="2" t="str">
         <x:v>Approved on</x:v>
@@ -3475,20 +3706,20 @@
       <x:c r="C22"/>
     </x:row>
     <x:row r="23" ht="26" customHeight="1">
-      <x:c r="A23" s="312" t="str">
+      <x:c r="A23" s="366" t="str">
         <x:v>Recovery playbook</x:v>
       </x:c>
-      <x:c r="B23" s="313"/>
-      <x:c r="C23" s="314"/>
+      <x:c r="B23" s="367"/>
+      <x:c r="C23" s="368"/>
     </x:row>
     <x:row r="24" ht="44" customHeight="1">
-      <x:c r="A24" s="320" t="str">
+      <x:c r="A24" s="374" t="str">
         <x:v>Failure</x:v>
       </x:c>
-      <x:c r="B24" s="321" t="str">
+      <x:c r="B24" s="375" t="str">
         <x:v>First action</x:v>
       </x:c>
-      <x:c r="C24" s="322" t="str">
+      <x:c r="C24" s="376" t="str">
         <x:v>Escalation</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
feat(interchange): define capacity tiers (#6)
</commit_message>
<xml_diff>
--- a/outputs/interchange-design/interchange.xlsx
+++ b/outputs/interchange-design/interchange.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profiles" sheetId="1" r:id="R801cbea57ead49c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Routing" sheetId="2" r:id="Rbe456525160944ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monitoring" sheetId="3" r:id="Rd03ae35d614a4084"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Recovery" sheetId="4" r:id="R78027977ff274756"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profiles" sheetId="1" r:id="R6e388f50fc5a4db4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Routing" sheetId="2" r:id="Rf8dca8fa3cb84187"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monitoring" sheetId="3" r:id="R99f2394bd14f4cb9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Recovery" sheetId="4" r:id="R51e7c5e621e944f0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -55,7 +55,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="67">
+  <x:fills count="79">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -85,6 +85,66 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFCE4D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -460,7 +520,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="323">
+  <x:cellXfs count="377">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1230,6 +1290,126 @@
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="66" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="67" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="67" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="68" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="68" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="67" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="69" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="69" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="69" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="69" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="69" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="70" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="70" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="70" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="70" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="70" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="70" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="70" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="70" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="71" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="71" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="72" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="72" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="71" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="73" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="73" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="73" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="73" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="73" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="74" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="74" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="74" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="74" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="74" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="74" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="74" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="74" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="75" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="75" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="76" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="76" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="75" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="77" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="77" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="77" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="77" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="77" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="78" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="78" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="78" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="78" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="78" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="78" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="78" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="78" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1474,7 +1654,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>Policy source: Interchange policy v0.8.0</x:v>
+        <x:v>Policy source: Interchange policy v0.9.0</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -1697,10 +1877,10 @@
       <x:c r="F16" s="34" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G16" s="305" t="str">
+      <x:c r="G16" s="359" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H16" s="307" t="str">
+      <x:c r="H16" s="361" t="str">
         <x:v>Profile documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I16" s="22" t="str">
@@ -1726,10 +1906,10 @@
       <x:c r="F17" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G17" s="306" t="str">
+      <x:c r="G17" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H17" s="308" t="str">
+      <x:c r="H17" s="362" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I17" s="24" t="str">
@@ -1755,10 +1935,10 @@
       <x:c r="F18" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G18" s="306" t="str">
+      <x:c r="G18" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H18" s="308" t="str">
+      <x:c r="H18" s="362" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I18" s="24" t="str">
@@ -1784,10 +1964,10 @@
       <x:c r="F19" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G19" s="306" t="str">
+      <x:c r="G19" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H19" s="308" t="str">
+      <x:c r="H19" s="362" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I19" s="24" t="str">
@@ -1813,10 +1993,10 @@
       <x:c r="F20" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G20" s="306" t="str">
+      <x:c r="G20" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H20" s="308" t="str">
+      <x:c r="H20" s="362" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I20" s="24" t="str">
@@ -1842,10 +2022,10 @@
       <x:c r="F21" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G21" s="306" t="str">
+      <x:c r="G21" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H21" s="308" t="str">
+      <x:c r="H21" s="362" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I21" s="24" t="str">
@@ -1871,10 +2051,10 @@
       <x:c r="F22" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G22" s="306" t="str">
+      <x:c r="G22" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H22" s="308" t="str">
+      <x:c r="H22" s="362" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I22" s="24" t="str">
@@ -1900,10 +2080,10 @@
       <x:c r="F23" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G23" s="306" t="str">
+      <x:c r="G23" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H23" s="308" t="str">
+      <x:c r="H23" s="362" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I23" s="24" t="str">
@@ -1929,10 +2109,10 @@
       <x:c r="F24" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G24" s="306" t="str">
+      <x:c r="G24" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H24" s="308" t="str">
+      <x:c r="H24" s="362" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I24" s="24" t="str">
@@ -1958,10 +2138,10 @@
       <x:c r="F25" s="35" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="G25" s="306" t="str">
+      <x:c r="G25" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H25" s="308" t="str">
+      <x:c r="H25" s="362" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I25" s="24" t="str">
@@ -1987,10 +2167,10 @@
       <x:c r="F26" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G26" s="306" t="str">
+      <x:c r="G26" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H26" s="308" t="str">
+      <x:c r="H26" s="362" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I26" s="24" t="str">
@@ -2016,10 +2196,10 @@
       <x:c r="F27" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G27" s="306" t="str">
+      <x:c r="G27" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H27" s="308" t="str">
+      <x:c r="H27" s="362" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I27" s="24" t="str">
@@ -2045,10 +2225,10 @@
       <x:c r="F28" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G28" s="306" t="str">
+      <x:c r="G28" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H28" s="308" t="str">
+      <x:c r="H28" s="362" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I28" s="24" t="str">
@@ -2074,10 +2254,10 @@
       <x:c r="F29" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G29" s="306" t="str">
+      <x:c r="G29" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H29" s="309" t="str">
+      <x:c r="H29" s="363" t="str">
         <x:v>Smoke-tested</x:v>
       </x:c>
       <x:c r="I29" s="24" t="str">
@@ -2103,10 +2283,10 @@
       <x:c r="F30" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G30" s="306" t="str">
+      <x:c r="G30" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H30" s="308" t="str">
+      <x:c r="H30" s="362" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I30" s="24" t="str">
@@ -2132,10 +2312,10 @@
       <x:c r="F31" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G31" s="306" t="str">
+      <x:c r="G31" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H31" s="308" t="str">
+      <x:c r="H31" s="362" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I31" s="24" t="str">
@@ -2161,10 +2341,10 @@
       <x:c r="F32" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G32" s="306" t="str">
+      <x:c r="G32" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H32" s="308" t="str">
+      <x:c r="H32" s="362" t="str">
         <x:v>CLI model and effort documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I32" s="24" t="str">
@@ -2190,10 +2370,10 @@
       <x:c r="F33" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G33" s="306" t="str">
+      <x:c r="G33" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H33" s="308" t="str">
+      <x:c r="H33" s="362" t="str">
         <x:v>CLI model and effort documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I33" s="24" t="str">
@@ -2219,10 +2399,10 @@
       <x:c r="F34" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G34" s="306" t="str">
+      <x:c r="G34" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H34" s="308" t="str">
+      <x:c r="H34" s="362" t="str">
         <x:v>Profile documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I34" s="24" t="str">
@@ -2248,10 +2428,10 @@
       <x:c r="F35" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G35" s="306" t="str">
+      <x:c r="G35" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H35" s="308" t="str">
+      <x:c r="H35" s="362" t="str">
         <x:v>Profile documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I35" s="24" t="str">
@@ -2277,10 +2457,10 @@
       <x:c r="F36" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G36" s="306" t="str">
+      <x:c r="G36" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H36" s="308" t="str">
+      <x:c r="H36" s="362" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I36" s="24" t="str">
@@ -2306,10 +2486,10 @@
       <x:c r="F37" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G37" s="306" t="str">
+      <x:c r="G37" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H37" s="308" t="str">
+      <x:c r="H37" s="362" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I37" s="24" t="str">
@@ -2335,10 +2515,10 @@
       <x:c r="F38" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G38" s="306" t="str">
+      <x:c r="G38" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H38" s="308" t="str">
+      <x:c r="H38" s="362" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I38" s="24" t="str">
@@ -2364,10 +2544,10 @@
       <x:c r="F39" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G39" s="306" t="str">
+      <x:c r="G39" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H39" s="308" t="str">
+      <x:c r="H39" s="362" t="str">
         <x:v>Profile documented; exact runtime unverified</x:v>
       </x:c>
       <x:c r="I39" s="24" t="str">
@@ -2393,10 +2573,10 @@
       <x:c r="F40" s="35" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="G40" s="306" t="str">
+      <x:c r="G40" s="360" t="str">
         <x:v>Allowed fixed profile</x:v>
       </x:c>
-      <x:c r="H40" s="308" t="str">
+      <x:c r="H40" s="362" t="str">
         <x:v>Supported by metadata; routing unverified</x:v>
       </x:c>
       <x:c r="I40" s="24" t="str">
@@ -2437,7 +2617,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>Policy source: Interchange policy v0.8.0</x:v>
+        <x:v>Policy source: Interchange policy v0.9.0</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2" t="str">
@@ -2517,7 +2697,7 @@
         <x:v>Local search/tool when immediate; worker-muse-xhigh when delegation frees the Codex brain or is faster overall</x:v>
       </x:c>
       <x:c r="C10" s="24" t="str">
-        <x:v>Another external read-only mechanical profile; Codex worker only under a recorded mechanical allowance</x:v>
+        <x:v>worker-luna-xhigh or worker-luna-max or another bounded read-only profile; Luna needs no balancing allowance</x:v>
       </x:c>
       <x:c r="D10" s="24" t="str">
         <x:v>Count startup, supervision and handback overhead; delegate when it improves accepted-result time or cost</x:v>
@@ -2531,7 +2711,7 @@
         <x:v>worker-muse-xhigh</x:v>
       </x:c>
       <x:c r="C11" s="24" t="str">
-        <x:v>Another external bounded worker; Luna xhigh/max only under a recorded Codex mechanical allowance</x:v>
+        <x:v>worker-luna-xhigh or worker-luna-max or another bounded worker; Luna, Muse and DeepSeek need no balancing allowance</x:v>
       </x:c>
       <x:c r="D11" s="24" t="str">
         <x:v>Repository search, localization, evidence collection, narrow checks and small explicit edits; no interpretation</x:v>
@@ -2545,7 +2725,7 @@
         <x:v>worker-deepseek-flash-high; worker-grok-high; worker-opus-medium; worker-terra-xhigh; worker-sol-medium</x:v>
       </x:c>
       <x:c r="C12" s="24" t="str">
-        <x:v>Codex worker from this pool only under a recorded mechanical allowance and after external fit/availability check</x:v>
+        <x:v>Prefer unrestricted DeepSeek/Muse/Luna when task-fit; Terra/Sol require measured Codex allowance and Claude Code remains moderate/balanced</x:v>
       </x:c>
       <x:c r="D12" s="24" t="str">
         <x:v>Settled behavior, objective acceptance and bounded dependencies; ambiguity already resolved by a brain</x:v>
@@ -2573,7 +2753,7 @@
         <x:v>lead-sol-high resolves judgment; worker-opus-high or another qualified external profile executes settled packets</x:v>
       </x:c>
       <x:c r="C14" s="24" t="str">
-        <x:v>lead-astra-medium resolves unusually large ambiguity; Codex mechanical worker requires a recorded allowance; every Astra invocation requires fresh owner authorization and a concrete reason Sol high cannot fit</x:v>
+        <x:v>lead-astra-medium resolves unusually large ambiguity; Terra/Sol mechanical worker requires a recorded allowance; every Astra invocation requires fresh owner authorization and a concrete reason Sol high cannot fit</x:v>
       </x:c>
       <x:c r="D14" s="24" t="str">
         <x:v>Separate consequential decisions from implementation; independent review remains mandatory</x:v>
@@ -2587,7 +2767,7 @@
         <x:v>worker-deepseek-flash-high; worker-opus-high</x:v>
       </x:c>
       <x:c r="C15" s="24" t="str">
-        <x:v>worker-terra-max only under a recorded Codex mechanical allowance; never DeepSeek V4 Pro</x:v>
+        <x:v>worker-terra-max only under a recorded Terra/Sol mechanical allowance; never DeepSeek V4 Pro</x:v>
       </x:c>
       <x:c r="D15" s="24" t="str">
         <x:v>Dense mechanical implementation or integration with exact contracts and tests; never assign interpretation or use effort to outlast a loop</x:v>
@@ -2615,7 +2795,7 @@
         <x:v>Current delivery manager coordinates settled packets across external mechanical workers</x:v>
       </x:c>
       <x:c r="C17" s="24" t="str">
-        <x:v>lead-terra-xhigh/max only under a recorded Codex mechanical allowance</x:v>
+        <x:v>lead-terra-xhigh/max only under a recorded Terra/Sol mechanical allowance</x:v>
       </x:c>
       <x:c r="D17" s="24" t="str">
         <x:v>Preserve Codex brain capacity; a mechanical lead coordinates only settled work and returns ambiguity to Sol high or Astra medium</x:v>
@@ -2676,20 +2856,20 @@
       <x:c r="D22"/>
     </x:row>
     <x:row r="23" ht="42" customHeight="1">
-      <x:c r="A23" s="312" t="str">
+      <x:c r="A23" s="366" t="str">
         <x:v>Selection rules</x:v>
       </x:c>
-      <x:c r="B23" s="313"/>
-      <x:c r="C23" s="313"/>
-      <x:c r="D23" s="314"/>
+      <x:c r="B23" s="367"/>
+      <x:c r="C23" s="367"/>
+      <x:c r="D23" s="368"/>
     </x:row>
     <x:row r="24" ht="42" customHeight="1">
-      <x:c r="A24" s="320" t="str">
+      <x:c r="A24" s="374" t="str">
         <x:v>Approved selection rule</x:v>
       </x:c>
-      <x:c r="B24" s="321"/>
-      <x:c r="C24" s="321"/>
-      <x:c r="D24" s="322"/>
+      <x:c r="B24" s="375"/>
+      <x:c r="C24" s="375"/>
+      <x:c r="D24" s="376"/>
     </x:row>
     <x:row r="25" ht="42" customHeight="1">
       <x:c r="A25" s="91" t="str">
@@ -2757,7 +2937,7 @@
     </x:row>
     <x:row r="33" ht="42" customHeight="1">
       <x:c r="A33" s="92" t="str">
-        <x:v>9. Codex capacity is reserved for product/architecture judgment, integration decisions and independent semantic/risk review across the full usage window. Model quality alone does not justify Codex mechanical execution.</x:v>
+        <x:v>9. Sol, Terra and Claude Code are moderate, balanced capacity. Preserve Sol for judgment, integration and independent semantic/risk review; use unrestricted Luna, DeepSeek and Muse for suitable mechanical work and balance premium work across Claude/Codex when fit is comparable.</x:v>
       </x:c>
       <x:c r="B33" s="69"/>
       <x:c r="C33" s="69"/>
@@ -2765,7 +2945,7 @@
     </x:row>
     <x:row r="34" ht="42" customHeight="1">
       <x:c r="A34" s="92" t="str">
-        <x:v>10. External houses are the default mechanical lane. A Codex mechanical worker needs a recorded delivery allowance and reason; absence of an allowance means zero Codex mechanical dispatch.</x:v>
+        <x:v>10. Luna xhigh/max, DeepSeek V4.1 Flash and Muse Spark 1.3 are the unrestricted mechanical tier. They require no balancing allowance and have no Interchange concurrency cap when packets are independent and non-overlapping.</x:v>
       </x:c>
       <x:c r="B34" s="69"/>
       <x:c r="C34" s="69"/>
@@ -2773,7 +2953,7 @@
     </x:row>
     <x:row r="35" ht="42" customHeight="1">
       <x:c r="A35" s="92" t="str">
-        <x:v>11. Codex mechanical concurrency defaults to one. Parallel Codex mechanical workers require explicit owner authorization; use qualified external houses for parallel execution.</x:v>
+        <x:v>11. Terra/Sol mechanical concurrency defaults to one and requires a recorded allowance; parallel Terra/Sol workers require explicit owner authorization. Luna is exempt unless Astra exclusivity or an owner zero-Codex override applies.</x:v>
       </x:c>
       <x:c r="B35" s="69"/>
       <x:c r="C35" s="69"/>
@@ -2853,7 +3033,7 @@
     </x:row>
     <x:row r="45" ht="42" customHeight="1">
       <x:c r="A45" s="92" t="str">
-        <x:v>21. House exclusivity has two scopes. Astra at any effort reserves Codex globally and Fable 5.1 at any effort reserves Claude globally. Sol high or higher reserves Codex only for assignments under the same delivery manager; Opus high or higher reserves Claude only for assignments under the same delivery manager.</x:v>
+        <x:v>21. House exclusivity has two scopes. Astra at any effort reserves Codex globally and Fable 5.1 at any effort reserves Claude globally. Sol high or higher reserves Codex under the same delivery manager except unrestricted Luna xhigh/max mechanical leaves; Opus high or higher reserves Claude under the same delivery manager without that exception.</x:v>
       </x:c>
       <x:c r="B45" s="69"/>
       <x:c r="C45" s="69"/>
@@ -2946,6 +3126,22 @@
       <x:c r="B56" s="69"/>
       <x:c r="C56" s="69"/>
       <x:c r="D56" s="69"/>
+    </x:row>
+    <x:row r="57" ht="42" customHeight="1">
+      <x:c r="A57" s="92" t="str">
+        <x:v>33. Unrestricted does not mean ungoverned: Luna, DeepSeek and Muse still require bounded mechanical packets, non-overlapping ownership, watchdogs, valid completion and independent acceptance. Do not duplicate work merely because capacity is available.</x:v>
+      </x:c>
+      <x:c r="B57" s="69"/>
+      <x:c r="C57" s="69"/>
+      <x:c r="D57" s="69"/>
+    </x:row>
+    <x:row r="58" ht="42" customHeight="1">
+      <x:c r="A58" s="92" t="str">
+        <x:v>34. Grok retains its approved task-fit routing but is not part of the unrestricted tier or the new Terra/Sol/Claude balancing rule.</x:v>
+      </x:c>
+      <x:c r="B58" s="69"/>
+      <x:c r="C58" s="69"/>
+      <x:c r="D58" s="69"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2982,6 +3178,8 @@
     <x:mergeCell ref="A54:D54"/>
     <x:mergeCell ref="A55:D55"/>
     <x:mergeCell ref="A56:D56"/>
+    <x:mergeCell ref="A57:D57"/>
+    <x:mergeCell ref="A58:D58"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -3013,7 +3211,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>Policy source: Interchange policy v0.8.0</x:v>
+        <x:v>Policy source: Interchange policy v0.9.0</x:v>
       </x:c>
       <x:c r="B3" s="2" t="str">
         <x:v>Approved on</x:v>
@@ -3146,40 +3344,40 @@
         <x:v>Explicit do-not-use-Codex-for-delegation-or-leading instruction</x:v>
       </x:c>
       <x:c r="C16" s="24" t="str">
-        <x:v>Set Codex mechanical worker and mechanical lead allowance to zero; retain only explicitly requested brain/review use</x:v>
+        <x:v>Set every Codex mechanical worker and lead allocation, including Luna, to zero; retain only explicitly requested brain/review use</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="50" customHeight="1">
       <x:c r="A17" s="24" t="str">
-        <x:v>Codex capacity preflight</x:v>
+        <x:v>Terra/Sol capacity preflight</x:v>
       </x:c>
       <x:c r="B17" s="24" t="str">
-        <x:v>Fresh usage snapshot when available + declared brain/review reserve + explicit mechanical allowance</x:v>
+        <x:v>Fresh usage snapshot when available + declared brain/review reserve + explicit Terra/Sol mechanical allowance</x:v>
       </x:c>
       <x:c r="C17" s="24" t="str">
-        <x:v>No recorded allowance means zero new Codex mechanical workers; external houses are the default execution lane</x:v>
+        <x:v>No recorded allowance means zero new Terra/Sol mechanical workers; Luna is exempt unless Astra exclusivity or an owner zero-Codex override applies</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="50" customHeight="1">
       <x:c r="A18" s="24" t="str">
-        <x:v>Codex mechanical concurrency</x:v>
+        <x:v>Terra/Sol mechanical concurrency</x:v>
       </x:c>
       <x:c r="B18" s="24" t="str">
         <x:v>At most 1 active by default</x:v>
       </x:c>
       <x:c r="C18" s="24" t="str">
-        <x:v>Parallel Codex mechanical workers require explicit owner authorization; prefer external-house parallelism</x:v>
+        <x:v>Parallel Terra/Sol mechanical workers require explicit owner authorization; Luna is unrestricted by this cap</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="50" customHeight="1">
       <x:c r="A19" s="24" t="str">
-        <x:v>Codex early burn checkpoint</x:v>
+        <x:v>Terra/Sol early burn checkpoint</x:v>
       </x:c>
       <x:c r="B19" s="24" t="str">
-        <x:v>Recheck after first mechanical checkpoint when usage is observable</x:v>
+        <x:v>Recheck after first Terra/Sol mechanical checkpoint when usage is observable</x:v>
       </x:c>
       <x:c r="C19" s="24" t="str">
-        <x:v>Freeze new Codex mechanical dispatch when burn exceeds allowance or threatens reserved brain/review capacity</x:v>
+        <x:v>Freeze new Terra/Sol mechanical dispatch when burn exceeds allowance or threatens reserved brain/review capacity</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="50" customHeight="1">
@@ -3279,6 +3477,39 @@
       </x:c>
       <x:c r="C28" s="24" t="str">
         <x:v>A completed, failed or suspended invocation consumes its authorization; the next invocation needs a new owner decision</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="50" customHeight="1">
+      <x:c r="A29" s="24" t="str">
+        <x:v>Unrestricted mechanical tier</x:v>
+      </x:c>
+      <x:c r="B29" s="24" t="str">
+        <x:v>Luna xhigh/max, DeepSeek V4.1 Flash high/max, Muse Spark 1.3 xhigh</x:v>
+      </x:c>
+      <x:c r="C29" s="24" t="str">
+        <x:v>No balancing prerequisite or Interchange concurrency cap; three, four, five or more may run when assignments are useful, independent and non-overlapping</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="50" customHeight="1">
+      <x:c r="A30" s="24" t="str">
+        <x:v>Unrestricted-tier safeguards</x:v>
+      </x:c>
+      <x:c r="B30" s="24" t="str">
+        <x:v>Normal ownership, watchdog, completion and independent-acceptance rules remain</x:v>
+      </x:c>
+      <x:c r="C30" s="24" t="str">
+        <x:v>Free use never permits duplicate writers, overlapping paths, interpretation, unbounded loops or extra spending</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="50" customHeight="1">
+      <x:c r="A31" s="24" t="str">
+        <x:v>Moderate balanced tier</x:v>
+      </x:c>
+      <x:c r="B31" s="24" t="str">
+        <x:v>Terra, Sol and Claude Code</x:v>
+      </x:c>
+      <x:c r="C31" s="24" t="str">
+        <x:v>Plan and observe usage, protect brain/review capacity, avoid unnecessary concentration and balance across Claude/Codex when task fit is comparable; no forced alternation</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3312,7 +3543,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>Policy source: Interchange policy v0.8.0</x:v>
+        <x:v>Policy source: Interchange policy v0.9.0</x:v>
       </x:c>
       <x:c r="B3" s="2" t="str">
         <x:v>Approved on</x:v>
@@ -3475,20 +3706,20 @@
       <x:c r="C22"/>
     </x:row>
     <x:row r="23" ht="26" customHeight="1">
-      <x:c r="A23" s="312" t="str">
+      <x:c r="A23" s="366" t="str">
         <x:v>Recovery playbook</x:v>
       </x:c>
-      <x:c r="B23" s="313"/>
-      <x:c r="C23" s="314"/>
+      <x:c r="B23" s="367"/>
+      <x:c r="C23" s="368"/>
     </x:row>
     <x:row r="24" ht="44" customHeight="1">
-      <x:c r="A24" s="320" t="str">
+      <x:c r="A24" s="374" t="str">
         <x:v>Failure</x:v>
       </x:c>
-      <x:c r="B24" s="321" t="str">
+      <x:c r="B24" s="375" t="str">
         <x:v>First action</x:v>
       </x:c>
-      <x:c r="C24" s="322" t="str">
+      <x:c r="C24" s="376" t="str">
         <x:v>Escalation</x:v>
       </x:c>
     </x:row>

</xml_diff>